<commit_message>
Refresh lore export and link it from the party reference
Rebuild the Google Sheets/Docs packages with current lore, include
birthday on the character sheet, and document export regeneration in
the Dezco update rule.

Co-authored-by: Dralorex <Dralorex@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/character/lore/exports/Dezco_Knoleburn_Lore_Tabs.xlsx
+++ b/character/lore/exports/Dezco_Knoleburn_Lore_Tabs.xlsx
@@ -899,7 +899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A121"/>
+  <dimension ref="A1:A123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -989,7 +989,7 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>I am seventeen years old, five foot and ten inches tall, slender, with black hair that never quite stays where I want it. I love the colors red and black. Always have. Maybe that says something about me. Maybe it doesn’t. My family tree is a tangled thing, roots sunk deep into both Dwarven stone and Elven blood, and I have spent half my life wondering which half of me people see first.</t>
+          <t>**Birthday:** November 6</t>
         </is>
       </c>
     </row>
@@ -999,7 +999,7 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>I don’t really understand why I’ve been chosen. But here I am, trying my best.</t>
+          <t>I am seventeen years old, five foot and ten inches tall, slender, with black hair that never quite stays where I want it. I love the colors red and black. Always have. Maybe that says something about me. Maybe it doesn’t. My family tree is a tangled thing, roots sunk deep into both Dwarven stone and Elven blood, and I have spent half my life wondering which half of me people see first.</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Home is not a barracks, and it is not a prophecy. Home is a hamlet called Alzenhiem.</t>
+          <t>I don’t really understand why I’ve been chosen. But here I am, trying my best.</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>## What our names mean</t>
+          <t>Home is not a barracks, and it is not a prophecy. Home is a hamlet called Alzenhiem.</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>In Alzenhiem, a name is the first charge laid on a life. Crest and sigil are painted to serve it.</t>
+          <t>## What our names mean</t>
         </is>
       </c>
     </row>
@@ -1039,59 +1039,59 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>1. **Alzenhiem:** sheltered home under a kind sky</t>
+          <t>In Alzenhiem, a name is the first charge laid on a life. Crest and sigil are painted to serve it.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>2. **Knoleburn:** stream by the knoll; a house tied to living land</t>
-        </is>
-      </c>
+      <c r="A28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>3. **Dolkin** (Dol kin): steadfast of kin</t>
+          <t>1. **Alzenhiem:** sheltered home under a kind sky</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>4. **Fulfein** (Fule fe in): full fair light</t>
+          <t>2. **Knoleburn:** stream by the knoll; a house tied to living land</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>5. **Dezco:** stands firm</t>
+          <t>3. **Dolkin** (Dol kin): steadfast of kin</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>6. **Kalhien** (Kal he en): rises in pursuit</t>
+          <t>4. **Fulfein** (Fule fe in): full fair light</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>7. **Astiale** (as T ale): gentle star</t>
+          <t>5. **Dezco:** stands firm</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="inlineStr"/>
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>6. **Kalhien** (Kal he en): rises in pursuit</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>The longer naming notes live in the Knoleburn names lore.</t>
+          <t>7. **Astiale** (as T ale): gentle star</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>## Alzenhiem</t>
+          <t>The longer naming notes live in the Knoleburn names lore.</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Alzenhiem is small enough that everyone knows your footsteps before they know your name. It sits where the land still feels honest: dirt paths, low roofs, smoke that smells like supper instead of war. There are no banners tall enough to impress a king there. No parade grounds. Just people who mend what breaks, share what they can, and keep their doors ready for neighbors.</t>
+          <t>## Alzenhiem</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>I call it home even when I am far from it. Especially when I am far from it.</t>
+          <t>Alzenhiem is small enough that everyone knows your footsteps before they know your name. It sits where the land still feels honest: dirt paths, low roofs, smoke that smells like supper instead of war. There are no banners tall enough to impress a king there. No parade grounds. Just people who mend what breaks, share what they can, and keep their doors ready for neighbors.</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>When I left for military training at eight years old, Alzenhiem was the last soft place my hands remembered. The yard taught me how to stand. Alzenhiem taught me what I was standing for. On hard nights under the Lion, I did not dream of glory. I dreamed of the lane behind our house, of my mother’s voice through an open window, of my father’s shadow crossing the doorway at dusk.</t>
+          <t>I call it home even when I am far from it. Especially when I am far from it.</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>If the world ever asks what I am protecting when I talk about hope, the true answer begins there.</t>
+          <t>When I left for military training at eight years old, Alzenhiem was the last soft place my hands remembered. The yard taught me how to stand. Alzenhiem taught me what I was standing for. On hard nights under the Lion, I did not dream of glory. I dreamed of the lane behind our house, of my mother’s voice through an open window, of my father’s shadow crossing the doorway at dusk.</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>## Crests of Alzenhiem</t>
+          <t>If the world ever asks what I am protecting when I talk about hope, the true answer begins there.</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>Alzenhiem keeps a quiet crest tradition. Signs are a naming rite, not noble vanity. The hamlet has its own flag: wheat, roof, and lane in gold, green, brown, and cream. When a child is born, they receive a crest that must hold three truths: the name they are given, their gender, and marks from both parents. Parent crests are fuller. Child crests stay simpler on purpose, so a newborn is not buried under a complicated fate. Colors follow the person’s vibe as the family first felt it.</t>
+          <t>## Crests of Alzenhiem</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>Ours run like this:</t>
+          <t>Alzenhiem keeps a quiet crest tradition. Signs are a naming rite, not noble vanity. The hamlet has its own flag: wheat, roof, and lane in gold, green, brown, and cream. When a child is born, they receive a crest that must hold three truths: the name they are given, their gender, and marks from both parents. Parent crests are fuller. Child crests stay simpler on purpose, so a newborn is not buried under a complicated fate. Colors follow the person’s vibe as the family first felt it.</t>
         </is>
       </c>
     </row>
@@ -1181,45 +1181,45 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>1. Dolkin: charcoal, iron, and bronze amber over stone and hammer, made for bearing weight and keeping shelter</t>
+          <t>Ours run like this:</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="6" t="inlineStr">
-        <is>
-          <t>2. Fulfein: sage, silver, and pale gold around leaf and crescent, made for care and watchfulness</t>
-        </is>
-      </c>
+      <c r="A54" s="6" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>3. Mine: red and black, a simple blade of balance between their marks, set that way at birth because both lines already lived in me</t>
+          <t>1. Dolkin: charcoal, iron, and bronze amber over stone and hammer, made for bearing weight and keeping shelter</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>4. Kalhien: ink blue and copper, eager and forward, colored apart from me so he would not grow under my shadow</t>
+          <t>2. Fulfein: sage, silver, and pale gold around leaf and crescent, made for care and watchfulness</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>5. Astiale: soft rose, cream, and a touch of sky, kept gentle on purpose so kindness stayed part of our house</t>
+          <t>3. Mine: red and black, a simple blade of balance between their marks, set that way at birth because both lines already lived in me</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="6" t="inlineStr"/>
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>4. Kalhien: ink blue and copper, eager and forward, colored apart from me so he would not grow under my shadow</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>Each of us also has a personal sigil made the same day as the crest: one simple mark in our colors, like a seal. Crests are the fuller signs. Sigils are the quick ones.</t>
+          <t>5. Astiale: soft rose, cream, and a touch of sky, kept gentle on purpose so kindness stayed part of our house</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1229,7 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>The full meanings, birth design reasons, and images live under the Alzenhiem crest archive.</t>
+          <t>Each of us also has a personal sigil made the same day as the crest: one simple mark in our colors, like a seal. Crests are the fuller signs. Sigils are the quick ones.</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>## The Knoleburn family</t>
+          <t>The full meanings, birth design reasons, and images live under the Alzenhiem crest archive.</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>We are not a house of lords. We are a family that stayed, worked, and loved in a place too small for maps to bother with. That is enough. That has always been enough.</t>
+          <t>## The Knoleburn family</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1259,7 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>### Dolkin Knoleburn (Dol kin), father, 38</t>
+          <t>We are not a house of lords. We are a family that stayed, worked, and loved in a place too small for maps to bother with. That is enough. That has always been enough.</t>
         </is>
       </c>
     </row>
@@ -1269,7 +1269,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>**Name meaning:** steadfast of kin</t>
+          <t>### Dolkin Knoleburn (Dol kin), father, 38</t>
         </is>
       </c>
     </row>
@@ -1279,7 +1279,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>My father is thirty eight. Steady in the way stone is steady: not flashy, not loud, simply there when weight needs somewhere to rest. Dolkin carries the Dwarven depth in our line more openly than the rest of us. He believes in work done properly, in keeping your word, and in protecting your own without making a speech about it.</t>
+          <t>**Name meaning:** steadfast of kin</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>He did not send me away at eight because he wanted a legend. He sent me because he believed a hard road might keep me alive in a harder world. I think that choice still sits heavy on him. Fathers like Dolkin do not waste words on guilt. They show it by asking if you have eaten, by checking your hands for new scars, by saying your name like it still belongs to Alzenhiem first.</t>
+          <t>My father is thirty eight. Steady in the way stone is steady: not flashy, not loud, simply there when weight needs somewhere to rest. Dolkin carries the Dwarven depth in our line more openly than the rest of us. He believes in work done properly, in keeping your word, and in protecting your own without making a speech about it.</t>
         </is>
       </c>
     </row>
@@ -1299,7 +1299,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>### Fulfein Knoleburn (Fule fe in), mother, 36</t>
+          <t>He did not send me away at eight because he wanted a legend. He sent me because he believed a hard road might keep me alive in a harder world. I think that choice still sits heavy on him. Fathers like Dolkin do not waste words on guilt. They show it by asking if you have eaten, by checking your hands for new scars, by saying your name like it still belongs to Alzenhiem first.</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1309,7 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>**Name meaning:** full fair light</t>
+          <t>### Fulfein Knoleburn (Fule fe in), mother, 36</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1319,7 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>My mother is thirty six. Fulfein holds more of the Elven grace in our blood, though she wears it quietly, the way soft light wears on water. She is warm without being fragile. Kind without being blind. If Alzenhiem has a center for me, it is her.</t>
+          <t>**Name meaning:** full fair light</t>
         </is>
       </c>
     </row>
@@ -1329,7 +1329,7 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>She writes when she can. She remembers dates nobody else keeps. She asked me once, when I was still small enough to fit under her arm, whether I was afraid of leaving. I told her no. She knew I was lying and loved me anyway. That is Fulfein: she sees the truth, then stays beside you while you grow brave enough to say it.</t>
+          <t>My mother is thirty six. Fulfein holds more of the Elven grace in our blood, though she wears it quietly, the way soft light wears on water. She is warm without being fragile. Kind without being blind. If Alzenhiem has a center for me, it is her.</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1339,7 @@
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>### Kalhien Knoleburn (Kal he en), younger brother, 15</t>
+          <t>She writes when she can. She remembers dates nobody else keeps. She asked me once, when I was still small enough to fit under her arm, whether I was afraid of leaving. I told her no. She knew I was lying and loved me anyway. That is Fulfein: she sees the truth, then stays beside you while you grow brave enough to say it.</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>**Name meaning:** rises in pursuit</t>
+          <t>### Kalhien Knoleburn (Kal he en), younger brother, 15</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1359,7 @@
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>Kalhien is fifteen. Two years behind me, and somehow already trying to walk like he can catch up. He was six when I left for the yard. Old enough to remember me as a brother, young enough that my absence became part of how he grew.</t>
+          <t>**Name meaning:** rises in pursuit</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>He is sharp, restless, and proud in the way younger brothers are proud when the older one becomes a story people tell. Sometimes that pride helps him. Sometimes it bruises him. He wants to be taken seriously. He wants to prove he is more than “Dezco’s little brother.” I understand that more than he thinks.</t>
+          <t>Kalhien is fifteen. Two years behind me, and somehow already trying to walk like he can catch up. He was six when I left for the yard. Old enough to remember me as a brother, young enough that my absence became part of how he grew.</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1379,7 @@
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>When I see him now, I still look for the boy who used to trail me down the lane. He looks back like he is measuring the distance between us and deciding whether to close it or race it.</t>
+          <t>He is sharp, restless, and proud in the way younger brothers are proud when the older one becomes a story people tell. Sometimes that pride helps him. Sometimes it bruises him. He wants to be taken seriously. He wants to prove he is more than “Dezco’s little brother.” I understand that more than he thinks.</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>### Astiale Knoleburn (as T ale), younger sister, 8</t>
+          <t>When I see him now, I still look for the boy who used to trail me down the lane. He looks back like he is measuring the distance between us and deciding whether to close it or race it.</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>**Name meaning:** gentle star</t>
+          <t>### Astiale Knoleburn (as T ale), younger sister, 8</t>
         </is>
       </c>
     </row>
@@ -1409,7 +1409,7 @@
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>Astiale is eight. Sweet in a way the world has not managed to sand down yet. She was not born when I first left Alzenhiem. I met my own sister in pieces: visits, letters, the sudden shock of a child who already knew my name before I knew her face.</t>
+          <t>**Name meaning:** gentle star</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1419,7 @@
     <row r="99">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>She calls me home even when the rest of the realm calls me other things. To Astiale I am not a rumor, not a prophecy, not the Lion’s apprentice. I am her older brother who comes and goes, who kneels so she can reach me, who pretends not to notice when she hides behind Fulfein for the first minute and then refuses to let go for the last.</t>
+          <t>Astiale is eight. Sweet in a way the world has not managed to sand down yet. She was not born when I first left Alzenhiem. I met my own sister in pieces: visits, letters, the sudden shock of a child who already knew my name before I knew her face.</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>If there is still softness left in me after years of training, a great deal of it has her name on it.</t>
+          <t>She calls me home even when the rest of the realm calls me other things. To Astiale I am not a rumor, not a prophecy, not the Lion’s apprentice. I am her older brother who comes and goes, who kneels so she can reach me, who pretends not to notice when she hides behind Fulfein for the first minute and then refuses to let go for the last.</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1439,7 @@
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>## Blood and belonging</t>
+          <t>If there is still softness left in me after years of training, a great deal of it has her name on it.</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1449,7 @@
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>People look at me and try to sort me: Dwarf or Elf, soldier or boy, omen or accident. In Alzenhiem, nobody sorted me first. They knew me as Dezco, son of Dolkin and Fulfein, brother to Kalhien and Astiale. Black hair, too thin for the work some expected, stubborn enough for the work that mattered.</t>
+          <t>## Blood and belonging</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1459,7 @@
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>The Dwarven stone and Elven blood in me are not costumes I put on for strangers. They are my parents’ gifts, living under one roof in a hamlet that never asked us to choose only one half. That is why leaving hurt. That is why returning, even briefly, steadies me.</t>
+          <t>People look at me and try to sort me: Dwarf or Elf, soldier or boy, omen or accident. In Alzenhiem, nobody sorted me first. They knew me as Dezco, son of Dolkin and Fulfein, brother to Kalhien and Astiale. Black hair, too thin for the work some expected, stubborn enough for the work that mattered.</t>
         </is>
       </c>
     </row>
@@ -1469,7 +1469,7 @@
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>I love red and black. I always have. I do not yet know all of why. What I do know is simpler: when I wear those colors into the wider world, I am still trying to bring Alzenhiem with me. Not the buildings. The people. The promise that someone from a small place can stand in a large darkness and not forget where the light first taught him his name.</t>
+          <t>The Dwarven stone and Elven blood in me are not costumes I put on for strangers. They are my parents’ gifts, living under one roof in a hamlet that never asked us to choose only one half. That is why leaving hurt. That is why returning, even briefly, steadies me.</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1479,7 @@
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>## As I am now</t>
+          <t>I love red and black. I always have. I do not yet know all of why. What I do know is simpler: when I wear those colors into the wider world, I am still trying to bring Alzenhiem with me. Not the buildings. The people. The promise that someone from a small place can stand in a large darkness and not forget where the light first taught him his name.</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1489,7 @@
     <row r="113">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>I am seventeen. A student no longer. A Hero by Yua’s charge, whether I feel ready or not. The realm has ideas about me. Some are rumor. Some are becoming true.</t>
+          <t>## As I am now</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
     <row r="115">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>Before any of that, I am Dezco Knoleburn of Alzenhiem.</t>
+          <t>I am seventeen. A student no longer. A Hero by Yua’s charge, whether I feel ready or not. The realm has ideas about me. Some are rumor. Some are becoming true.</t>
         </is>
       </c>
     </row>
@@ -1509,7 +1509,7 @@
     <row r="117">
       <c r="A117" s="6" t="inlineStr">
         <is>
-          <t>Son of Dolkin and Fulfein.</t>
+          <t>Before any of that, I am Dezco Knoleburn of Alzenhiem.</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1519,7 @@
     <row r="119">
       <c r="A119" s="6" t="inlineStr">
         <is>
-          <t>Brother of Kalhien and Astiale.</t>
+          <t>Son of Dolkin and Fulfein.</t>
         </is>
       </c>
     </row>
@@ -1528,6 +1528,16 @@
     </row>
     <row r="121">
       <c r="A121" s="6" t="inlineStr">
+        <is>
+          <t>Brother of Kalhien and Astiale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="6" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="6" t="inlineStr">
         <is>
           <t>Trying my best to become someone worth the home that made me.</t>
         </is>
@@ -5039,7 +5049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A268"/>
+  <dimension ref="A1:A272"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -5089,7 +5099,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">**Last updated:** 2026-07-25 (Yua Mana Well plot added; journal 03 dash clarified)  </t>
+          <t xml:space="preserve">**Last updated:** 2026-07-25 (Google Drive lore export pack added)  </t>
         </is>
       </c>
     </row>
@@ -5191,1378 +5201,1382 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>| Height | 5'10" |</t>
+          <t>| Birthday | November 6 |</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>| Build | slender |</t>
+          <t>| Height | 5'10" |</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>| Hair | black |</t>
+          <t>| Build | slender |</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>| Favorite colors | red and black |</t>
+          <t>| Hair | black |</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>| Ancestry | Dwarven + Elven |</t>
+          <t>| Favorite colors | red and black |</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>| Home | Alzenhiem (hamlet) |</t>
+          <t>| Ancestry | Dwarven + Elven |</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>| Title now | Hero (given by Yua at 17) |</t>
+          <t>| Home | Alzenhiem (hamlet) |</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>| Master | The King’s Lion |</t>
+          <t>| Title now | Hero (given by Yua at 17) |</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>| Companion | Yua (often appears as a small pixie) |</t>
+          <t>| Master | The King’s Lion |</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>| Crest colors | crimson red + deep black |</t>
+          <t>| Companion | Yua (often appears as a small pixie) |</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>| Sigil | vertical blade / flame split red and black |</t>
+          <t>| Crest colors | crimson red + deep black |</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>| Current location | Saltrock general building (doors sealed; under attack) |</t>
+          <t>| Sigil | vertical blade / flame split red and black |</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
+          <t>| Current location | Saltrock general building (doors sealed; under attack) |</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
           <t>| Travel status | Adventure day 2 gone wrong; protective staff fell; mid siege |</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr"/>
-    </row>
     <row r="41">
-      <c r="A41" s="6" t="inlineStr">
+      <c r="A41" s="6" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr"/>
-    </row>
     <row r="43">
-      <c r="A43" s="6" t="inlineStr">
+      <c r="A43" s="6" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
         <is>
           <t>## What I am / am not</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="6" t="inlineStr"/>
-    </row>
     <row r="45">
-      <c r="A45" s="6" t="inlineStr">
-        <is>
-          <t>| True | Not true (or not yet) |</t>
-        </is>
-      </c>
+      <c r="A45" s="6" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| True | Not true (or not yet) |</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>| Hero by Yua’s formal charge at age 17 | Born already crowned as Hero |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>| Trained hard under the King’s Lion | Famous because of easy blessing alone |</t>
+          <t>| Hero by Yua’s formal charge at age 17 | Born already crowned as Hero |</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>| People rumored I was the Hero of centuries during ages 12 to 17 | Those years were title + sacred charge (they were rumor) |</t>
+          <t>| Trained hard under the King’s Lion | Famous because of easy blessing alone |</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>| Yua watched me from childhood | I always understood why she chose me |</t>
+          <t>| People rumored I was the Hero of centuries during ages 12 to 17 | Those years were title + sacred charge (they were rumor) |</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>| I love red and black | I already know the deep reason why (Yua has not told me yet) |</t>
+          <t>| Yua watched me from childhood | I always understood why she chose me |</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>| Yua set a Mana Well in me when she made me Hero | I understood it before Saltrock (I did not) |</t>
+          <t>| I love red and black | I already know the deep reason why (Yua has not told me yet) |</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
+          <t>| Yua set a Mana Well in me when she made me Hero | I understood it before Saltrock (I did not) |</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
           <t>| I accidentally used a simple imbue in Saltrock | I meant to dash 15 feet and faceplant on purpose |</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="6" t="inlineStr"/>
-    </row>
     <row r="55">
-      <c r="A55" s="6" t="inlineStr">
+      <c r="A55" s="6" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="6" t="inlineStr"/>
-    </row>
     <row r="57">
-      <c r="A57" s="6" t="inlineStr">
+      <c r="A57" s="6" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
         <is>
           <t>## Family (quick)</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="6" t="inlineStr"/>
-    </row>
     <row r="59">
-      <c r="A59" s="6" t="inlineStr">
-        <is>
-          <t>| Person | Who | Age | Name means | Colors | One line |</t>
-        </is>
-      </c>
+      <c r="A59" s="6" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>|---|---|---|---|---|---|</t>
+          <t>| Person | Who | Age | Name means | Colors | One line |</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>| Dolkin | Father | 38 | steadfast of kin | charcoal, iron, bronze | Steady, Dwarven depth, sent me to train to keep me alive |</t>
+          <t>|---|---|---|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>| Fulfein | Mother | 36 | full fair light | sage, silver, pale gold | Warm Elven grace; Alzenhiem’s center for me |</t>
+          <t>| Dolkin | Father | 38 | steadfast of kin | charcoal, iron, bronze | Steady, Dwarven depth, sent me to train to keep me alive |</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>| Kalhien | Younger brother | 15 | rises in pursuit | ink blue + copper | Restless, proud, does not want to be only “Dezco’s brother” |</t>
+          <t>| Fulfein | Mother | 36 | full fair light | sage, silver, pale gold | Warm Elven grace; Alzenhiem’s center for me |</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
+          <t>| Kalhien | Younger brother | 15 | rises in pursuit | ink blue + copper | Restless, proud, does not want to be only “Dezco’s brother” |</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
           <t>| Astiale | Younger sister | 8 | gentle star | rose, cream, sky | Sweet; not born when I left at 8 |</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="6" t="inlineStr"/>
-    </row>
     <row r="66">
-      <c r="A66" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">**Surname Knoleburn means:** stream by the knoll  </t>
-        </is>
-      </c>
+      <c r="A66" s="6" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">**Surname Knoleburn means:** stream by the knoll  </t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
           <t>**Alzenhiem means:** sheltered home under a kind sky</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="6" t="inlineStr"/>
-    </row>
     <row r="69">
-      <c r="A69" s="6" t="inlineStr">
+      <c r="A69" s="6" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="6" t="inlineStr"/>
-    </row>
     <row r="71">
-      <c r="A71" s="6" t="inlineStr">
+      <c r="A71" s="6" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
         <is>
           <t>## Home</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="6" t="inlineStr"/>
-    </row>
     <row r="73">
-      <c r="A73" s="6" t="inlineStr">
-        <is>
-          <t>| | |</t>
-        </is>
-      </c>
+      <c r="A73" s="6" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| | |</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>| Place | Alzenhiem |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>| Type | Small hamlet |</t>
+          <t>| Place | Alzenhiem |</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>| Vibe | Dirt paths, low roofs, neighbors first, no royal banners |</t>
+          <t>| Type | Small hamlet |</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>| Why it matters | What I stand for when I talk about hope |</t>
+          <t>| Vibe | Dirt paths, low roofs, neighbors first, no royal banners |</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>| Town flag colors | wheat gold, meadow green, earth brown, cream |</t>
+          <t>| Why it matters | What I stand for when I talk about hope |</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
+          <t>| Town flag colors | wheat gold, meadow green, earth brown, cream |</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
           <t>| Town flag idea | roof + wheat + lane |</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="6" t="inlineStr"/>
-    </row>
     <row r="82">
-      <c r="A82" s="6" t="inlineStr">
+      <c r="A82" s="6" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="6" t="inlineStr"/>
-    </row>
     <row r="84">
-      <c r="A84" s="6" t="inlineStr">
+      <c r="A84" s="6" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="inlineStr">
         <is>
           <t>## Timeline (memorize this order)</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="6" t="inlineStr"/>
-    </row>
     <row r="86">
-      <c r="A86" s="6" t="inlineStr">
-        <is>
-          <t>| Age | What happened |</t>
-        </is>
-      </c>
+      <c r="A86" s="6" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| Age | What happened |</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>| 0 | Named Dezco; red/black crest + sigil at birth |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>| 8 | Left Alzenhiem for military training; Kalhien was 6; Astiale not born yet |</t>
+          <t>| 0 | Born November 6; named Dezco; red/black crest + sigil at birth |</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>| 8 to 12 | Overshadowed by a stronger rival; Yua watched unseen |</t>
+          <t>| 8 | Left Alzenhiem for military training; Kalhien was 6; Astiale not born yet |</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>| 12 | Rival (nearly 18) dueled me; Yua secretly blessed my speed/strength; only the King’s Lion truly saw her |</t>
+          <t>| 8 to 12 | Overshadowed by a stronger rival; Yua watched unseen |</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>| 12 | Became the King’s Lion’s personal apprentice |</t>
+          <t>| 12 | Rival (nearly 18) dueled me; Yua secretly blessed my speed/strength; only the King’s Lion truly saw her |</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>| 12 to 17 | Merciless real missions; reputation spread; people falsely called me Hero of centuries |</t>
+          <t>| 12 | Became the King’s Lion’s personal apprentice |</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>| Before 15 | Name known across much of the realm |</t>
+          <t>| 12 to 17 | Merciless real missions; reputation spread; people falsely called me Hero of centuries |</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Master said I had learned all he could teach |</t>
+          <t>| Before 15 | Name known across much of the realm |</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Yua appeared to me and the Lion; gave me the ancient title Hero + sacred mission |</t>
+          <t>| 17 | Master said I had learned all he could teach |</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Final goodbye at Alzenhiem; family gifts; left for the road |</t>
+          <t>| 17 | Yua appeared to me and the Lion; gave me the ancient title Hero + sacred mission |</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Reached Saltrock; lodging at the tavern; seeking where to travel next |</t>
+          <t>| 17 | Final goodbye at Alzenhiem; family gifts; left for the road |</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Saltrock staff fell; monsters attacked (massive crabs + others) |</t>
+          <t>| 17 | Reached Saltrock; lodging at the tavern; seeking where to travel next |</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Fought with 4 other defenders; missed a short bow creature; saved by an elf girl’s arrow |</t>
+          <t>| 17 | Saltrock staff fell; monsters attacked (massive crabs + others) |</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Barely sealed inside the general building; many townsfolk fate unknown |</t>
+          <t>| 17 | Fought with 4 other defenders; missed a short bow creature; saved by an elf girl’s arrow |</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="6" t="inlineStr">
         <is>
+          <t>| 17 | Barely sealed inside the general building; many townsfolk fate unknown |</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="6" t="inlineStr">
+        <is>
           <t>| Now | Trapped in Saltrock general building during the attack; entry open ended |</t>
         </is>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="6" t="inlineStr"/>
-    </row>
     <row r="104">
-      <c r="A104" s="6" t="inlineStr">
+      <c r="A104" s="6" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="6" t="inlineStr"/>
-    </row>
     <row r="106">
-      <c r="A106" s="6" t="inlineStr">
+      <c r="A106" s="6" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="6" t="inlineStr">
         <is>
           <t>## Important people (outside family)</t>
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" s="6" t="inlineStr"/>
-    </row>
     <row r="108">
-      <c r="A108" s="6" t="inlineStr">
-        <is>
-          <t>| Person | Who they are to me |</t>
-        </is>
-      </c>
+      <c r="A108" s="6" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| Person | Who they are to me |</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>| Yua | Ancient being tied to magic; broke a millennia oath to act; watched me since childhood; gave me Hero title; often appears as a small pixie |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>| The King’s Lion | King’s greatest swordsman; only one who truly saw Yua at the duel; my master |</t>
+          <t>| Yua | Ancient being tied to magic; broke a millennia oath to act; watched me since childhood; gave me Hero title; often appears as a small pixie |</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>| The Rival | Older trainee who believed he was the chosen one; challenged me at 12; lost after Yua’s hidden aid |</t>
+          <t>| The King’s Lion | King’s greatest swordsman; only one who truly saw Yua at the duel; my master |</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>| Elf girl archer | One of 4 defenders in Saltrock attack; pinned a short bow creature through the mouth and into the ground; name not known yet |</t>
+          <t>| The Rival | Older trainee who believed he was the chosen one; challenged me at 12; lost after Yua’s hidden aid |</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="6" t="inlineStr">
         <is>
+          <t>| Elf girl archer | One of 4 defenders in Saltrock attack; pinned a short bow creature through the mouth and into the ground; name not known yet |</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="6" t="inlineStr">
+        <is>
           <t>| 3 other defenders | Fought beside us getting townsfolk to the general building; names not known yet |</t>
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" s="6" t="inlineStr"/>
-    </row>
     <row r="116">
-      <c r="A116" s="6" t="inlineStr">
+      <c r="A116" s="6" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" s="6" t="inlineStr"/>
-    </row>
     <row r="118">
-      <c r="A118" s="6" t="inlineStr">
+      <c r="A118" s="6" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="6" t="inlineStr">
         <is>
           <t>## Current gear / gifts from home</t>
         </is>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="6" t="inlineStr"/>
-    </row>
     <row r="120">
-      <c r="A120" s="6" t="inlineStr">
-        <is>
-          <t>| Item | From | Notes |</t>
-        </is>
-      </c>
+      <c r="A120" s="6" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="6" t="inlineStr">
         <is>
-          <t>|---|---|---|</t>
+          <t>| Item | From | Notes |</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="6" t="inlineStr">
         <is>
-          <t>| New sword | Dolkin | Hand forged goodbye; his love without saying the words |</t>
+          <t>|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
         <is>
-          <t>| First smithing tools | Dolkin | His original set; “you are the master of your steel” |</t>
+          <t>| New sword | Dolkin | Hand forged goodbye; his love without saying the words |</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="6" t="inlineStr">
         <is>
-          <t>| 10 gold pieces | Fulfein | Travel money |</t>
+          <t>| First smithing tools | Dolkin | His original set; “you are the master of your steel” |</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="6" t="inlineStr">
         <is>
-          <t>| Cooking pot | Fulfein | Eat warm when you can |</t>
+          <t>| 10 gold pieces | Fulfein | Travel money |</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="6" t="inlineStr">
         <is>
-          <t>| New clothing | Fulfein | Wearing them out of respect; left home in them |</t>
+          <t>| Cooking pot | Fulfein | Eat warm when you can |</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="6" t="inlineStr">
         <is>
+          <t>| New clothing | Fulfein | Wearing them out of respect; left home in them |</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="6" t="inlineStr">
+        <is>
           <t>| Shovel | Fulfein | Funny gift for roadside “number two” duty; also quietly useful if not everyone makes it |</t>
         </is>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" s="6" t="inlineStr"/>
-    </row>
     <row r="129">
-      <c r="A129" s="6" t="inlineStr">
+      <c r="A129" s="6" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="130">
-      <c r="A130" s="6" t="inlineStr"/>
-    </row>
     <row r="131">
-      <c r="A131" s="6" t="inlineStr">
+      <c r="A131" s="6" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="6" t="inlineStr">
         <is>
           <t>## Places</t>
         </is>
       </c>
     </row>
-    <row r="132">
-      <c r="A132" s="6" t="inlineStr"/>
-    </row>
     <row r="133">
-      <c r="A133" s="6" t="inlineStr">
-        <is>
-          <t>| Place | What it is |</t>
-        </is>
-      </c>
+      <c r="A133" s="6" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| Place | What it is |</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="6" t="inlineStr">
         <is>
-          <t>| Alzenhiem | Home hamlet; my center |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="6" t="inlineStr">
         <is>
-          <t>| Saltrock | Traveling town of people coming and going; I know it well |</t>
+          <t>| Alzenhiem | Home hamlet; my center |</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>| Saltrock general building | Holds the protective magic staff; we are sealed inside it during the attack |</t>
+          <t>| Saltrock | Traveling town of people coming and going; I know it well |</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
         <is>
-          <t>| Saltrock protective staff | Used to float and block named monsters/creatures; has fallen; reason unknown |</t>
+          <t>| Saltrock general building | Holds the protective magic staff; we are sealed inside it during the attack |</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
         <is>
+          <t>| Saltrock protective staff | Used to float and block named monsters/creatures; has fallen; reason unknown |</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="6" t="inlineStr">
+        <is>
           <t>| Saltrock tavern | Where I lodged the night before the attack; “best bread” only with nostalgia |</t>
         </is>
       </c>
     </row>
-    <row r="140">
-      <c r="A140" s="6" t="inlineStr"/>
-    </row>
     <row r="141">
-      <c r="A141" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">**First magic item I ever saw:** the floating protective staff in Saltrock.  </t>
-        </is>
-      </c>
+      <c r="A141" s="6" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">**First magic item I ever saw:** the floating protective staff in Saltrock.  </t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="6" t="inlineStr">
+        <is>
           <t>**Current crisis:** staff down; crabs and other creatures overran the streets; unknown how many people remain outside.</t>
         </is>
       </c>
     </row>
-    <row r="143">
-      <c r="A143" s="6" t="inlineStr"/>
-    </row>
     <row r="144">
-      <c r="A144" s="6" t="inlineStr">
+      <c r="A144" s="6" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="145">
-      <c r="A145" s="6" t="inlineStr"/>
-    </row>
     <row r="146">
-      <c r="A146" s="6" t="inlineStr">
+      <c r="A146" s="6" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="6" t="inlineStr">
         <is>
           <t>## My Hero mission (from Yua)</t>
         </is>
       </c>
     </row>
-    <row r="147">
-      <c r="A147" s="6" t="inlineStr"/>
-    </row>
     <row r="148">
-      <c r="A148" s="6" t="inlineStr">
-        <is>
-          <t>1. Restore magic before it disappears completely</t>
-        </is>
-      </c>
+      <c r="A148" s="6" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="6" t="inlineStr">
         <is>
-          <t>2. Stand against the darkness consuming the world</t>
+          <t>1. Restore magic before it disappears completely</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="6" t="inlineStr">
         <is>
-          <t>3. Unite the fractured kingdoms and races</t>
+          <t>2. Stand against the darkness consuming the world</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="6" t="inlineStr">
         <is>
-          <t>4. Become the symbol of hope the world has long forgotten</t>
+          <t>3. Unite the fractured kingdoms and races</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="6" t="inlineStr">
         <is>
+          <t>4. Become the symbol of hope the world has long forgotten</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="6" t="inlineStr">
+        <is>
           <t>5. Bring together the two halves of the world</t>
         </is>
       </c>
     </row>
-    <row r="153">
-      <c r="A153" s="6" t="inlineStr"/>
-    </row>
     <row r="154">
-      <c r="A154" s="6" t="inlineStr">
+      <c r="A154" s="6" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="155">
-      <c r="A155" s="6" t="inlineStr"/>
-    </row>
     <row r="156">
-      <c r="A156" s="6" t="inlineStr">
+      <c r="A156" s="6" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="6" t="inlineStr">
         <is>
           <t>## Training under the Lion included</t>
         </is>
       </c>
     </row>
-    <row r="157">
-      <c r="A157" s="6" t="inlineStr"/>
-    </row>
     <row r="158">
-      <c r="A158" s="6" t="inlineStr">
-        <is>
-          <t>1. Endless swordsmanship drills</t>
-        </is>
-      </c>
+      <c r="A158" s="6" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="6" t="inlineStr">
         <is>
-          <t>2. Physical conditioning beyond normal limits</t>
+          <t>1. Endless swordsmanship drills</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="6" t="inlineStr">
         <is>
-          <t>3. Pain tolerance and endurance</t>
+          <t>2. Physical conditioning beyond normal limits</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="6" t="inlineStr">
         <is>
-          <t>4. Tactical education</t>
+          <t>3. Pain tolerance and endurance</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="6" t="inlineStr">
         <is>
+          <t>4. Tactical education</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="6" t="inlineStr">
+        <is>
           <t>5. Real combat missions (not simulations; death was possible)</t>
         </is>
       </c>
     </row>
-    <row r="163">
-      <c r="A163" s="6" t="inlineStr"/>
-    </row>
     <row r="164">
-      <c r="A164" s="6" t="inlineStr">
+      <c r="A164" s="6" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="165">
-      <c r="A165" s="6" t="inlineStr"/>
-    </row>
     <row r="166">
-      <c r="A166" s="6" t="inlineStr">
+      <c r="A166" s="6" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="6" t="inlineStr">
         <is>
           <t>## Colors, crest, sigil</t>
         </is>
       </c>
     </row>
-    <row r="167">
-      <c r="A167" s="6" t="inlineStr"/>
-    </row>
     <row r="168">
-      <c r="A168" s="6" t="inlineStr">
-        <is>
-          <t>| Item | Quick fact |</t>
-        </is>
-      </c>
+      <c r="A168" s="6" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| Item | Quick fact |</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="6" t="inlineStr">
         <is>
-          <t>| Why I wear red + black | I have always loved them; deep reason not revealed to me yet |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="6" t="inlineStr">
         <is>
-          <t>| My crest | Simple child crest: blade/flame between small parent marks |</t>
+          <t>| Why I wear red + black | I have always loved them; deep reason not revealed to me yet |</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="6" t="inlineStr">
         <is>
-          <t>| My sigil | One red/black blade or flame mark |</t>
+          <t>| My crest | Simple child crest: blade/flame between small parent marks |</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="6" t="inlineStr">
         <is>
-          <t>| Crest tradition | Child crest = name + gender + both parents; simpler than parents; unique |</t>
+          <t>| My sigil | One red/black blade or flame mark |</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="6" t="inlineStr">
         <is>
+          <t>| Crest tradition | Child crest = name + gender + both parents; simpler than parents; unique |</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="6" t="inlineStr">
+        <is>
           <t>| Sigil tradition | Same day as crest; one quick seal mark |</t>
         </is>
       </c>
     </row>
-    <row r="175">
-      <c r="A175" s="6" t="inlineStr"/>
-    </row>
     <row r="176">
-      <c r="A176" s="6" t="inlineStr">
+      <c r="A176" s="6" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="6" t="inlineStr">
         <is>
           <t>### Family crest / sigil cheat sheet</t>
         </is>
       </c>
     </row>
-    <row r="177">
-      <c r="A177" s="6" t="inlineStr"/>
-    </row>
     <row r="178">
-      <c r="A178" s="6" t="inlineStr">
-        <is>
-          <t>| Person | Colors | Crest idea | Sigil idea |</t>
-        </is>
-      </c>
+      <c r="A178" s="6" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="6" t="inlineStr">
         <is>
-          <t>|---|---|---|---|</t>
+          <t>| Person | Colors | Crest idea | Sigil idea |</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="6" t="inlineStr">
         <is>
-          <t>| Dolkin | charcoal / iron / bronze | stone arch + hammer | hammer in arch |</t>
+          <t>|---|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="6" t="inlineStr">
         <is>
-          <t>| Fulfein | sage / silver / pale gold | leaf + crescent | leaf into crescent |</t>
+          <t>| Dolkin | charcoal / iron / bronze | stone arch + hammer | hammer in arch |</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="6" t="inlineStr">
         <is>
-          <t>| Dezco | red / black | balanced blade/flame | red/black split blade |</t>
+          <t>| Fulfein | sage / silver / pale gold | leaf + crescent | leaf into crescent |</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="6" t="inlineStr">
         <is>
-          <t>| Kalhien | blue / copper | forward eager mark | forward chevron |</t>
+          <t>| Dezco | red / black | balanced blade/flame | red/black split blade |</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="6" t="inlineStr">
         <is>
+          <t>| Kalhien | blue / copper | forward eager mark | forward chevron |</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="6" t="inlineStr">
+        <is>
           <t>| Astiale | rose / cream / sky | soft bud or star | soft bud/star |</t>
         </is>
       </c>
     </row>
-    <row r="185">
-      <c r="A185" s="6" t="inlineStr"/>
-    </row>
     <row r="186">
-      <c r="A186" s="6" t="inlineStr">
+      <c r="A186" s="6" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="6" t="inlineStr">
         <is>
           <t>Images: `assets/crests/alzenhiem/`</t>
         </is>
       </c>
     </row>
-    <row r="187">
-      <c r="A187" s="6" t="inlineStr"/>
-    </row>
     <row r="188">
-      <c r="A188" s="6" t="inlineStr">
+      <c r="A188" s="6" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="189">
-      <c r="A189" s="6" t="inlineStr"/>
-    </row>
     <row r="190">
-      <c r="A190" s="6" t="inlineStr">
+      <c r="A190" s="6" t="inlineStr"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="6" t="inlineStr">
         <is>
           <t>## Secrets / do not spoil yet</t>
         </is>
       </c>
     </row>
-    <row r="191">
-      <c r="A191" s="6" t="inlineStr"/>
-    </row>
     <row r="192">
-      <c r="A192" s="6" t="inlineStr">
+      <c r="A192" s="6" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="6" t="inlineStr">
         <is>
           <t>Use this when roleplaying what party members know.</t>
         </is>
       </c>
     </row>
-    <row r="193">
-      <c r="A193" s="6" t="inlineStr"/>
-    </row>
     <row r="194">
-      <c r="A194" s="6" t="inlineStr">
-        <is>
-          <t>| Topic | Party can know? | Notes |</t>
-        </is>
-      </c>
+      <c r="A194" s="6" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="6" t="inlineStr">
         <is>
-          <t>|---|---|---|</t>
+          <t>| Topic | Party can know? | Notes |</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="6" t="inlineStr">
         <is>
-          <t>| I am from Alzenhiem + family basics | Yes | Safe to share |</t>
+          <t>|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="6" t="inlineStr">
         <is>
-          <t>| Trained since 8 under the Lion | Yes | Safe to share |</t>
+          <t>| I am from Alzenhiem + family basics | Yes | Safe to share |</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="6" t="inlineStr">
         <is>
-          <t>| People rumored I was Hero early | Yes | Emphasize it was rumor then |</t>
+          <t>| Trained since 8 under the Lion | Yes | Safe to share |</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="6" t="inlineStr">
         <is>
-          <t>| Yua made me Hero at 17 | Yes, if trust is there | She often looks like a pixie |</t>
+          <t>| People rumored I was Hero early | Yes | Emphasize it was rumor then |</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="6" t="inlineStr">
         <is>
-          <t>| Exact red/black blood meaning | No | Yua will tell me later; I do not know yet |</t>
+          <t>| Yua made me Hero at 17 | Yes, if trust is there | She often looks like a pixie |</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="6" t="inlineStr">
         <is>
-          <t>| Mana Well / sword imbue details | Not yet / soon | Yua stayed quiet on purpose; after my Saltrock faceplant she will explain |</t>
+          <t>| Exact red/black blood meaning | No | Yua will tell me later; I do not know yet |</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="6" t="inlineStr">
         <is>
+          <t>| Mana Well / sword imbue details | Not yet / soon | Yua stayed quiet on purpose; after my Saltrock faceplant she will explain |</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="6" t="inlineStr">
+        <is>
           <t>| Full private family crest theology | Optional | Share lightly unless asked |</t>
         </is>
       </c>
     </row>
-    <row r="203">
-      <c r="A203" s="6" t="inlineStr"/>
-    </row>
     <row r="204">
-      <c r="A204" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">**Red/black truth (for you / DM only, not my current knowledge):**  </t>
-        </is>
-      </c>
+      <c r="A204" s="6" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">**Red/black truth (for you / DM only, not my current knowledge):**  </t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="6" t="inlineStr">
+        <is>
           <t>Black = Dwarven caves / void / dark over light. Red = Elven holy blood after ill happens. Together = balance.</t>
         </is>
       </c>
     </row>
-    <row r="206">
-      <c r="A206" s="6" t="inlineStr"/>
-    </row>
     <row r="207">
-      <c r="A207" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">**Mana Well truth (for you / DM; Yua explains after Saltrock biff):**  </t>
-        </is>
-      </c>
+      <c r="A207" s="6" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">**Mana Well truth (for you / DM; Yua explains after Saltrock biff):**  </t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="6" t="inlineStr">
+        <is>
           <t>Mana pool stored within soul confines but separate from the soul. Simple imbue makes sword lighter/sharper and grants a short agility burst. First accidental use: ~15 ft dash mid swing in journal 03, causing the faceplant. Needs training.</t>
         </is>
       </c>
     </row>
-    <row r="209">
-      <c r="A209" s="6" t="inlineStr"/>
-    </row>
     <row r="210">
-      <c r="A210" s="6" t="inlineStr">
+      <c r="A210" s="6" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="211">
-      <c r="A211" s="6" t="inlineStr"/>
-    </row>
     <row r="212">
-      <c r="A212" s="6" t="inlineStr">
+      <c r="A212" s="6" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="6" t="inlineStr">
         <is>
           <t>## Abilities (Mana Well)</t>
         </is>
       </c>
     </row>
-    <row r="213">
-      <c r="A213" s="6" t="inlineStr"/>
-    </row>
     <row r="214">
-      <c r="A214" s="6" t="inlineStr">
-        <is>
-          <t>| Piece | Quick fact |</t>
-        </is>
-      </c>
+      <c r="A214" s="6" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| Piece | Quick fact |</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="6" t="inlineStr">
         <is>
-          <t>| Source | Bestowed by Yua with the Hero charge; unexplained at first |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="6" t="inlineStr">
         <is>
-          <t>| Well | Stored mana pool within soul confines; separate from the soul |</t>
+          <t>| Source | Bestowed by Yua with the Hero charge; unexplained at first |</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="6" t="inlineStr">
         <is>
-          <t>| Simple imbue | Innate; should feel as easy as breathing once understood |</t>
+          <t>| Well | Stored mana pool within soul confines; separate from the soul |</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="6" t="inlineStr">
         <is>
-          <t>| Sword effect | Lighter, sharper; short burst of swiftness / agility |</t>
+          <t>| Simple imbue | Innate; should feel as easy as breathing once understood |</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="6" t="inlineStr">
         <is>
-          <t>| First use | Saltrock battle (journal 03); accidental ~15 ft dash mid swing = faceplant |</t>
+          <t>| Sword effect | Lighter, sharper; short burst of swiftness / agility |</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="6" t="inlineStr">
         <is>
-          <t>| Training needed | Control timing, avoid waste, move with the burst instead of being thrown |</t>
+          <t>| First use | Saltrock battle (journal 03); accidental ~15 ft dash mid swing = faceplant |</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="6" t="inlineStr">
         <is>
+          <t>| Training needed | Control timing, avoid waste, move with the burst instead of being thrown |</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="6" t="inlineStr">
+        <is>
           <t>| Yua’s plan | Stay quiet until I ask or figure it out; changed after watching me biff |</t>
         </is>
       </c>
     </row>
-    <row r="223">
-      <c r="A223" s="6" t="inlineStr"/>
-    </row>
     <row r="224">
-      <c r="A224" s="6" t="inlineStr">
+      <c r="A224" s="6" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="225">
-      <c r="A225" s="6" t="inlineStr"/>
-    </row>
     <row r="226">
-      <c r="A226" s="6" t="inlineStr">
+      <c r="A226" s="6" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="6" t="inlineStr">
         <is>
           <t>## How I sound when I talk about myself</t>
         </is>
       </c>
     </row>
-    <row r="227">
-      <c r="A227" s="6" t="inlineStr"/>
-    </row>
     <row r="228">
-      <c r="A228" s="6" t="inlineStr">
-        <is>
-          <t>1. Honest, a little unsure about being chosen</t>
-        </is>
-      </c>
+      <c r="A228" s="6" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" s="6" t="inlineStr">
         <is>
-          <t>2. Proud of Alzenhiem without boasting</t>
+          <t>1. Honest, a little unsure about being chosen</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="6" t="inlineStr">
         <is>
-          <t>3. Corrects “Hero of centuries” rumors for the training years</t>
+          <t>2. Proud of Alzenhiem without boasting</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="6" t="inlineStr">
         <is>
-          <t>4. Speaks kindly about family, especially Astiale</t>
+          <t>3. Corrects “Hero of centuries” rumors for the training years</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="6" t="inlineStr">
         <is>
-          <t>5. Does not claim to understand Yua fully</t>
+          <t>4. Speaks kindly about family, especially Astiale</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="6" t="inlineStr">
         <is>
+          <t>5. Does not claim to understand Yua fully</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="6" t="inlineStr">
+        <is>
           <t>6. Prefers no dramatic dash heavy speech; plain and direct</t>
         </is>
       </c>
     </row>
-    <row r="234">
-      <c r="A234" s="6" t="inlineStr"/>
-    </row>
     <row r="235">
-      <c r="A235" s="6" t="inlineStr">
+      <c r="A235" s="6" t="inlineStr"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="236">
-      <c r="A236" s="6" t="inlineStr"/>
-    </row>
     <row r="237">
-      <c r="A237" s="6" t="inlineStr">
+      <c r="A237" s="6" t="inlineStr"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="6" t="inlineStr">
         <is>
           <t>## Where the long versions are</t>
         </is>
       </c>
     </row>
-    <row r="238">
-      <c r="A238" s="6" t="inlineStr"/>
-    </row>
     <row r="239">
-      <c r="A239" s="6" t="inlineStr">
-        <is>
-          <t>| Need | File |</t>
-        </is>
-      </c>
+      <c r="A239" s="6" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| Need | File |</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="6" t="inlineStr">
         <is>
-          <t>| Full character intro | `character/lore/dezco-knoleburn-character.md` |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="6" t="inlineStr">
         <is>
-          <t>| Journal index | `character/lore/journal/README.md` |</t>
+          <t>| Full character intro | `character/lore/dezco-knoleburn-character.md` |</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="6" t="inlineStr">
         <is>
-          <t>| Journal 01 (backstory) | `character/lore/journal/01-after-the-charge.md` |</t>
+          <t>| Journal index | `character/lore/journal/README.md` |</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="6" t="inlineStr">
         <is>
-          <t>| Journal 02 (leave home / Saltrock) | `character/lore/journal/02-leaving-home-for-saltrock.md` |</t>
+          <t>| Journal 01 (backstory) | `character/lore/journal/01-after-the-charge.md` |</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 (staff falls / mid siege) | `character/lore/journal/03-saltrock-staff-falls.md` |</t>
+          <t>| Journal 02 (leave home / Saltrock) | `character/lore/journal/02-leaving-home-for-saltrock.md` |</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="6" t="inlineStr">
         <is>
-          <t>| Name meanings | `character/lore/knoleburn-names.md` |</t>
+          <t>| Journal 03 (staff falls / mid siege) | `character/lore/journal/03-saltrock-staff-falls.md` |</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="6" t="inlineStr">
         <is>
-          <t>| Crest / sigil deep meanings | `assets/crests/alzenhiem/README.md` |</t>
+          <t>| Name meanings | `character/lore/knoleburn-names.md` |</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="6" t="inlineStr">
         <is>
-          <t>| Yua story plots index | `character/lore/yua-story-plots/README.md` |</t>
+          <t>| Crest / sigil deep meanings | `assets/crests/alzenhiem/README.md` |</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="6" t="inlineStr">
         <is>
-          <t>| Red/black reveal (future) | `character/lore/yua-story-plots/yua-on-red-and-black.md` |</t>
+          <t>| Yua story plots index | `character/lore/yua-story-plots/README.md` |</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="6" t="inlineStr">
         <is>
+          <t>| Red/black reveal (future) | `character/lore/yua-story-plots/yua-on-red-and-black.md` |</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="6" t="inlineStr">
+        <is>
           <t>| Mana Well / sword imbue | `character/lore/yua-story-plots/yua-mana-well.md` |</t>
         </is>
       </c>
-    </row>
-    <row r="251">
-      <c r="A251" s="6" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" s="6" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>| Downloadable Google export | `character/lore/exports/` (Sheets tabs `.xlsx` + Docs `.docx`) |</t>
         </is>
       </c>
     </row>
@@ -6572,7 +6586,7 @@
     <row r="254">
       <c r="A254" s="6" t="inlineStr">
         <is>
-          <t>## Blank lines for new party facts</t>
+          <t>---</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6596,7 @@
     <row r="256">
       <c r="A256" s="6" t="inlineStr">
         <is>
-          <t>Add new rows here whenever something new becomes true in play:</t>
+          <t>## Blank lines for new party facts</t>
         </is>
       </c>
     </row>
@@ -6592,75 +6606,99 @@
     <row r="258">
       <c r="A258" s="6" t="inlineStr">
         <is>
-          <t>| Date / session | New fact | Share with party? |</t>
+          <t>Add new rows here whenever something new becomes true in play:</t>
         </is>
       </c>
     </row>
     <row r="259">
-      <c r="A259" s="6" t="inlineStr">
-        <is>
-          <t>|---|---|---|</t>
-        </is>
-      </c>
+      <c r="A259" s="6" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" s="6" t="inlineStr">
         <is>
-          <t>| Journal 02 | Left Alzenhiem with Dolkin’s sword + smithing tools; Fulfein’s gold, pot, clothes, shovel | Yes |</t>
+          <t>| Date / session | New fact | Share with party? |</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="6" t="inlineStr">
         <is>
-          <t>| Journal 02 | Shovel is mom’s bathroom dig joke first; burial meaning is the quiet second read | Optional / tonal |</t>
+          <t>|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="6" t="inlineStr">
         <is>
-          <t>| Journal 02 | In Saltrock tavern overnight; knows the floating protective staff | Yes |</t>
+          <t>| Journal 02 | Left Alzenhiem with Dolkin’s sword + smithing tools; Fulfein’s gold, pot, clothes, shovel | Yes |</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Saltrock staff fell; crabs + creatures attacked | Yes |</t>
+          <t>| Journal 02 | Shovel is mom’s bathroom dig joke first; burial meaning is the quiet second read | Optional / tonal |</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Missed a short bow creature; faceplant; nearly shot; saved by elf girl archer | Yes |</t>
+          <t>| Journal 02 | In Saltrock tavern overnight; knows the floating protective staff | Yes |</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Faceplant tied to accidental ~15 ft mana dash / simple imbue (not understood yet) | After Yua explains |</t>
+          <t>| Journal 03 | Saltrock staff fell; crabs + creatures attacked | Yes |</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Sealed in general building with townsfolk; people outside unknown; story paused mid siege | Yes |</t>
+          <t>| Journal 03 | Missed a short bow creature; faceplant; nearly shot; saved by elf girl archer | Yes |</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="6" t="inlineStr">
         <is>
-          <t>| Yua plots | Mana Well bestowed at Hero charge; Yua will explain after watching the biff | After she tells me |</t>
+          <t>| Journal 03 | Faceplant tied to accidental ~15 ft mana dash / simple imbue (not understood yet) | After Yua explains |</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="6" t="inlineStr">
+        <is>
+          <t>| Journal 03 | Sealed in general building with townsfolk; people outside unknown; story paused mid siege | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="6" t="inlineStr">
+        <is>
+          <t>| Yua plots | Mana Well bestowed at Hero charge; Yua will explain after watching the biff | After she tells me |</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="6" t="inlineStr">
+        <is>
+          <t>| Lore | Birthday is November 6 | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="6" t="inlineStr">
+        <is>
+          <t>| Export | Tabbed Sheets + Docs lore pack in character/lore/exports/ | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="6" t="inlineStr">
         <is>
           <t>| | | |</t>
         </is>

</xml_diff>

<commit_message>
Clarify Dezco’s trainer as Rilock under the King’s Lion
The King’s Lion witnessed Yua and directed training; Rilock, royal
master swordsman of his guard, is the day to day master. Update journal,
party reference, character intro, and regenerate Google exports.

Co-authored-by: Dralorex <Dralorex@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/character/lore/exports/Dezco_Knoleburn_Lore_Tabs.xlsx
+++ b/character/lore/exports/Dezco_Knoleburn_Lore_Tabs.xlsx
@@ -1141,7 +1141,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>When I left for military training at eight years old, Alzenhiem was the last soft place my hands remembered. The yard taught me how to stand. Alzenhiem taught me what I was standing for. On hard nights under the Lion, I did not dream of glory. I dreamed of the lane behind our house, of my mother’s voice through an open window, of my father’s shadow crossing the doorway at dusk.</t>
+          <t>When I left for military training at eight years old, Alzenhiem was the last soft place my hands remembered. The yard taught me how to stand. Alzenhiem taught me what I was standing for. On hard nights under Rilock, I did not dream of glory. I dreamed of the lane behind our house, of my mother’s voice through an open window, of my father’s shadow crossing the doorway at dusk.</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>She calls me home even when the rest of the realm calls me other things. To Astiale I am not a rumor, not a prophecy, not the Lion’s apprentice. I am her older brother who comes and goes, who kneels so she can reach me, who pretends not to notice when she hides behind Fulfein for the first minute and then refuses to let go for the last.</t>
+          <t>She calls me home even when the rest of the realm calls me other things. To Astiale I am not a rumor, not a prophecy, not Rilock’s student or the Lion’s chosen trainee. I am her older brother who comes and goes, who kneels so she can reach me, who pretends not to notice when she hides behind Fulfein for the first minute and then refuses to let go for the last.</t>
         </is>
       </c>
     </row>
@@ -1554,7 +1554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A165"/>
+  <dimension ref="A1:A167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1641,7 +1641,7 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Before the yard, before the Lion, before anyone called me anything larger than my name, there was Alzenhiem. My father Dolkin. My mother Fulfein. My brother Kalhien. Later, my sister Astiale. I carry them through every page that follows, even when I do not write their names.</t>
+          <t>Before the yard, before the Lion’s order, before Rilock’s training, before anyone called me anything larger than my name, there was Alzenhiem. My father Dolkin. My mother Fulfein. My brother Kalhien. Later, my sister Astiale. I carry them through every page that follows, even when I do not write their names.</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2011,7 @@
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>## The King’s Lion</t>
+          <t>## The King’s Lion and Rilock</t>
         </is>
       </c>
     </row>
@@ -2041,7 +2041,7 @@
     <row r="96">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>He accepted me as his personal apprentice.</t>
+          <t>He did not take me as his personal apprentice.</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>Many believed Yua’s appearance marked the beginning of an ancient prophecy long thought impossible. Her kind had not been seen for hundreds of years. If she had returned, if she had chosen, then the old stories were no longer stories. They were warnings. Or promises. Or both.</t>
+          <t>Instead, the Lion directed one of his royal guard to train me: Rilock, the royal master swordsman. If the Lion was the will that chose my path, Rilock was the steel that carved it. The Lion pointed. Rilock taught. That distinction mattered to me even when the realm blurred it.</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2061,7 @@
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>I did not feel like prophecy.</t>
+          <t>Many believed Yua’s appearance marked the beginning of an ancient prophecy long thought impossible. Her kind had not been seen for hundreds of years. If she had returned, if she had chosen, then the old stories were no longer stories. They were warnings. Or promises. Or both.</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2071,7 @@
     <row r="102">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>I felt like a boy who had been handed a future too large for his hands.</t>
+          <t>I did not feel like prophecy.</t>
         </is>
       </c>
     </row>
@@ -2081,7 +2081,7 @@
     <row r="104">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>The Lion did not care what I felt. He cared what I would become.</t>
+          <t>I felt like a boy who had been handed a future too large for his hands.</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2091,7 @@
     <row r="106">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>## Years Under the Lion (Twelve to Seventeen)</t>
+          <t>The Lion did not care what I felt. He cared what I would become. Rilock cared how I would survive becoming it.</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
     <row r="108">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>Training under the King’s Lion was merciless.</t>
+          <t>## Years Under Rilock (Twelve to Seventeen)</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2111,7 @@
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>Endless swordsmanship drills until form lived in muscle instead of thought. Physical conditioning beyond what any ordinary human body should endure. Pain tolerance and endurance until pain became information, not a reason to stop. Tactical education: maps, supply lines, the cruel arithmetic of when to hold and when to cut. And real combat missions throughout the kingdom, each one harder than the last.</t>
+          <t>Training under Rilock was merciless.</t>
         </is>
       </c>
     </row>
@@ -2121,7 +2121,7 @@
     <row r="112">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>These were never simulations.</t>
+          <t>Endless swordsmanship drills until form lived in muscle instead of thought. Physical conditioning beyond what any ordinary human body should endure. Pain tolerance and endurance until pain became information, not a reason to stop. Tactical education: maps, supply lines, the cruel arithmetic of when to hold and when to cut. And real combat missions throughout the kingdom, each one harder than the last. The Lion’s direction hung over the work like a seal. Rilock’s hands did the forging.</t>
         </is>
       </c>
     </row>
@@ -2131,7 +2131,7 @@
     <row r="114">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>Every assignment carried the possibility of death. My master believed that growth stolen from practice alone was fragile growth, and that only experience with blood in it could forge something that would not shatter when the world pressed back.</t>
+          <t>These were never simulations.</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2141,7 @@
     <row r="116">
       <c r="A116" s="6" t="inlineStr">
         <is>
-          <t>I nearly died more times than I care to count. I saved people whose names I still remember. I failed people whose names I remember better. Each successful mission spread my reputation farther across the kingdoms, whether I wanted it or not.</t>
+          <t>Every assignment carried the possibility of death. My master believed that growth stolen from practice alone was fragile growth, and that only experience with blood in it could forge something that would not shatter when the world pressed back.</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
     <row r="118">
       <c r="A118" s="6" t="inlineStr">
         <is>
-          <t>Before I reached fifteen, my name was already known throughout much of the realm.</t>
+          <t>I nearly died more times than I care to count. I saved people whose names I still remember. I failed people whose names I remember better. Each successful mission spread my reputation farther across the kingdoms, whether I wanted it or not.</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2161,7 @@
     <row r="120">
       <c r="A120" s="6" t="inlineStr">
         <is>
-          <t>That is when the stories turned wrong.</t>
+          <t>Before I reached fifteen, my name was already known throughout much of the realm.</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
     <row r="122">
       <c r="A122" s="6" t="inlineStr">
         <is>
-          <t>They did not only speak of the Lion’s apprentice. They spoke of me as the Hero of centuries. The one prophecy had waited for. The boy marked by a forgotten being. The answer to fading magic. Red and black on a battlefield, moving faster than sense allowed, as if destiny itself had dressed me for the part. Inns repeated it. Markets sold it. Soldiers whispered it like a comfort they could not afford to question.</t>
+          <t>That is when the stories turned wrong.</t>
         </is>
       </c>
     </row>
@@ -2181,7 +2181,7 @@
     <row r="124">
       <c r="A124" s="6" t="inlineStr">
         <is>
-          <t>I was no such thing.</t>
+          <t>They spoke of the Lion’s apprentice, as if I had trained at the Lion’s hip. Closer to truth: I trained under Rilock by the Lion’s order. Then the stories grew teeth. They spoke of me as the Hero of centuries. The one prophecy had waited for. The boy marked by a forgotten being. The answer to fading magic. Red and black on a battlefield, moving faster than sense allowed, as if destiny itself had dressed me for the part. Inns repeated it. Markets sold it. Soldiers whispered it like a comfort they could not afford to question.</t>
         </is>
       </c>
     </row>
@@ -2191,7 +2191,7 @@
     <row r="126">
       <c r="A126" s="6" t="inlineStr">
         <is>
-          <t>In those years I had no blessing that made me a Hero. No ancient title. No sacred charge. Only pure training under a merciless master, and whatever skill pain and survival could carve into me. The duel in the yard had been real. The Lion’s choice had been real. The sweat, the blood, the missions that could have killed me: all real. The rest was a fabrication that spread from people’s own ideas and rumors, grown fat on hope and fear and the hunger for a legend the world had gone too long without.</t>
+          <t>I was no such thing.</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2201,7 @@
     <row r="128">
       <c r="A128" s="6" t="inlineStr">
         <is>
-          <t>I tried, once or twice, to correct it. It never mattered. A boy denying a prophecy only sounds like humility to those who already believe. So I trained. I fought. I lived. I let their story walk ahead of me like a stranger wearing my face.</t>
+          <t>In those years I had no blessing that made me a Hero. No ancient title. No sacred charge. Only pure training under a merciless master, and whatever skill pain and survival could carve into me. The duel in the yard had been real. The Lion’s direction had been real. Rilock’s teaching had been real. The sweat, the blood, the missions that could have killed me: all real. The rest was a fabrication that spread from people’s own ideas and rumors, grown fat on hope and fear and the hunger for a legend the world had gone too long without.</t>
         </is>
       </c>
     </row>
@@ -2211,7 +2211,7 @@
     <row r="130">
       <c r="A130" s="6" t="inlineStr">
         <is>
-          <t>And still, as more people came to know my name, Yua’s favor toward me continued to grow. Not because their rumors were true. Not as a prize for a title I did not hold. As a bond. Lives saved. Selflessness chosen when selfishness would have been easier. Hope placed in me by strangers who had never seen my face, even when that hope was aimed at a Hero I was not yet, and somehow, through that hope, she grew stronger beside me.</t>
+          <t>I tried, once or twice, to correct it. It never mattered. A boy denying a prophecy only sounds like humility to those who already believe. So I trained. I fought. I lived. I let their story walk ahead of me like a stranger wearing my face.</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2221,7 @@
     <row r="132">
       <c r="A132" s="6" t="inlineStr">
         <is>
-          <t>I still rarely saw her clearly in those years. A flicker at the edge of campfire light. A presence in the breath before a fight I should not have survived. Always near. Almost never held. She did not step forward to crown their rumor. She let me become something first, the hard way.</t>
+          <t>And still, as more people came to know my name, Yua’s favor toward me continued to grow. Not because their rumors were true. Not as a prize for a title I did not hold. As a bond. Lives saved. Selflessness chosen when selfishness would have been easier. Hope placed in me by strangers who had never seen my face, even when that hope was aimed at a Hero I was not yet, and somehow, through that hope, she grew stronger beside me.</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2231,7 @@
     <row r="134">
       <c r="A134" s="6" t="inlineStr">
         <is>
-          <t>## The Title of Hero</t>
+          <t>I still rarely saw her clearly in those years. A flicker at the edge of campfire light. A presence in the breath before a fight I should not have survived. Always near. Almost never held. She did not step forward to crown their rumor. She let me become something first, the hard way.</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2241,7 @@
     <row r="136">
       <c r="A136" s="6" t="inlineStr">
         <is>
-          <t>At seventeen, after years of relentless training, my master declared that I had learned everything he could teach. It was time for me to venture into the world and help restore the peace.</t>
+          <t>## The Title of Hero</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
         <is>
-          <t>He meant to name me his successor.</t>
+          <t>At seventeen, after years of relentless training, my master Rilock declared that I had learned everything he could teach. It was time for me to venture into the world and help restore the peace.</t>
         </is>
       </c>
     </row>
@@ -2261,7 +2261,7 @@
     <row r="140">
       <c r="A140" s="6" t="inlineStr">
         <is>
-          <t>Until that day, Hero had been other people’s word for me. A rumor. A fabrication. Then Yua appeared once more, this time before both of us, and the word stopped belonging only to strangers.</t>
+          <t>He meant to name me his successor.</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
     <row r="142">
       <c r="A142" s="6" t="inlineStr">
         <is>
-          <t>For the first time in centuries, she openly revealed herself to another witness and did not run from my gaze. No trick at the corner of the eye. No vanishing when I turned. She stood there, ancient and present, and I finally understood that every shadow I had doubted since I was eight years old had been her choosing me in silence.</t>
+          <t>Until that day, Hero had been other people’s word for me. A rumor. A fabrication. Then Yua appeared once more, this time before Rilock and me, with the King’s Lion present as the one who had set this path in motion, and the word stopped belonging only to strangers.</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2281,7 @@
     <row r="144">
       <c r="A144" s="6" t="inlineStr">
         <is>
-          <t>Standing before the King’s Lion, she bestowed upon me the ancient title of Hero.</t>
+          <t>For the first time in centuries, she openly revealed herself to other witnesses and did not run from my gaze. No trick at the corner of the eye. No vanishing when I turned. She stood there, ancient and present, and I finally understood that every shadow I had doubted since I was eight years old had been her choosing me in silence.</t>
         </is>
       </c>
     </row>
@@ -2291,7 +2291,7 @@
     <row r="146">
       <c r="A146" s="6" t="inlineStr">
         <is>
-          <t>She entrusted me with a sacred mission:</t>
+          <t>Standing before the King’s Lion and my master Rilock, she bestowed upon me the ancient title of Hero.</t>
         </is>
       </c>
     </row>
@@ -2301,45 +2301,45 @@
     <row r="148">
       <c r="A148" s="6" t="inlineStr">
         <is>
-          <t>1. Restore magic before it disappears completely.</t>
+          <t>She entrusted me with a sacred mission:</t>
         </is>
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="6" t="inlineStr">
-        <is>
-          <t>2. Stand against the darkness consuming the world.</t>
-        </is>
-      </c>
+      <c r="A149" s="6" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="6" t="inlineStr">
         <is>
-          <t>3. Unite the fractured kingdoms and races.</t>
+          <t>1. Restore magic before it disappears completely.</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="6" t="inlineStr">
         <is>
-          <t>4. Become the symbol of hope the world has long forgotten.</t>
+          <t>2. Stand against the darkness consuming the world.</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="6" t="inlineStr">
         <is>
-          <t>5. Bring together the two halves of the world.</t>
+          <t>3. Unite the fractured kingdoms and races.</t>
         </is>
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="6" t="inlineStr"/>
+      <c r="A153" s="6" t="inlineStr">
+        <is>
+          <t>4. Become the symbol of hope the world has long forgotten.</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="6" t="inlineStr">
         <is>
-          <t>My master gave his blessing. Yua gave her charge. I left my training behind, not as a student, but as the first Hero the world had seen in generations.</t>
+          <t>5. Bring together the two halves of the world.</t>
         </is>
       </c>
     </row>
@@ -2349,7 +2349,7 @@
     <row r="156">
       <c r="A156" s="6" t="inlineStr">
         <is>
-          <t>Yua joins me on this adventure. She aids me in the times I fall short. Most days she appears only as the shape of a small pixie, light enough to perch near my shoulder, old enough to remember when the world still believed magic would last forever.</t>
+          <t>My master gave his blessing. The Lion’s silence felt like permission edged in steel. Yua gave her charge. I left my training behind, not as a student, but as the first Hero the world had seen in generations.</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
     <row r="158">
       <c r="A158" s="6" t="inlineStr">
         <is>
-          <t>I am seventeen. Five foot ten. Slender. Black hair. Half of one people and half of another, carrying red and black into a world that has forgotten how to hope. Somewhere behind all of that, Alzenhiem is still waiting: Dolkin, Fulfein, Kalhien, and sweet Astiale, who should never have to learn my title before she learns my face.</t>
+          <t>Yua joins me on this adventure. She aids me in the times I fall short. Most days she appears only as the shape of a small pixie, light enough to perch near my shoulder, old enough to remember when the world still believed magic would last forever.</t>
         </is>
       </c>
     </row>
@@ -2369,7 +2369,7 @@
     <row r="160">
       <c r="A160" s="6" t="inlineStr">
         <is>
-          <t>I still don’t fully understand why I was chosen.</t>
+          <t>I am seventeen. Five foot ten. Slender. Black hair. Half of one people and half of another, carrying red and black into a world that has forgotten how to hope. Somewhere behind all of that, Alzenhiem is still waiting: Dolkin, Fulfein, Kalhien, and sweet Astiale, who should never have to learn my title before she learns my face.</t>
         </is>
       </c>
     </row>
@@ -2379,7 +2379,7 @@
     <row r="162">
       <c r="A162" s="6" t="inlineStr">
         <is>
-          <t>But I am writing this so that if I fail, or if I don’t, there will be a record of how it began: with a boy from a small hamlet, a yard that tried to remake him, a rival who thought destiny belonged only to him, a Lion who saw what others missed, and a forgotten being who broke an oath older than kingdoms because magic was dying… and because, for reasons I may never earn, she looked at me and decided the world was not finished yet.</t>
+          <t>I still don’t fully understand why I was chosen.</t>
         </is>
       </c>
     </row>
@@ -2389,12 +2389,22 @@
     <row r="164">
       <c r="A164" s="6" t="inlineStr">
         <is>
+          <t>But I am writing this so that if I fail, or if I don’t, there will be a record of how it began: with a boy from a small hamlet, a yard that tried to remake him, a rival who thought destiny belonged only to him, a Lion who saw what others missed, a royal master swordsman named Rilock who made the seeing into training, and a forgotten being who broke an oath older than kingdoms because magic was dying… and because, for reasons I may never earn, she looked at me and decided the world was not finished yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="6" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="6" t="inlineStr">
+        <is>
           <t>*Dezco Knoleburn of Alzenhiem*</t>
         </is>
       </c>
     </row>
-    <row r="165">
-      <c r="A165" s="6" t="inlineStr">
+    <row r="167">
+      <c r="A167" s="6" t="inlineStr">
         <is>
           <t>*Hero, whether I am ready or not*</t>
         </is>
@@ -5049,7 +5059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A272"/>
+  <dimension ref="A1:A275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -5099,7 +5109,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">**Last updated:** 2026-07-25 (Google Drive lore export pack added)  </t>
+          <t xml:space="preserve">**Last updated:** 2026-07-26 (trainer clarified: Rilock under the King’s Lion)  </t>
         </is>
       </c>
     </row>
@@ -5136,7 +5146,7 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>&gt; I’m Dezco Knoleburn. Seventeen. From a hamlet called Alzenhiem. Dwarven and Elven blood. Trained since I was eight under the King’s Lion. People called me Hero for years before it was true. Yua made it true at seventeen. I love red and black. I’m trying my best.</t>
+          <t>&gt; I’m Dezco Knoleburn. Seventeen. From a hamlet called Alzenhiem. Dwarven and Elven blood. Trained since twelve by Rilock, royal master swordsman, by order of the King’s Lion. People called me Hero for years before it was true. Yua made it true at seventeen. I love red and black. I’m trying my best.</t>
         </is>
       </c>
     </row>
@@ -5257,513 +5267,517 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>| Master | The King’s Lion |</t>
+          <t>| Master / trainer | Rilock (royal master swordsman; King’s Lion royal guard) |</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>| Companion | Yua (often appears as a small pixie) |</t>
+          <t>| Directed by | The King’s Lion (ordered Rilock to train me) |</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>| Crest colors | crimson red + deep black |</t>
+          <t>| Companion | Yua (often appears as a small pixie) |</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>| Sigil | vertical blade / flame split red and black |</t>
+          <t>| Crest colors | crimson red + deep black |</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>| Current location | Saltrock general building (doors sealed; under attack) |</t>
+          <t>| Sigil | vertical blade / flame split red and black |</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
+          <t>| Current location | Saltrock general building (doors sealed; under attack) |</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
           <t>| Travel status | Adventure day 2 gone wrong; protective staff fell; mid siege |</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr"/>
-    </row>
     <row r="42">
-      <c r="A42" s="6" t="inlineStr">
+      <c r="A42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr"/>
-    </row>
     <row r="44">
-      <c r="A44" s="6" t="inlineStr">
+      <c r="A44" s="6" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>## What I am / am not</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="6" t="inlineStr"/>
-    </row>
     <row r="46">
-      <c r="A46" s="6" t="inlineStr">
-        <is>
-          <t>| True | Not true (or not yet) |</t>
-        </is>
-      </c>
+      <c r="A46" s="6" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| True | Not true (or not yet) |</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>| Hero by Yua’s formal charge at age 17 | Born already crowned as Hero |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>| Trained hard under the King’s Lion | Famous because of easy blessing alone |</t>
+          <t>| Hero by Yua’s formal charge at age 17 | Born already crowned as Hero |</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>| People rumored I was the Hero of centuries during ages 12 to 17 | Those years were title + sacred charge (they were rumor) |</t>
+          <t>| Trained hard under Rilock by the Lion’s order | Trained personally day to day by the King’s Lion himself |</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>| Yua watched me from childhood | I always understood why she chose me |</t>
+          <t>| People rumored I was the Hero of centuries during ages 12 to 17 | Those years were title + sacred charge (they were rumor) |</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>| I love red and black | I already know the deep reason why (Yua has not told me yet) |</t>
+          <t>| Yua watched me from childhood | I always understood why she chose me |</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>| Yua set a Mana Well in me when she made me Hero | I understood it before Saltrock (I did not) |</t>
+          <t>| I love red and black | I already know the deep reason why (Yua has not told me yet) |</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
+          <t>| Yua set a Mana Well in me when she made me Hero | I understood it before Saltrock (I did not) |</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
           <t>| I accidentally used a simple imbue in Saltrock | I meant to dash 15 feet and faceplant on purpose |</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="6" t="inlineStr"/>
-    </row>
     <row r="56">
-      <c r="A56" s="6" t="inlineStr">
+      <c r="A56" s="6" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="6" t="inlineStr"/>
-    </row>
     <row r="58">
-      <c r="A58" s="6" t="inlineStr">
+      <c r="A58" s="6" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
         <is>
           <t>## Family (quick)</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="6" t="inlineStr"/>
-    </row>
     <row r="60">
-      <c r="A60" s="6" t="inlineStr">
-        <is>
-          <t>| Person | Who | Age | Name means | Colors | One line |</t>
-        </is>
-      </c>
+      <c r="A60" s="6" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>|---|---|---|---|---|---|</t>
+          <t>| Person | Who | Age | Name means | Colors | One line |</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>| Dolkin | Father | 38 | steadfast of kin | charcoal, iron, bronze | Steady, Dwarven depth, sent me to train to keep me alive |</t>
+          <t>|---|---|---|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>| Fulfein | Mother | 36 | full fair light | sage, silver, pale gold | Warm Elven grace; Alzenhiem’s center for me |</t>
+          <t>| Dolkin | Father | 38 | steadfast of kin | charcoal, iron, bronze | Steady, Dwarven depth, sent me to train to keep me alive |</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>| Kalhien | Younger brother | 15 | rises in pursuit | ink blue + copper | Restless, proud, does not want to be only “Dezco’s brother” |</t>
+          <t>| Fulfein | Mother | 36 | full fair light | sage, silver, pale gold | Warm Elven grace; Alzenhiem’s center for me |</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
+          <t>| Kalhien | Younger brother | 15 | rises in pursuit | ink blue + copper | Restless, proud, does not want to be only “Dezco’s brother” |</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
           <t>| Astiale | Younger sister | 8 | gentle star | rose, cream, sky | Sweet; not born when I left at 8 |</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="6" t="inlineStr"/>
-    </row>
     <row r="67">
-      <c r="A67" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">**Surname Knoleburn means:** stream by the knoll  </t>
-        </is>
-      </c>
+      <c r="A67" s="6" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">**Surname Knoleburn means:** stream by the knoll  </t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
           <t>**Alzenhiem means:** sheltered home under a kind sky</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="6" t="inlineStr"/>
-    </row>
     <row r="70">
-      <c r="A70" s="6" t="inlineStr">
+      <c r="A70" s="6" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="6" t="inlineStr"/>
-    </row>
     <row r="72">
-      <c r="A72" s="6" t="inlineStr">
+      <c r="A72" s="6" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
         <is>
           <t>## Home</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="6" t="inlineStr"/>
-    </row>
     <row r="74">
-      <c r="A74" s="6" t="inlineStr">
-        <is>
-          <t>| | |</t>
-        </is>
-      </c>
+      <c r="A74" s="6" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| | |</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>| Place | Alzenhiem |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>| Type | Small hamlet |</t>
+          <t>| Place | Alzenhiem |</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>| Vibe | Dirt paths, low roofs, neighbors first, no royal banners |</t>
+          <t>| Type | Small hamlet |</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>| Why it matters | What I stand for when I talk about hope |</t>
+          <t>| Vibe | Dirt paths, low roofs, neighbors first, no royal banners |</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>| Town flag colors | wheat gold, meadow green, earth brown, cream |</t>
+          <t>| Why it matters | What I stand for when I talk about hope |</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
+          <t>| Town flag colors | wheat gold, meadow green, earth brown, cream |</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
           <t>| Town flag idea | roof + wheat + lane |</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="6" t="inlineStr"/>
-    </row>
     <row r="83">
-      <c r="A83" s="6" t="inlineStr">
+      <c r="A83" s="6" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="6" t="inlineStr"/>
-    </row>
     <row r="85">
-      <c r="A85" s="6" t="inlineStr">
+      <c r="A85" s="6" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr">
         <is>
           <t>## Timeline (memorize this order)</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="6" t="inlineStr"/>
-    </row>
     <row r="87">
-      <c r="A87" s="6" t="inlineStr">
-        <is>
-          <t>| Age | What happened |</t>
-        </is>
-      </c>
+      <c r="A87" s="6" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| Age | What happened |</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>| 0 | Born November 6; named Dezco; red/black crest + sigil at birth |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>| 8 | Left Alzenhiem for military training; Kalhien was 6; Astiale not born yet |</t>
+          <t>| 0 | Born November 6; named Dezco; red/black crest + sigil at birth |</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>| 8 to 12 | Overshadowed by a stronger rival; Yua watched unseen |</t>
+          <t>| 8 | Left Alzenhiem for military training; Kalhien was 6; Astiale not born yet |</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>| 12 | Rival (nearly 18) dueled me; Yua secretly blessed my speed/strength; only the King’s Lion truly saw her |</t>
+          <t>| 8 to 12 | Overshadowed by a stronger rival; Yua watched unseen |</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>| 12 | Became the King’s Lion’s personal apprentice |</t>
+          <t>| 12 | Rival (nearly 18) dueled me; Yua secretly blessed my speed/strength; only the King’s Lion truly saw her |</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>| 12 to 17 | Merciless real missions; reputation spread; people falsely called me Hero of centuries |</t>
+          <t>| 12 | King’s Lion directed royal master swordsman Rilock (royal guard) to train me |</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>| Before 15 | Name known across much of the realm |</t>
+          <t>| 12 to 17 | Merciless real missions under Rilock; reputation spread; people falsely called me Hero of centuries |</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Master said I had learned all he could teach |</t>
+          <t>| Before 15 | Name known across much of the realm |</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Yua appeared to me and the Lion; gave me the ancient title Hero + sacred mission |</t>
+          <t>| 17 | Master Rilock said I had learned all he could teach |</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Final goodbye at Alzenhiem; family gifts; left for the road |</t>
+          <t>| 17 | Yua appeared before me, Rilock, and the Lion; gave me the ancient title Hero + sacred mission |</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Reached Saltrock; lodging at the tavern; seeking where to travel next |</t>
+          <t>| 17 | Final goodbye at Alzenhiem; family gifts; left for the road |</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Saltrock staff fell; monsters attacked (massive crabs + others) |</t>
+          <t>| 17 | Reached Saltrock; lodging at the tavern; seeking where to travel next |</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Fought with 4 other defenders; missed a short bow creature; saved by an elf girl’s arrow |</t>
+          <t>| 17 | Saltrock staff fell; monsters attacked (massive crabs + others) |</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Barely sealed inside the general building; many townsfolk fate unknown |</t>
+          <t>| 17 | Fought with 4 other defenders; missed a short bow creature; saved by an elf girl’s arrow |</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
+          <t>| 17 | Barely sealed inside the general building; many townsfolk fate unknown |</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="6" t="inlineStr">
+        <is>
           <t>| Now | Trapped in Saltrock general building during the attack; entry open ended |</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="6" t="inlineStr"/>
-    </row>
     <row r="105">
-      <c r="A105" s="6" t="inlineStr">
+      <c r="A105" s="6" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="6" t="inlineStr"/>
-    </row>
     <row r="107">
-      <c r="A107" s="6" t="inlineStr">
+      <c r="A107" s="6" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="6" t="inlineStr">
         <is>
           <t>## Important people (outside family)</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" s="6" t="inlineStr"/>
-    </row>
     <row r="109">
-      <c r="A109" s="6" t="inlineStr">
-        <is>
-          <t>| Person | Who they are to me |</t>
-        </is>
-      </c>
+      <c r="A109" s="6" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| Person | Who they are to me |</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>| Yua | Ancient being tied to magic; broke a millennia oath to act; watched me since childhood; gave me Hero title; often appears as a small pixie |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>| The King’s Lion | King’s greatest swordsman; only one who truly saw Yua at the duel; my master |</t>
+          <t>| Yua | Ancient being tied to magic; broke a millennia oath to act; watched me since childhood; gave me Hero title; often appears as a small pixie |</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>| The Rival | Older trainee who believed he was the chosen one; challenged me at 12; lost after Yua’s hidden aid |</t>
+          <t>| The King’s Lion | King’s greatest swordsman; only one who truly saw Yua at the duel; directed that I be trained |</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>| Elf girl archer | One of 4 defenders in Saltrock attack; pinned a short bow creature through the mouth and into the ground; name not known yet |</t>
+          <t>| Rilock | Royal master swordsman; one of the King’s Lion’s royal guard; my actual trainer/master from ages 12 to 17 |</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>| 3 other defenders | Fought beside us getting townsfolk to the general building; names not known yet |</t>
+          <t>| The Rival | Older trainee who believed he was the chosen one; challenged me at 12; lost after Yua’s hidden aid |</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="6" t="inlineStr"/>
+      <c r="A116" s="6" t="inlineStr">
+        <is>
+          <t>| Elf girl archer | One of 4 defenders in Saltrock attack; pinned a short bow creature through the mouth and into the ground; name not known yet |</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="6" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>| 3 other defenders | Fought beside us getting townsfolk to the general building; names not known yet |</t>
         </is>
       </c>
     </row>
@@ -5773,7 +5787,7 @@
     <row r="119">
       <c r="A119" s="6" t="inlineStr">
         <is>
-          <t>## Current gear / gifts from home</t>
+          <t>---</t>
         </is>
       </c>
     </row>
@@ -5783,66 +5797,66 @@
     <row r="121">
       <c r="A121" s="6" t="inlineStr">
         <is>
-          <t>| Item | From | Notes |</t>
+          <t>## Current gear / gifts from home</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="6" t="inlineStr">
-        <is>
-          <t>|---|---|---|</t>
-        </is>
-      </c>
+      <c r="A122" s="6" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
         <is>
-          <t>| New sword | Dolkin | Hand forged goodbye; his love without saying the words |</t>
+          <t>| Item | From | Notes |</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="6" t="inlineStr">
         <is>
-          <t>| First smithing tools | Dolkin | His original set; “you are the master of your steel” |</t>
+          <t>|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="6" t="inlineStr">
         <is>
-          <t>| 10 gold pieces | Fulfein | Travel money |</t>
+          <t>| New sword | Dolkin | Hand forged goodbye; his love without saying the words |</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="6" t="inlineStr">
         <is>
-          <t>| Cooking pot | Fulfein | Eat warm when you can |</t>
+          <t>| First smithing tools | Dolkin | His original set; “you are the master of your steel” |</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="6" t="inlineStr">
         <is>
-          <t>| New clothing | Fulfein | Wearing them out of respect; left home in them |</t>
+          <t>| 10 gold pieces | Fulfein | Travel money |</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="6" t="inlineStr">
         <is>
-          <t>| Shovel | Fulfein | Funny gift for roadside “number two” duty; also quietly useful if not everyone makes it |</t>
+          <t>| Cooking pot | Fulfein | Eat warm when you can |</t>
         </is>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="6" t="inlineStr"/>
+      <c r="A129" s="6" t="inlineStr">
+        <is>
+          <t>| New clothing | Fulfein | Wearing them out of respect; left home in them |</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="6" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>| Shovel | Fulfein | Funny gift for roadside “number two” duty; also quietly useful if not everyone makes it |</t>
         </is>
       </c>
     </row>
@@ -5852,7 +5866,7 @@
     <row r="132">
       <c r="A132" s="6" t="inlineStr">
         <is>
-          <t>## Places</t>
+          <t>---</t>
         </is>
       </c>
     </row>
@@ -5862,76 +5876,76 @@
     <row r="134">
       <c r="A134" s="6" t="inlineStr">
         <is>
-          <t>| Place | What it is |</t>
+          <t>## Places</t>
         </is>
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="6" t="inlineStr">
-        <is>
-          <t>|---|---|</t>
-        </is>
-      </c>
+      <c r="A135" s="6" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="6" t="inlineStr">
         <is>
-          <t>| Alzenhiem | Home hamlet; my center |</t>
+          <t>| Place | What it is |</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>| Saltrock | Traveling town of people coming and going; I know it well |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
         <is>
-          <t>| Saltrock general building | Holds the protective magic staff; we are sealed inside it during the attack |</t>
+          <t>| Alzenhiem | Home hamlet; my center |</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
         <is>
-          <t>| Saltrock protective staff | Used to float and block named monsters/creatures; has fallen; reason unknown |</t>
+          <t>| Saltrock | Traveling town of people coming and going; I know it well |</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="6" t="inlineStr">
         <is>
-          <t>| Saltrock tavern | Where I lodged the night before the attack; “best bread” only with nostalgia |</t>
+          <t>| Saltrock general building | Holds the protective magic staff; we are sealed inside it during the attack |</t>
         </is>
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="6" t="inlineStr"/>
+      <c r="A141" s="6" t="inlineStr">
+        <is>
+          <t>| Saltrock protective staff | Used to float and block named monsters/creatures; has fallen; reason unknown |</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="6" t="inlineStr">
         <is>
+          <t>| Saltrock tavern | Where I lodged the night before the attack; “best bread” only with nostalgia |</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="6" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">**First magic item I ever saw:** the floating protective staff in Saltrock.  </t>
         </is>
       </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="6" t="inlineStr">
-        <is>
-          <t>**Current crisis:** staff down; crabs and other creatures overran the streets; unknown how many people remain outside.</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="6" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="6" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>**Current crisis:** staff down; crabs and other creatures overran the streets; unknown how many people remain outside.</t>
         </is>
       </c>
     </row>
@@ -5941,7 +5955,7 @@
     <row r="147">
       <c r="A147" s="6" t="inlineStr">
         <is>
-          <t>## My Hero mission (from Yua)</t>
+          <t>---</t>
         </is>
       </c>
     </row>
@@ -5951,45 +5965,45 @@
     <row r="149">
       <c r="A149" s="6" t="inlineStr">
         <is>
-          <t>1. Restore magic before it disappears completely</t>
+          <t>## My Hero mission (from Yua)</t>
         </is>
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="6" t="inlineStr">
-        <is>
-          <t>2. Stand against the darkness consuming the world</t>
-        </is>
-      </c>
+      <c r="A150" s="6" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="6" t="inlineStr">
         <is>
-          <t>3. Unite the fractured kingdoms and races</t>
+          <t>1. Restore magic before it disappears completely</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="6" t="inlineStr">
         <is>
-          <t>4. Become the symbol of hope the world has long forgotten</t>
+          <t>2. Stand against the darkness consuming the world</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="6" t="inlineStr">
         <is>
-          <t>5. Bring together the two halves of the world</t>
+          <t>3. Unite the fractured kingdoms and races</t>
         </is>
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="6" t="inlineStr"/>
+      <c r="A154" s="6" t="inlineStr">
+        <is>
+          <t>4. Become the symbol of hope the world has long forgotten</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="6" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>5. Bring together the two halves of the world</t>
         </is>
       </c>
     </row>
@@ -5999,7 +6013,7 @@
     <row r="157">
       <c r="A157" s="6" t="inlineStr">
         <is>
-          <t>## Training under the Lion included</t>
+          <t>---</t>
         </is>
       </c>
     </row>
@@ -6009,45 +6023,45 @@
     <row r="159">
       <c r="A159" s="6" t="inlineStr">
         <is>
-          <t>1. Endless swordsmanship drills</t>
+          <t>## Training under Rilock included</t>
         </is>
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="6" t="inlineStr">
-        <is>
-          <t>2. Physical conditioning beyond normal limits</t>
-        </is>
-      </c>
+      <c r="A160" s="6" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="6" t="inlineStr">
         <is>
-          <t>3. Pain tolerance and endurance</t>
+          <t>1. Endless swordsmanship drills</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="6" t="inlineStr">
         <is>
-          <t>4. Tactical education</t>
+          <t>2. Physical conditioning beyond normal limits</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="6" t="inlineStr">
         <is>
-          <t>5. Real combat missions (not simulations; death was possible)</t>
+          <t>3. Pain tolerance and endurance</t>
         </is>
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="6" t="inlineStr"/>
+      <c r="A164" s="6" t="inlineStr">
+        <is>
+          <t>4. Tactical education</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="6" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>5. Real combat missions (not simulations; death was possible)</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6071,7 @@
     <row r="167">
       <c r="A167" s="6" t="inlineStr">
         <is>
-          <t>## Colors, crest, sigil</t>
+          <t>---</t>
         </is>
       </c>
     </row>
@@ -6067,59 +6081,59 @@
     <row r="169">
       <c r="A169" s="6" t="inlineStr">
         <is>
-          <t>| Item | Quick fact |</t>
+          <t>## Colors, crest, sigil</t>
         </is>
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="6" t="inlineStr">
-        <is>
-          <t>|---|---|</t>
-        </is>
-      </c>
+      <c r="A170" s="6" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="6" t="inlineStr">
         <is>
-          <t>| Why I wear red + black | I have always loved them; deep reason not revealed to me yet |</t>
+          <t>| Item | Quick fact |</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="6" t="inlineStr">
         <is>
-          <t>| My crest | Simple child crest: blade/flame between small parent marks |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="6" t="inlineStr">
         <is>
-          <t>| My sigil | One red/black blade or flame mark |</t>
+          <t>| Why I wear red + black | I have always loved them; deep reason not revealed to me yet |</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="6" t="inlineStr">
         <is>
-          <t>| Crest tradition | Child crest = name + gender + both parents; simpler than parents; unique |</t>
+          <t>| My crest | Simple child crest: blade/flame between small parent marks |</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="6" t="inlineStr">
         <is>
-          <t>| Sigil tradition | Same day as crest; one quick seal mark |</t>
+          <t>| My sigil | One red/black blade or flame mark |</t>
         </is>
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="6" t="inlineStr"/>
+      <c r="A176" s="6" t="inlineStr">
+        <is>
+          <t>| Crest tradition | Child crest = name + gender + both parents; simpler than parents; unique |</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="6" t="inlineStr">
         <is>
-          <t>### Family crest / sigil cheat sheet</t>
+          <t>| Sigil tradition | Same day as crest; one quick seal mark |</t>
         </is>
       </c>
     </row>
@@ -6129,59 +6143,59 @@
     <row r="179">
       <c r="A179" s="6" t="inlineStr">
         <is>
-          <t>| Person | Colors | Crest idea | Sigil idea |</t>
+          <t>### Family crest / sigil cheat sheet</t>
         </is>
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="6" t="inlineStr">
-        <is>
-          <t>|---|---|---|---|</t>
-        </is>
-      </c>
+      <c r="A180" s="6" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="6" t="inlineStr">
         <is>
-          <t>| Dolkin | charcoal / iron / bronze | stone arch + hammer | hammer in arch |</t>
+          <t>| Person | Colors | Crest idea | Sigil idea |</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="6" t="inlineStr">
         <is>
-          <t>| Fulfein | sage / silver / pale gold | leaf + crescent | leaf into crescent |</t>
+          <t>|---|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="6" t="inlineStr">
         <is>
-          <t>| Dezco | red / black | balanced blade/flame | red/black split blade |</t>
+          <t>| Dolkin | charcoal / iron / bronze | stone arch + hammer | hammer in arch |</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="6" t="inlineStr">
         <is>
-          <t>| Kalhien | blue / copper | forward eager mark | forward chevron |</t>
+          <t>| Fulfein | sage / silver / pale gold | leaf + crescent | leaf into crescent |</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="6" t="inlineStr">
         <is>
-          <t>| Astiale | rose / cream / sky | soft bud or star | soft bud/star |</t>
+          <t>| Dezco | red / black | balanced blade/flame | red/black split blade |</t>
         </is>
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="6" t="inlineStr"/>
+      <c r="A186" s="6" t="inlineStr">
+        <is>
+          <t>| Kalhien | blue / copper | forward eager mark | forward chevron |</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="6" t="inlineStr">
         <is>
-          <t>Images: `assets/crests/alzenhiem/`</t>
+          <t>| Astiale | rose / cream / sky | soft bud or star | soft bud/star |</t>
         </is>
       </c>
     </row>
@@ -6191,7 +6205,7 @@
     <row r="189">
       <c r="A189" s="6" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>Images: `assets/crests/alzenhiem/`</t>
         </is>
       </c>
     </row>
@@ -6201,7 +6215,7 @@
     <row r="191">
       <c r="A191" s="6" t="inlineStr">
         <is>
-          <t>## Secrets / do not spoil yet</t>
+          <t>---</t>
         </is>
       </c>
     </row>
@@ -6211,7 +6225,7 @@
     <row r="193">
       <c r="A193" s="6" t="inlineStr">
         <is>
-          <t>Use this when roleplaying what party members know.</t>
+          <t>## Secrets / do not spoil yet</t>
         </is>
       </c>
     </row>
@@ -6221,107 +6235,107 @@
     <row r="195">
       <c r="A195" s="6" t="inlineStr">
         <is>
-          <t>| Topic | Party can know? | Notes |</t>
+          <t>Use this when roleplaying what party members know.</t>
         </is>
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="6" t="inlineStr">
-        <is>
-          <t>|---|---|---|</t>
-        </is>
-      </c>
+      <c r="A196" s="6" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="6" t="inlineStr">
         <is>
-          <t>| I am from Alzenhiem + family basics | Yes | Safe to share |</t>
+          <t>| Topic | Party can know? | Notes |</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="6" t="inlineStr">
         <is>
-          <t>| Trained since 8 under the Lion | Yes | Safe to share |</t>
+          <t>|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="6" t="inlineStr">
         <is>
-          <t>| People rumored I was Hero early | Yes | Emphasize it was rumor then |</t>
+          <t>| I am from Alzenhiem + family basics | Yes | Safe to share |</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="6" t="inlineStr">
         <is>
-          <t>| Yua made me Hero at 17 | Yes, if trust is there | She often looks like a pixie |</t>
+          <t>| Trained since 8 in the yard; from 12 under Rilock by Lion’s order | Yes | Clarify: Lion directed, Rilock taught |</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="6" t="inlineStr">
         <is>
-          <t>| Exact red/black blood meaning | No | Yua will tell me later; I do not know yet |</t>
+          <t>| People rumored I was Hero early | Yes | Emphasize it was rumor then |</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="6" t="inlineStr">
         <is>
-          <t>| Mana Well / sword imbue details | Not yet / soon | Yua stayed quiet on purpose; after my Saltrock faceplant she will explain |</t>
+          <t>| Yua made me Hero at 17 | Yes, if trust is there | She often looks like a pixie |</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="6" t="inlineStr">
         <is>
-          <t>| Full private family crest theology | Optional | Share lightly unless asked |</t>
+          <t>| Exact red/black blood meaning | No | Yua will tell me later; I do not know yet |</t>
         </is>
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="6" t="inlineStr"/>
+      <c r="A204" s="6" t="inlineStr">
+        <is>
+          <t>| Mana Well / sword imbue details | Not yet / soon | Yua stayed quiet on purpose; after my Saltrock faceplant she will explain |</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="6" t="inlineStr">
         <is>
+          <t>| Full private family crest theology | Optional | Share lightly unless asked |</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="6" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">**Red/black truth (for you / DM only, not my current knowledge):**  </t>
         </is>
       </c>
-    </row>
-    <row r="206">
-      <c r="A206" s="6" t="inlineStr">
-        <is>
-          <t>Black = Dwarven caves / void / dark over light. Red = Elven holy blood after ill happens. Together = balance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" s="6" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" s="6" t="inlineStr">
         <is>
+          <t>Black = Dwarven caves / void / dark over light. Red = Elven holy blood after ill happens. Together = balance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="6" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">**Mana Well truth (for you / DM; Yua explains after Saltrock biff):**  </t>
         </is>
       </c>
-    </row>
-    <row r="209">
-      <c r="A209" s="6" t="inlineStr">
-        <is>
-          <t>Mana pool stored within soul confines but separate from the soul. Simple imbue makes sword lighter/sharper and grants a short agility burst. First accidental use: ~15 ft dash mid swing in journal 03, causing the faceplant. Needs training.</t>
-        </is>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" s="6" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" s="6" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>Mana pool stored within soul confines but separate from the soul. Simple imbue makes sword lighter/sharper and grants a short agility burst. First accidental use: ~15 ft dash mid swing in journal 03, causing the faceplant. Needs training.</t>
         </is>
       </c>
     </row>
@@ -6331,7 +6345,7 @@
     <row r="213">
       <c r="A213" s="6" t="inlineStr">
         <is>
-          <t>## Abilities (Mana Well)</t>
+          <t>---</t>
         </is>
       </c>
     </row>
@@ -6341,73 +6355,73 @@
     <row r="215">
       <c r="A215" s="6" t="inlineStr">
         <is>
-          <t>| Piece | Quick fact |</t>
+          <t>## Abilities (Mana Well)</t>
         </is>
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="6" t="inlineStr">
-        <is>
-          <t>|---|---|</t>
-        </is>
-      </c>
+      <c r="A216" s="6" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" s="6" t="inlineStr">
         <is>
-          <t>| Source | Bestowed by Yua with the Hero charge; unexplained at first |</t>
+          <t>| Piece | Quick fact |</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="6" t="inlineStr">
         <is>
-          <t>| Well | Stored mana pool within soul confines; separate from the soul |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="6" t="inlineStr">
         <is>
-          <t>| Simple imbue | Innate; should feel as easy as breathing once understood |</t>
+          <t>| Source | Bestowed by Yua with the Hero charge; unexplained at first |</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="6" t="inlineStr">
         <is>
-          <t>| Sword effect | Lighter, sharper; short burst of swiftness / agility |</t>
+          <t>| Well | Stored mana pool within soul confines; separate from the soul |</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="6" t="inlineStr">
         <is>
-          <t>| First use | Saltrock battle (journal 03); accidental ~15 ft dash mid swing = faceplant |</t>
+          <t>| Simple imbue | Innate; should feel as easy as breathing once understood |</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="6" t="inlineStr">
         <is>
-          <t>| Training needed | Control timing, avoid waste, move with the burst instead of being thrown |</t>
+          <t>| Sword effect | Lighter, sharper; short burst of swiftness / agility |</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="6" t="inlineStr">
         <is>
-          <t>| Yua’s plan | Stay quiet until I ask or figure it out; changed after watching me biff |</t>
+          <t>| First use | Saltrock battle (journal 03); accidental ~15 ft dash mid swing = faceplant |</t>
         </is>
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="6" t="inlineStr"/>
+      <c r="A224" s="6" t="inlineStr">
+        <is>
+          <t>| Training needed | Control timing, avoid waste, move with the burst instead of being thrown |</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="6" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>| Yua’s plan | Stay quiet until I ask or figure it out; changed after watching me biff |</t>
         </is>
       </c>
     </row>
@@ -6417,7 +6431,7 @@
     <row r="227">
       <c r="A227" s="6" t="inlineStr">
         <is>
-          <t>## How I sound when I talk about myself</t>
+          <t>---</t>
         </is>
       </c>
     </row>
@@ -6427,52 +6441,52 @@
     <row r="229">
       <c r="A229" s="6" t="inlineStr">
         <is>
-          <t>1. Honest, a little unsure about being chosen</t>
+          <t>## How I sound when I talk about myself</t>
         </is>
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="6" t="inlineStr">
-        <is>
-          <t>2. Proud of Alzenhiem without boasting</t>
-        </is>
-      </c>
+      <c r="A230" s="6" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" s="6" t="inlineStr">
         <is>
-          <t>3. Corrects “Hero of centuries” rumors for the training years</t>
+          <t>1. Honest, a little unsure about being chosen</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="6" t="inlineStr">
         <is>
-          <t>4. Speaks kindly about family, especially Astiale</t>
+          <t>2. Proud of Alzenhiem without boasting</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="6" t="inlineStr">
         <is>
-          <t>5. Does not claim to understand Yua fully</t>
+          <t>3. Corrects “Hero of centuries” rumors for the training years</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="6" t="inlineStr">
         <is>
-          <t>6. Prefers no dramatic dash heavy speech; plain and direct</t>
+          <t>4. Speaks kindly about family, especially Astiale</t>
         </is>
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="6" t="inlineStr"/>
+      <c r="A235" s="6" t="inlineStr">
+        <is>
+          <t>5. Does not claim to understand Yua fully</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="6" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>6. Prefers no dramatic dash heavy speech; plain and direct</t>
         </is>
       </c>
     </row>
@@ -6482,7 +6496,7 @@
     <row r="238">
       <c r="A238" s="6" t="inlineStr">
         <is>
-          <t>## Where the long versions are</t>
+          <t>---</t>
         </is>
       </c>
     </row>
@@ -6492,101 +6506,101 @@
     <row r="240">
       <c r="A240" s="6" t="inlineStr">
         <is>
-          <t>| Need | File |</t>
+          <t>## Where the long versions are</t>
         </is>
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="6" t="inlineStr">
-        <is>
-          <t>|---|---|</t>
-        </is>
-      </c>
+      <c r="A241" s="6" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" s="6" t="inlineStr">
         <is>
-          <t>| Full character intro | `character/lore/dezco-knoleburn-character.md` |</t>
+          <t>| Need | File |</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="6" t="inlineStr">
         <is>
-          <t>| Journal index | `character/lore/journal/README.md` |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="6" t="inlineStr">
         <is>
-          <t>| Journal 01 (backstory) | `character/lore/journal/01-after-the-charge.md` |</t>
+          <t>| Full character intro | `character/lore/dezco-knoleburn-character.md` |</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="6" t="inlineStr">
         <is>
-          <t>| Journal 02 (leave home / Saltrock) | `character/lore/journal/02-leaving-home-for-saltrock.md` |</t>
+          <t>| Journal index | `character/lore/journal/README.md` |</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 (staff falls / mid siege) | `character/lore/journal/03-saltrock-staff-falls.md` |</t>
+          <t>| Journal 01 (backstory) | `character/lore/journal/01-after-the-charge.md` |</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="6" t="inlineStr">
         <is>
-          <t>| Name meanings | `character/lore/knoleburn-names.md` |</t>
+          <t>| Journal 02 (leave home / Saltrock) | `character/lore/journal/02-leaving-home-for-saltrock.md` |</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="6" t="inlineStr">
         <is>
-          <t>| Crest / sigil deep meanings | `assets/crests/alzenhiem/README.md` |</t>
+          <t>| Journal 03 (staff falls / mid siege) | `character/lore/journal/03-saltrock-staff-falls.md` |</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="6" t="inlineStr">
         <is>
-          <t>| Yua story plots index | `character/lore/yua-story-plots/README.md` |</t>
+          <t>| Name meanings | `character/lore/knoleburn-names.md` |</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="6" t="inlineStr">
         <is>
-          <t>| Red/black reveal (future) | `character/lore/yua-story-plots/yua-on-red-and-black.md` |</t>
+          <t>| Crest / sigil deep meanings | `assets/crests/alzenhiem/README.md` |</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="6" t="inlineStr">
         <is>
-          <t>| Mana Well / sword imbue | `character/lore/yua-story-plots/yua-mana-well.md` |</t>
+          <t>| Yua story plots index | `character/lore/yua-story-plots/README.md` |</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="6" t="inlineStr">
         <is>
-          <t>| Downloadable Google export | `character/lore/exports/` (Sheets tabs `.xlsx` + Docs `.docx`) |</t>
+          <t>| Red/black reveal (future) | `character/lore/yua-story-plots/yua-on-red-and-black.md` |</t>
         </is>
       </c>
     </row>
     <row r="253">
-      <c r="A253" s="6" t="inlineStr"/>
+      <c r="A253" s="6" t="inlineStr">
+        <is>
+          <t>| Mana Well / sword imbue | `character/lore/yua-story-plots/yua-mana-well.md` |</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="6" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>| Downloadable Google export | `character/lore/exports/` (Sheets tabs `.xlsx` + Docs `.docx`) |</t>
         </is>
       </c>
     </row>
@@ -6596,7 +6610,7 @@
     <row r="256">
       <c r="A256" s="6" t="inlineStr">
         <is>
-          <t>## Blank lines for new party facts</t>
+          <t>---</t>
         </is>
       </c>
     </row>
@@ -6606,7 +6620,7 @@
     <row r="258">
       <c r="A258" s="6" t="inlineStr">
         <is>
-          <t>Add new rows here whenever something new becomes true in play:</t>
+          <t>## Blank lines for new party facts</t>
         </is>
       </c>
     </row>
@@ -6616,89 +6630,106 @@
     <row r="260">
       <c r="A260" s="6" t="inlineStr">
         <is>
-          <t>| Date / session | New fact | Share with party? |</t>
+          <t>Add new rows here whenever something new becomes true in play:</t>
         </is>
       </c>
     </row>
     <row r="261">
-      <c r="A261" s="6" t="inlineStr">
-        <is>
-          <t>|---|---|---|</t>
-        </is>
-      </c>
+      <c r="A261" s="6" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" s="6" t="inlineStr">
         <is>
-          <t>| Journal 02 | Left Alzenhiem with Dolkin’s sword + smithing tools; Fulfein’s gold, pot, clothes, shovel | Yes |</t>
+          <t>| Date / session | New fact | Share with party? |</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="6" t="inlineStr">
         <is>
-          <t>| Journal 02 | Shovel is mom’s bathroom dig joke first; burial meaning is the quiet second read | Optional / tonal |</t>
+          <t>|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="6" t="inlineStr">
         <is>
-          <t>| Journal 02 | In Saltrock tavern overnight; knows the floating protective staff | Yes |</t>
+          <t>| Journal 02 | Left Alzenhiem with Dolkin’s sword + smithing tools; Fulfein’s gold, pot, clothes, shovel | Yes |</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Saltrock staff fell; crabs + creatures attacked | Yes |</t>
+          <t>| Journal 02 | Shovel is mom’s bathroom dig joke first; burial meaning is the quiet second read | Optional / tonal |</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Missed a short bow creature; faceplant; nearly shot; saved by elf girl archer | Yes |</t>
+          <t>| Journal 02 | In Saltrock tavern overnight; knows the floating protective staff | Yes |</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Faceplant tied to accidental ~15 ft mana dash / simple imbue (not understood yet) | After Yua explains |</t>
+          <t>| Journal 03 | Saltrock staff fell; crabs + creatures attacked | Yes |</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Sealed in general building with townsfolk; people outside unknown; story paused mid siege | Yes |</t>
+          <t>| Journal 03 | Missed a short bow creature; faceplant; nearly shot; saved by elf girl archer | Yes |</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="6" t="inlineStr">
         <is>
-          <t>| Yua plots | Mana Well bestowed at Hero charge; Yua will explain after watching the biff | After she tells me |</t>
+          <t>| Journal 03 | Faceplant tied to accidental ~15 ft mana dash / simple imbue (not understood yet) | After Yua explains |</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="6" t="inlineStr">
         <is>
-          <t>| Lore | Birthday is November 6 | Yes |</t>
+          <t>| Journal 03 | Sealed in general building with townsfolk; people outside unknown; story paused mid siege | Yes |</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="6" t="inlineStr">
         <is>
-          <t>| Export | Tabbed Sheets + Docs lore pack in character/lore/exports/ | Yes |</t>
+          <t>| Yua plots | Mana Well bestowed at Hero charge; Yua will explain after watching the biff | After she tells me |</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="6" t="inlineStr">
+        <is>
+          <t>| Lore | Birthday is November 6 | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="6" t="inlineStr">
+        <is>
+          <t>| Export | Tabbed Sheets + Docs lore pack in character/lore/exports/ | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="6" t="inlineStr">
+        <is>
+          <t>| Lore | Trainer is Rilock (royal master swordsman); King’s Lion directed him | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="6" t="inlineStr">
         <is>
           <t>| | | |</t>
         </is>
@@ -6715,7 +6746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -6884,70 +6915,82 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Master</t>
+          <t>Master / trainer</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>The King’s Lion</t>
+          <t>Rilock (royal master swordsman; King’s Lion royal guard)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Companion</t>
+          <t>Directed by</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Yua (often appears as a small pixie)</t>
+          <t>The King’s Lion (ordered Rilock to train me)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Crest colors</t>
+          <t>Companion</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>crimson red + deep black</t>
+          <t>Yua (often appears as a small pixie)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Sigil</t>
+          <t>Crest colors</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>vertical blade / flame split red and black</t>
+          <t>crimson red + deep black</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Current location</t>
+          <t>Sigil</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Saltrock general building (doors sealed; under attack)</t>
+          <t>vertical blade / flame split red and black</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
+          <t>Current location</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Saltrock general building (doors sealed; under attack)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
           <t>Travel status</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Adventure day 2 gone wrong; protective staff fell; mid siege</t>
         </is>
@@ -7489,7 +7532,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Became the King’s Lion’s personal apprentice</t>
+          <t>King’s Lion directed Rilock (royal master swordsman / royal guard) to train Dezco</t>
         </is>
       </c>
     </row>
@@ -7501,7 +7544,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Real missions; false Hero of centuries rumors</t>
+          <t>Real missions under Rilock; false Hero of centuries rumors</t>
         </is>
       </c>
     </row>
@@ -7525,7 +7568,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Master said training was complete</t>
+          <t>Master Rilock said training was complete</t>
         </is>
       </c>
     </row>
@@ -7537,7 +7580,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Yua gave ancient title Hero + sacred mission + Mana Well (unexplained)</t>
+          <t>Yua gave ancient title Hero + sacred mission + Mana Well (unexplained); Lion and Rilock present</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Rilock timing and Hero charge wording errors
Keep Rilock out of the age-8 yard years, restore trained-since-eight
in the party intro, and clarify that Yua laid the Hero charge while
Rilock gave his blessing.

Co-authored-by: Dralorex <Dralorex@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/character/lore/exports/Dezco_Knoleburn_Lore_Tabs.xlsx
+++ b/character/lore/exports/Dezco_Knoleburn_Lore_Tabs.xlsx
@@ -1141,7 +1141,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>When I left for military training at eight years old, Alzenhiem was the last soft place my hands remembered. The yard taught me how to stand. Alzenhiem taught me what I was standing for. On hard nights under Rilock, I did not dream of glory. I dreamed of the lane behind our house, of my mother’s voice through an open window, of my father’s shadow crossing the doorway at dusk.</t>
+          <t>When I left for military training at eight years old, Alzenhiem was the last soft place my hands remembered. The yard taught me how to stand. Alzenhiem taught me what I was standing for. Later, on hard nights under Rilock, I did not dream of glory. I dreamed of the lane behind our house, of my mother’s voice through an open window, of my father’s shadow crossing the doorway at dusk.</t>
         </is>
       </c>
     </row>
@@ -1587,7 +1587,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>*Written at seventeen, after Yua and my master laid the Hero’s charge on me.*</t>
+          <t>*Written at seventeen, after Yua laid the Hero’s charge on me, with Rilock and the King’s Lion present.*</t>
         </is>
       </c>
     </row>
@@ -1611,7 +1611,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>This is my first journal entry after Yua and my master bestrode a heavy responsibility on my shoulders.</t>
+          <t>This is my first journal entry after Yua bestrode a heavy responsibility on my shoulders, and my master Rilock sent me into the world with his blessing.</t>
         </is>
       </c>
     </row>
@@ -5109,7 +5109,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">**Last updated:** 2026-07-26 (trainer clarified: Rilock under the King’s Lion)  </t>
+          <t xml:space="preserve">**Last updated:** 2026-07-26 (fixed Rilock age timing + intro training start)  </t>
         </is>
       </c>
     </row>
@@ -5146,7 +5146,7 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>&gt; I’m Dezco Knoleburn. Seventeen. From a hamlet called Alzenhiem. Dwarven and Elven blood. Trained since twelve by Rilock, royal master swordsman, by order of the King’s Lion. People called me Hero for years before it was true. Yua made it true at seventeen. I love red and black. I’m trying my best.</t>
+          <t>&gt; I’m Dezco Knoleburn. Seventeen. From a hamlet called Alzenhiem. Dwarven and Elven blood. Military trained since eight. From twelve, trained by Rilock, royal master swordsman of the King’s Lion’s royal guard, by the Lion’s order. People called me Hero for years before it was true. Yua made it true at seventeen. I love red and black. I’m trying my best.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete Journal 03 Saltrock arc and sync lore exports
Rewrite journal 03 as a cohesive story from the staff falling through
the tomb quest, focus restoration, feast, and dawn choice. Update the
party reference with Eden, Alice, Jylia, Vita, Alem, Yeara, and new
places. Add Yua hidden plot file and regenerate Google export pack.

Co-authored-by: Dralorex <Dralorex@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/character/lore/exports/Dezco_Knoleburn_Lore_Tabs.xlsx
+++ b/character/lore/exports/Dezco_Knoleburn_Lore_Tabs.xlsx
@@ -23,7 +23,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Journal 03" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 Yua Red And Black" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 Yua Mana Well" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 Crest Lore Full" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 Yua Stays Hidden" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 Crest Lore Full" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -465,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -708,10 +709,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>16 Crest Lore Full</t>
+          <t>16 Yua Stays Hidden</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
+        <is>
+          <t>Why Dezco hides Yua from the party</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>17 Crest Lore Full</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
         <is>
           <t>Full crest/sigil writeups</t>
         </is>
@@ -728,12 +741,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="39" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -840,7 +853,7 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Exact red/black blood meaning</t>
+          <t>Yua walks with Dezco daily</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -850,39 +863,90 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Later Yua reveal</t>
+          <t>Only King’s Lion + Rilock know</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Mana Well / sword imbue details</t>
+          <t>Divine being seen in the world</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Not yet / soon</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Yua explains after Saltrock faceplant</t>
+          <t>Public knowledge; not tied to Dezco</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
+          <t>Exact red/black blood meaning</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Later Yua reveal</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Mana Well / Lord AO gift</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Named in private woods talk; training ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Why Dezco hides Yua</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>See yua-why-she-stays-hidden.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
           <t>Birthday November 6</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Safe</t>
         </is>
@@ -2776,7 +2840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A51"/>
+  <dimension ref="A1:A173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2809,14 +2873,14 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>*Written at seventeen, inside Saltrock’s general building, after the protective staff fell.*</t>
+          <t>*Written at seventeen, after Saltrock’s first night of peace since the attack began.*</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>*This entry is unfinished. The night is not over. I will write more after the next stretch of it.*</t>
+          <t>*This entry covers the storm, the keep, the tomb road, and the choice waiting for us at dawn.*</t>
         </is>
       </c>
     </row>
@@ -2836,7 +2900,7 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>I woke to shouting, then stone, then the kind of silence that means something holy has broken. The staff in the general building, the floating one that keeps Saltrock safe, had fallen. I do not know why yet. I only know what followed.</t>
+          <t>I woke to shouting, then stone grinding, then thunder so close the walls seemed to flinch. Rain hammered the roof. Lightning bleached the room white for a heartbeat and left the dark thicker on the other side. In that split brightness I understood what had broken: the staff in the general building, the floating relic that keeps Saltrock safe, had fallen.</t>
         </is>
       </c>
     </row>
@@ -2846,7 +2910,7 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Monsters came from all sides.</t>
+          <t>Monsters came from every direction at once.</t>
         </is>
       </c>
     </row>
@@ -2856,7 +2920,7 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>I barely made it out of my room in time. The tavern stairs were already a panic of boots and spilled mugs. Outside, Saltrock looked wrong: a traveling town turned into a kill yard. Massive crabs hauled themselves between buildings, claws wide enough to shear a cart horse. Other creatures poured with them, crawling, shrieking, filling every lane that used to mean trade and bad bread and safe passage.</t>
+          <t>I barely escaped my room. The tavern stairs were already a stampede of boots and overturned mugs. When I reached the street, the town looked unrecognizable. Water sheeted down alleys. Crabs the size of carts dragged themselves through the flood, claws shining each time lightning touched them. Other things crawled with them, shrieking, filling lanes that yesterday only meant trade, bad bread, and safe passage.</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2930,7 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>A full frontal attack. No warning worth the name. No time for speeches.</t>
+          <t>No warning. No speeches. Only storm and teeth.</t>
         </is>
       </c>
     </row>
@@ -2876,7 +2940,7 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Townsfolk ran for the general building. Four others and I tried to hold back the creatures that had already closed too far into town. I do not know those four well yet. Names can wait when teeth are present. What I know is that they stood when standing mattered.</t>
+          <t>Townsfolk ran for the general building. Four strangers and I tried to hold the creatures that had already pushed too deep into Saltrock. I did not know their names yet. Names wait until the blood cools.</t>
         </is>
       </c>
     </row>
@@ -2886,7 +2950,7 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>During the panic of battle I swung at a creature I had only ever read about. It was so short I was not prepared. Then something else happened that I still do not have clean words for. Mid swing, my body shoved forward hard, maybe fifteen feet in a blink, sword coming from my side to my front as if the steel had grown eager. My blade cut clean air where a taller foe’s chest should have been. The creature was still below the arc. Momentum and that sudden dash put me face first into gravel.</t>
+          <t>In the panic I swung at something I had only read about: a short bow creature, low enough that my training had never truly prepared me for its height. Then the wrong miracle happened again. Mid arc, my body launched forward, maybe fifteen feet in a blink, blade sweeping from my side to my front as if the steel had a will of its own. I missed. The thing was still beneath my cut. Momentum and that sudden surge sent me face first into the lane.</t>
         </is>
       </c>
     </row>
@@ -2896,7 +2960,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Disappointment hit harder than the ground. So did confusion. I know my own footwork. That was not only a bad read on height. Something in me answered the fight before I understood the question.</t>
+          <t>The gravel was wet and muddy. It smeared my mouth, my cheeks, my new clothes from Fulfein. Rain and filth ran into my eyes. Disappointment hit harder than the ground. Confusion came with it. I know my footwork. That was not only misjudging height. Something inside me had answered the fight before I knew the question.</t>
         </is>
       </c>
     </row>
@@ -2906,7 +2970,7 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>The creature turned on me with a bow already drawn. Point blank. I had time to understand that Hero is a title, not armor. Then luck, or Yua, or sheer stupid mercy, stepped in. The shot missed. At that range it should not have. I am not proud enough to call it skill. It was survival wearing a borrowed face.</t>
+          <t>The creature turned with a bow already drawn. Point blank. Hero is a title, not armor. The shot missed. At that distance it should not have. I will not call that skill.</t>
         </is>
       </c>
     </row>
@@ -2916,7 +2980,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Next thing I knew, an elf girl among the four loosed an arrow of her own.</t>
+          <t>An elf among the four answered with her own arrow. The shot drove through the creature’s mouth and pinned it to the earth so hard the shaft stood in the mud and the head hung above it like a warning I will never unsee. Ugly. Perfect. I owe her more than thanks.</t>
         </is>
       </c>
     </row>
@@ -2926,7 +2990,7 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>The shot pinned the creature to the floor through its mouth. The power in it was ugly and perfect: the arrow drove on into the ground, and the creature’s head stayed lifted on the shaft, skewered, floating above the dirt like a warning carved in flesh. I will not forget that image. Gratitude and horror braided tight.</t>
+          <t>We cleared that pocket of street and fled with the crowd toward the keep. Wood slammed. Bars dropped. Outside became muffled thunder and screaming.</t>
         </is>
       </c>
     </row>
@@ -2936,41 +3000,45 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Once that pocket of street was cleared, we followed the townsfolk toward the general building. We barely made it inside before they sealed the doors fully. Wood slammed. Bars dropped. Outside sound became muffled nightmare.</t>
+          <t>I still do not know how many remained out there.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr"/>
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Trapped in homes.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>I could not say how many people were still out there.</t>
+          <t>Fallen in the lanes.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="inlineStr"/>
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Beating on doors we had already sealed…</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Stuck in their homes.</t>
+          <t>…until the next moment answered with silence.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>Lying lifeless on the ground.</t>
-        </is>
-      </c>
+      <c r="A36" s="6" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Or banging on the door for someone to open up…</t>
+          <t>## Inside the Keep</t>
         </is>
       </c>
     </row>
@@ -2980,7 +3048,7 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>…only for the next moment to answer with silence.</t>
+          <t>We made it inside alive. That counts for something, though the room did not feel like victory.</t>
         </is>
       </c>
     </row>
@@ -2990,7 +3058,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>We are inside now. Crowded. Breathing too loud. The fallen staff is close enough that its wrongness feels like a pulled tooth in the middle of the room. The crabs and the rest are still beyond the walls. The elf girl who saved me has not asked my name yet, or I have not managed to give it. The other three are the same: allies by blood heat, strangers by every other measure.</t>
+          <t>The fallen staff lay near enough that its wrongness ached in my teeth. Rain kept drumming the roof. People breathed too loud. The elf archer who saved me turned out to have a twin sister. Her name is Eden. She handles a bow like punishment made elegant. She is also, I learned quickly, terrible with frightened children. Her sister Alice is the opposite: soft voice, steady hands, the kind of presence that makes panic sit down.</t>
         </is>
       </c>
     </row>
@@ -3000,7 +3068,7 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>I left Alzenhiem yesterday with my father’s sword and my mother’s shovel and a head full of purpose.</t>
+          <t>The halfling who fought beside us is Jylia. Where steel could not reach fear, she tried dance. She spun and stepped through the crowded hall until some of the terror unclenched its jaw. It helped. Not enough. But it helped.</t>
         </is>
       </c>
     </row>
@@ -3010,7 +3078,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Tonight Saltrock is teaching me that purpose arrives late to some doors.</t>
+          <t>We did what we could after that: calming villagers, carrying word to town leaders, pretending the walls were thicker than they felt.</t>
         </is>
       </c>
     </row>
@@ -3020,7 +3088,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>More when I know whether we open those doors again… or what opens them for us.</t>
+          <t>Then the back of the keep screamed.</t>
         </is>
       </c>
     </row>
@@ -3030,19 +3098,629 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>*Dezco Knoleburn*</t>
+          <t>BOOM. BOOM. BOOM.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>*Saltrock general building, during the attack*</t>
-        </is>
-      </c>
+      <c r="A50" s="6" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>A troll broke through with five goblins pouring behind it. The same defenders gathered again. A human priest joined us in the chaos, Vita, early thirties, robes soaked, voice steady. He had already healed a snake man among us, Alem, who speaks mind to mind when words are too slow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>I had seen trolls in training records. I had never stood against one. This one was worse than the texts. Spells slid off it like rain off slate. Wounds closed as soon as they opened. Eden found the crack in its hide: fire. While the others hammered it from the front, I slipped to the rear to keep the goblins from flanking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>Two saw me. I raised Dolkin’s sword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>The tingling returned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>Not fear this time. Not accident alone. The blade felt hungry. My legs felt ready. I surged forward through the space in front of me and cleaved the first goblin clean at the waist. The momentum did not stop. The edge found a second goblin more than ten feet away and opened his gut. He stumbled, ruined but not yet dead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>When I turned, the troll was a burning heap collapsing to the floor. Goblins broke and ran. The wounded one made it only a few strides before Eden put an arrow through his back.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>For a moment the hall actually quieted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>Then the mayor found us and said the fight was not over.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>## The First King’s Lion</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>He spoke of a title I already knew from my own life, though not this far back in its bloodline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>The King’s Lion serves the holy city’s king and is said to be the realm’s greatest living swordsman. Each Lion succeeds the last. The first of that line is buried in a tomb somewhere beyond Saltrock. The mayor did not know where. The library might.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>He was right.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>Vita deciphered an old book the rest of us could barely read. More than a hundred years of shifting land lay between its map and the world. Still, it gave a direction. We left at once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>On the path Yua appeared at my shoulder, visible only to me, and pointed the way the road should bend. The others doubted me. I told them to check the book. Vita did. The scrappy map inside matched the terrain in the direction I had named. They stopped arguing. They did not stop watching me oddly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>I need to write this plainly, because if I lie to my own page I will forget why I am lying to everyone else.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>The world knows a divine being was seen once. It does not know she walks with me. Only the current King’s Lion and Rilock know Yua travels at my side. I have told no one in this new company.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>I tell myself it is for her safety. That is true. Hunters, kings, zealots, and worse would reach for her if they understood. But safety is not the whole truth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t>Yua does not feed on worship. She grows through hope, courage, and faith placed in those who still choose to stand. If my companions learn a goddess walks beside me, their hope will slide off my shoulders and onto hers. They will wait for miracles instead of making them. They will pray at the wrong altar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t>Then I am no longer the Hero she charged me to become. I am only the escort of a goddess.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="inlineStr">
+        <is>
+          <t>I hide her not because I am ashamed. Because her silence is part of the gift. If hope is to return, it must land in mortal hands again. Including mine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="6" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="inlineStr">
+        <is>
+          <t>## Yolon</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="inlineStr">
+        <is>
+          <t>Rain had not stopped when we found the statue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="6" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="inlineStr">
+        <is>
+          <t>It rose from the hillside crusted in moss, mud, and old vines: a dragon carved in stone with a bowl at its feet. Something in me wanted to pray there, not to the dragon itself, but near it. When I did, warmth moved through my chest like an ember carefully placed. I felt steadier on the road we were already walking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="6" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="6" t="inlineStr">
+        <is>
+          <t>Jylia drank the rainwater pooled in the bowl.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="6" t="inlineStr">
+        <is>
+          <t>The statue spoke without moving its mouth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="6" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="6" t="inlineStr">
+        <is>
+          <t>His name is Yolon. He was a true dragon once, turned to stone as magic thinned from the world. He has stood there more than a hundred years waiting to be freed. When we asked about the first King’s Lion, he laughed until the sound rolled through the wet trees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="6" t="inlineStr">
+        <is>
+          <t>He had fought that Lion many times. Battles that went on until both of them were spent. Every duel ended in a draw. Every duel made them stronger. In time they stopped trying to kill each other and simply tested one another, as if respect had outgrown victory. Yolon never learned the Lion’s final fate, but he knew where the tomb lay.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="6" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
+          <t>Keep on this path, he said. Eventually take the right fork.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="6" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="6" t="inlineStr">
+        <is>
+          <t>We thanked him and went on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="6" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="6" t="inlineStr">
+        <is>
+          <t>## The Bridge and the Owlbear</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="6" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="6" t="inlineStr">
+        <is>
+          <t>The right fork brought us to a wooden bridge so old it complained under its own weight. Across it sat a boulder that looked deliberately wrong, like a lump dropped by a careless giant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="6" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="6" t="inlineStr">
+        <is>
+          <t>Eden vanished while we debated how to cross. By the time we noticed, she was already on the far side.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="6" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="6" t="inlineStr">
+        <is>
+          <t>Alem reached her with telepathy. Eden’s thoughts came back to us in pieces. Inside the stone slept an owlbear, the largest she had ever seen: bear body, owl head, claws long enough to split a person in two. Lucky for us, it was still sleeping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="6" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="6" t="inlineStr">
+        <is>
+          <t>One by one we crossed as Eden directed our steps. One board. One breath. No sound. Somehow every one of us made it over.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="6" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="6" t="inlineStr">
+        <is>
+          <t>At the next split, the elven sisters went down toward the river. The rest of us climbed the cliff stairs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="6" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="6" t="inlineStr">
+        <is>
+          <t>## The Tomb and the Focus</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="6" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="6" t="inlineStr">
+        <is>
+          <t>At the hilltop we found a heavy door set into stone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="6" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="6" t="inlineStr">
+        <is>
+          <t>Jylia pushed it open without hesitation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="6" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="6" t="inlineStr">
+        <is>
+          <t>Goblins. Maybe five. The same breed that hit the keep. We cut them down fast, almost embarrassingly so. We dragged the bodies aside and went deeper.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="6" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="6" t="inlineStr">
+        <is>
+          <t>The real tomb waited beyond.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="6" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="6" t="inlineStr">
+        <is>
+          <t>Inside we found a focus, faintly glowing, beautiful, and completely mysterious. None of us knew what it did. I wanted to hold it longer than I should have.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="6" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="6" t="inlineStr">
+        <is>
+          <t>When we climbed back out, sunlight hit my face for the first time since the attack began. I thought that meant relief.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="6" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="6" t="inlineStr">
+        <is>
+          <t>I spoke to Yua about the tingling in battle. She knew what it was and could not say. Like the knowledge lived beneath language and would not come up when I demanded it. I did not ask well. I think I angered her.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="6" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="6" t="inlineStr">
+        <is>
+          <t>On the return path something lifted me two feet off the ground and dropped me over a fifteen foot edge. No proof. Strong suspicion. My foot hurts. So does whatever pride I had left.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="6" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="6" t="inlineStr">
+        <is>
+          <t>At the bridge the owlbear was gone. We saw no sign of it. We counted that as blessing and did not question fortune too loudly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="6" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="6" t="inlineStr">
+        <is>
+          <t>I tried to recreate the lift Yua had given me, if it was her at all. I attempted to leap a gap back onto the bridge. Nothing answered. I fell. One hand caught the edge. Eden reached with her bow to help. She smacked my fingers instead. I dropped farther. Alice caught my other hand. Vita hauled us both up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="6" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="6" t="inlineStr">
+        <is>
+          <t>I shouted at empty air afterward. Yua was furious, or hurt, or both. She said we would need to talk later. The party saw only a boy cursing at nothing. I blamed the vines on Yolon’s statue. That lie held.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="6" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="6" t="inlineStr">
+        <is>
+          <t>On the way back Vita collected those same vines for herbs, or so he said. I hope that is true. The vines did nothing to me. I was only scrambling for an excuse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="6" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="6" t="inlineStr">
+        <is>
+          <t>## What Yua Told Me in the Woods</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="6" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="6" t="inlineStr">
+        <is>
+          <t>When Saltrock came into view again, I slipped away to speak with her alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="6" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="6" t="inlineStr">
+        <is>
+          <t>She remembered more there than she had on the mountain. She said I had received a gift directly from Lord AO. We would have to grow together and learn the power through training. No shortcuts. No temper.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="6" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="6" t="inlineStr">
+        <is>
+          <t>She also said she feels a darkness unlike any she has known. She does not know its source yet. Only that I should be careful.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="6" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="6" t="inlineStr">
+        <is>
+          <t>I rejoined the group with mud on my knees and no good answers for their questions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="6" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="6" t="inlineStr">
+        <is>
+          <t>## The Focus Restored</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="6" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="6" t="inlineStr">
+        <is>
+          <t>We brought the glowing focus home.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="6" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="6" t="inlineStr">
+        <is>
+          <t>The mayor, Vita, and a priestess named Yeara set it back into place. Protection returned to Saltrock. For the first time since the staff fell, the town felt like it might hold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="6" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="6" t="inlineStr">
+        <is>
+          <t>Then choice arrived with gratitude.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="6" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="6" t="inlineStr">
+        <is>
+          <t>The mayor wants us to escort him to Lyndor, the capital, to stand before Lord Keivan. Yeara wants us instead to travel with her to Lořel, the city of churches. We are to decide by morning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="6" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="6" t="inlineStr">
+        <is>
+          <t>Tonight they threw a feast to celebrate survival. After the food, the music, and too many eyes on me, I finally slept.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="6" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="6" t="inlineStr">
+        <is>
+          <t>Tomorrow we choose a road.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="6" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="6" t="inlineStr">
+        <is>
+          <t>*Dezco Knoleburn*</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="6" t="inlineStr">
+        <is>
+          <t>*Saltrock, after the feast*</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="6" t="inlineStr">
         <is>
           <t>*To be continued*</t>
         </is>
@@ -3459,7 +4137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A83"/>
+  <dimension ref="A1:A95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -3852,7 +4530,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>She will explain the Well: what it is, that it is not his soul, how simple imbument should feel once understood, and that sword mana can lighten, sharpen, and briefly hasten him. She will also make clear that knowing is not mastery. He must train. He must practice draws, bursts, recovery, and control until the Well’s breath matches his own.</t>
+          <t>On the tomb return, alone in the woods near Saltrock, she remembered more than she had on the mountain. She named the gift as coming directly from Lord AO. They would have to grow together and learn the power through training. No shortcuts. No temper.</t>
         </is>
       </c>
     </row>
@@ -3862,7 +4540,7 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>Until that training is real, every panic swing risks another fifteen feet of unwanted truth.</t>
+          <t>She also warned that she feels a darkness unlike any she has known. Source unknown yet.</t>
         </is>
       </c>
     </row>
@@ -3872,7 +4550,7 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>## Story use notes</t>
+          <t>## Second use: keep goblin fight</t>
         </is>
       </c>
     </row>
@@ -3882,26 +4560,86 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>1. Red and black meaning can stay a later reveal; the Well may be explained sooner because combat forced it</t>
+          <t>During the troll breach at the keep, Dezco used the simple imbue again, this time with less accident and more hunger.</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="6" t="inlineStr">
-        <is>
-          <t>2. Party members may see sudden speed or a lighter looking blade before they hear the word mana</t>
-        </is>
-      </c>
+      <c r="A81" s="6" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
+          <t>The blade felt eager. His body matched it. He surged forward, cleaved one goblin at the waist, and the momentum carried the edge to a second goblin more than ten feet away, opening his gut. Still untrained, but no faceplant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr">
+        <is>
+          <t>## What remains to teach</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
+          <t>She will still explain the Well in full: what it is, that it is not his soul, how simple imbue should feel once understood, and that sword mana can lighten, sharpen, and briefly hasten him. Naming Lord AO is not the same as mastery. He must train. He must practice draws, bursts, recovery, and control until the Well’s breath matches his own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t>Until that training is real, every panic swing risks another fifteen feet of unwanted truth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="6" t="inlineStr">
+        <is>
+          <t>## Story use notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="inlineStr">
+        <is>
+          <t>1. Red and black meaning can stay a later reveal; the Well may be explained sooner because combat forced it</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="inlineStr">
+        <is>
+          <t>2. Party members may see sudden speed or a lighter looking blade before they hear the word mana</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="6" t="inlineStr">
+        <is>
           <t>3. Dezco should sound frustrated that the gift tripped him before it saved him</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="6" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="6" t="inlineStr">
         <is>
           <t>4. Future journal entries can cover Yua’s explanation and his first deliberate training drills</t>
         </is>
@@ -3913,6 +4651,413 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A71"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="100" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>16 Yua Stays Hidden</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Source: character/lore/yua-story-plots/yua-why-she-stays-hidden.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t># Why Yua Stays Hidden From the Party</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>*Yua story plot. Dezco knows this logic. The party does not.*</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>*Journal 03 records his private reasoning on the tomb road.*</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>## What the world already knows</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>A divine being was seen once. That sighting cannot be undone. Saltrock and the wider realm may still talk about it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>What they must not learn is that she walks with Dezco day to day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>## Who knows she travels with him</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>| Person | Knows? |</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>|---|---|</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>| The current King’s Lion | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>| Rilock | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>| Dezco | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>| Saltrock party (Eden, Alice, Jylia, Vita, Alem, etc.) | No |</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>| General public | No |</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>## Why Dezco hides her</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>### The reason he tells himself first</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Safety. Hunters, kings, zealots, and worse would reach for Yua if they understood she is bound to a seventeen year old Hero on the road.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>That is true. It is not the whole truth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>### The reason he will not say aloud at camp</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Yua does not feed on worship. She grows through hope, courage, and faith placed in mortals who still choose to stand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>If companions learn a goddess walks at Dezco’s shoulder:</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>1. Their hope slides off him and onto her</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>2. They wait for miracles instead of making them</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>3. They pray at the wrong altar</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>Then Dezco stops being the Hero she charged him to become. He becomes only the escort of a goddess.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>He hides her not from shame. Her silence is part of the gift. If hope is to return to the world, it must land in mortal hands again, including his.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>## What happens when he slips</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>On the return from the tomb road, Dezco shouted at empty air after the bridge fall. The party saw a boy cursing at nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>He blamed vines from Yolon’s statue. The lie held for now. They think he may have eaten something he should not have, not that he communes with the divine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>## Roleplay notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>| Topic | Party can know? |</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>|---|---|</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>| A divine being was seen somewhere in the world | Yes (public knowledge) |</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>| Yua travels with Dezco | No |</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>| Dezco talks to “no one” when stressed | Yes (they witnessed it) |</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>| Vine excuse from dragon statue | Yes (his cover story) |</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>| Why he really hides her | No (private journal logic) |</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>## Future pressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>This secret will strain whenever:</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>1. Yua nudges him in front of others (direction on the path, the two foot lift, the bridge)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>2. Someone holy (Vita, Yeara) senses wrongness or grace they cannot name</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>3. Dezco needs party trust while acting on guidance only he receives</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>When the secret breaks, the hope corruption fear should drive how Yua and Dezco respond, not simple embarrassment.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3927,7 +5072,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>16 Crest Lore Full</t>
+          <t>17 Crest Lore Full</t>
         </is>
       </c>
     </row>
@@ -5059,7 +6204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A275"/>
+  <dimension ref="A1:A310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -5109,7 +6254,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">**Last updated:** 2026-07-26 (fixed Rilock age timing + intro training start)  </t>
+          <t xml:space="preserve">**Last updated:** 2026-08-23 (Journal 03 complete: tomb quest, focus restored, feast, dawn choice)  </t>
         </is>
       </c>
     </row>
@@ -5302,14 +6447,14 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>| Current location | Saltrock general building (doors sealed; under attack) |</t>
+          <t>| Current location | Saltrock (protection restored; feast over; resting for dawn choice) |</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>| Travel status | Adventure day 2 gone wrong; protective staff fell; mid siege |</t>
+          <t>| Travel status | Adventure day 2; staff fell then focus restored; escort vs church city decision by morning |</t>
         </is>
       </c>
     </row>
@@ -5395,557 +6540,565 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>| I accidentally used a simple imbue in Saltrock | I meant to dash 15 feet and faceplant on purpose |</t>
+          <t>| I accidentally used a simple imbue in Saltrock street fight | I have also used imbue on purpose in the keep goblin fight (still learning) |</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="6" t="inlineStr"/>
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>| Yua travels with me | Only the King’s Lion and Rilock know; Saltrock party does not |</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="6" t="inlineStr">
+      <c r="A57" s="6" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="6" t="inlineStr"/>
-    </row>
     <row r="59">
-      <c r="A59" s="6" t="inlineStr">
+      <c r="A59" s="6" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
         <is>
           <t>## Family (quick)</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="6" t="inlineStr"/>
-    </row>
     <row r="61">
-      <c r="A61" s="6" t="inlineStr">
-        <is>
-          <t>| Person | Who | Age | Name means | Colors | One line |</t>
-        </is>
-      </c>
+      <c r="A61" s="6" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>|---|---|---|---|---|---|</t>
+          <t>| Person | Who | Age | Name means | Colors | One line |</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>| Dolkin | Father | 38 | steadfast of kin | charcoal, iron, bronze | Steady, Dwarven depth, sent me to train to keep me alive |</t>
+          <t>|---|---|---|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>| Fulfein | Mother | 36 | full fair light | sage, silver, pale gold | Warm Elven grace; Alzenhiem’s center for me |</t>
+          <t>| Dolkin | Father | 38 | steadfast of kin | charcoal, iron, bronze | Steady, Dwarven depth, sent me to train to keep me alive |</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>| Kalhien | Younger brother | 15 | rises in pursuit | ink blue + copper | Restless, proud, does not want to be only “Dezco’s brother” |</t>
+          <t>| Fulfein | Mother | 36 | full fair light | sage, silver, pale gold | Warm Elven grace; Alzenhiem’s center for me |</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
+          <t>| Kalhien | Younger brother | 15 | rises in pursuit | ink blue + copper | Restless, proud, does not want to be only “Dezco’s brother” |</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
           <t>| Astiale | Younger sister | 8 | gentle star | rose, cream, sky | Sweet; not born when I left at 8 |</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="6" t="inlineStr"/>
-    </row>
     <row r="68">
-      <c r="A68" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">**Surname Knoleburn means:** stream by the knoll  </t>
-        </is>
-      </c>
+      <c r="A68" s="6" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">**Surname Knoleburn means:** stream by the knoll  </t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
           <t>**Alzenhiem means:** sheltered home under a kind sky</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="6" t="inlineStr"/>
-    </row>
     <row r="71">
-      <c r="A71" s="6" t="inlineStr">
+      <c r="A71" s="6" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="6" t="inlineStr"/>
-    </row>
     <row r="73">
-      <c r="A73" s="6" t="inlineStr">
+      <c r="A73" s="6" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
         <is>
           <t>## Home</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="6" t="inlineStr"/>
-    </row>
     <row r="75">
-      <c r="A75" s="6" t="inlineStr">
-        <is>
-          <t>| | |</t>
-        </is>
-      </c>
+      <c r="A75" s="6" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| | |</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>| Place | Alzenhiem |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>| Type | Small hamlet |</t>
+          <t>| Place | Alzenhiem |</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>| Vibe | Dirt paths, low roofs, neighbors first, no royal banners |</t>
+          <t>| Type | Small hamlet |</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>| Why it matters | What I stand for when I talk about hope |</t>
+          <t>| Vibe | Dirt paths, low roofs, neighbors first, no royal banners |</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>| Town flag colors | wheat gold, meadow green, earth brown, cream |</t>
+          <t>| Why it matters | What I stand for when I talk about hope |</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
+          <t>| Town flag colors | wheat gold, meadow green, earth brown, cream |</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
           <t>| Town flag idea | roof + wheat + lane |</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="6" t="inlineStr"/>
-    </row>
     <row r="84">
-      <c r="A84" s="6" t="inlineStr">
+      <c r="A84" s="6" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="6" t="inlineStr"/>
-    </row>
     <row r="86">
-      <c r="A86" s="6" t="inlineStr">
+      <c r="A86" s="6" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="inlineStr">
         <is>
           <t>## Timeline (memorize this order)</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="6" t="inlineStr"/>
-    </row>
     <row r="88">
-      <c r="A88" s="6" t="inlineStr">
-        <is>
-          <t>| Age | What happened |</t>
-        </is>
-      </c>
+      <c r="A88" s="6" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| Age | What happened |</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>| 0 | Born November 6; named Dezco; red/black crest + sigil at birth |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>| 8 | Left Alzenhiem for military training; Kalhien was 6; Astiale not born yet |</t>
+          <t>| 0 | Born November 6; named Dezco; red/black crest + sigil at birth |</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>| 8 to 12 | Overshadowed by a stronger rival; Yua watched unseen |</t>
+          <t>| 8 | Left Alzenhiem for military training; Kalhien was 6; Astiale not born yet |</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>| 12 | Rival (nearly 18) dueled me; Yua secretly blessed my speed/strength; only the King’s Lion truly saw her |</t>
+          <t>| 8 to 12 | Overshadowed by a stronger rival; Yua watched unseen |</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>| 12 | King’s Lion directed royal master swordsman Rilock (royal guard) to train me |</t>
+          <t>| 12 | Rival (nearly 18) dueled me; Yua secretly blessed my speed/strength; only the King’s Lion truly saw her |</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>| 12 to 17 | Merciless real missions under Rilock; reputation spread; people falsely called me Hero of centuries |</t>
+          <t>| 12 | King’s Lion directed royal master swordsman Rilock (royal guard) to train me |</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>| Before 15 | Name known across much of the realm |</t>
+          <t>| 12 to 17 | Merciless real missions under Rilock; reputation spread; people falsely called me Hero of centuries |</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Master Rilock said I had learned all he could teach |</t>
+          <t>| Before 15 | Name known across much of the realm |</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Yua appeared before me, Rilock, and the Lion; gave me the ancient title Hero + sacred mission |</t>
+          <t>| 17 | Master Rilock said I had learned all he could teach |</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Final goodbye at Alzenhiem; family gifts; left for the road |</t>
+          <t>| 17 | Yua appeared before me, Rilock, and the Lion; gave me the ancient title Hero + sacred mission |</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Reached Saltrock; lodging at the tavern; seeking where to travel next |</t>
+          <t>| 17 | Final goodbye at Alzenhiem; family gifts; left for the road |</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Saltrock staff fell; monsters attacked (massive crabs + others) |</t>
+          <t>| 17 | Reached Saltrock; lodging at the tavern; seeking where to travel next |</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Fought with 4 other defenders; missed a short bow creature; saved by an elf girl’s arrow |</t>
+          <t>| 17 | Saltrock staff fell; storm, crabs, and other creatures attacked |</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>| 17 | Barely sealed inside the general building; many townsfolk fate unknown |</t>
+          <t>| 17 | Fought with defenders; missed short bow creature; faceplant in wet muddy gravel; saved by Eden’s arrow |</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>| Now | Trapped in Saltrock general building during the attack; entry open ended |</t>
+          <t>| 17 | Sealed in keep; troll + goblins; second imbue cleaved goblins; Eden/fire ended troll |</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="6" t="inlineStr"/>
+      <c r="A105" s="6" t="inlineStr">
+        <is>
+          <t>| 17 | Quest for first King’s Lion tomb; library map; Yolon stone dragon; owlbear bridge; tomb focus recovered |</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="6" t="inlineStr">
         <is>
+          <t>| 17 | Focus restored Saltrock with mayor, Vita, Yeara; feast; choice by dawn: Lyndor or Lořel |</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="6" t="inlineStr">
+        <is>
+          <t>| Now | Resting after feast; foot bruised from cliff fall; Yua and I still need to talk |</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="6" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="6" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" s="6" t="inlineStr"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="6" t="inlineStr">
-        <is>
-          <t>## Important people (outside family)</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="6" t="inlineStr"/>
-    </row>
     <row r="110">
-      <c r="A110" s="6" t="inlineStr">
-        <is>
-          <t>| Person | Who they are to me |</t>
-        </is>
-      </c>
+      <c r="A110" s="6" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>## Important people (outside family)</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="6" t="inlineStr">
-        <is>
-          <t>| Yua | Ancient being tied to magic; broke a millennia oath to act; watched me since childhood; gave me Hero title; often appears as a small pixie |</t>
-        </is>
-      </c>
+      <c r="A112" s="6" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>| The King’s Lion | King’s greatest swordsman; only one who truly saw Yua at the duel; directed that I be trained |</t>
+          <t>| Person | Who they are to me |</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>| Rilock | Royal master swordsman; one of the King’s Lion’s royal guard; my actual trainer/master from ages 12 to 17 |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>| The Rival | Older trainee who believed he was the chosen one; challenged me at 12; lost after Yua’s hidden aid |</t>
+          <t>| Yua | Ancient being tied to magic; broke a millennia oath to act; watched me since childhood; gave me Hero title; often appears as a small pixie; only Lion + Rilock know she walks with me |</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="6" t="inlineStr">
         <is>
-          <t>| Elf girl archer | One of 4 defenders in Saltrock attack; pinned a short bow creature through the mouth and into the ground; name not known yet |</t>
+          <t>| The King’s Lion | King’s greatest swordsman; only one who truly saw Yua at the duel; directed that I be trained; knows Yua travels with me |</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="6" t="inlineStr">
         <is>
-          <t>| 3 other defenders | Fought beside us getting townsfolk to the general building; names not known yet |</t>
+          <t>| Rilock | Royal master swordsman; one of the King’s Lion’s royal guard; my actual trainer/master from ages 12 to 17; knows Yua travels with me |</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="6" t="inlineStr"/>
+      <c r="A118" s="6" t="inlineStr">
+        <is>
+          <t>| The Rival | Older trainee who believed he was the chosen one; challenged me at 12; lost after Yua’s hidden aid |</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="6" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>| Eden | Elf archer; twin to Alice; bow like punishment made elegant; terrible with frightened children; saved me in the street fight |</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="6" t="inlineStr"/>
+      <c r="A120" s="6" t="inlineStr">
+        <is>
+          <t>| Alice | Eden’s twin; soft with scared people; good with children; pulled me up on the owlbear bridge |</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="6" t="inlineStr">
         <is>
-          <t>## Current gear / gifts from home</t>
+          <t>| Jylia | Halfling dancer; fought in the keep; danced to calm the hall; pushed open the tomb door without hesitation |</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="6" t="inlineStr"/>
+      <c r="A122" s="6" t="inlineStr">
+        <is>
+          <t>| Vita | Human priest (~30s); healer and spellcaster; read the old library map; helped restore the focus; collected Yolon statue vines |</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
         <is>
-          <t>| Item | From | Notes |</t>
+          <t>| Alem | Snake man; telepathy mind to mind; healed before I met him properly; relayed Eden’s owlbear scouting |</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="6" t="inlineStr">
         <is>
-          <t>|---|---|---|</t>
+          <t>| Yeara | Priestess in Saltrock; worked with Vita and the mayor to set the focus back; wants us at Lořel by morning decision |</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="6" t="inlineStr">
         <is>
-          <t>| New sword | Dolkin | Hand forged goodbye; his love without saying the words |</t>
+          <t>| Yolon | Stone dragon statue (&gt;100 years); spoke after Jylia drank bowl rain; fought first King’s Lion to endless draws; gave tomb direction |</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="6" t="inlineStr">
         <is>
-          <t>| First smithing tools | Dolkin | His original set; “you are the master of your steel” |</t>
+          <t>| Saltrock mayor | Town leader; sent us to the tomb; wants escort to Lord Keivan in Lyndor |</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="6" t="inlineStr">
         <is>
-          <t>| 10 gold pieces | Fulfein | Travel money |</t>
+          <t>| Lord Keivan | Ruler in capital Lyndor; mayor wants to present us there |</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="6" t="inlineStr">
-        <is>
-          <t>| Cooking pot | Fulfein | Eat warm when you can |</t>
-        </is>
-      </c>
+      <c r="A128" s="6" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="6" t="inlineStr">
         <is>
-          <t>| New clothing | Fulfein | Wearing them out of respect; left home in them |</t>
+          <t>---</t>
         </is>
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="6" t="inlineStr">
-        <is>
-          <t>| Shovel | Fulfein | Funny gift for roadside “number two” duty; also quietly useful if not everyone makes it |</t>
-        </is>
-      </c>
+      <c r="A130" s="6" t="inlineStr"/>
     </row>
     <row r="131">
-      <c r="A131" s="6" t="inlineStr"/>
+      <c r="A131" s="6" t="inlineStr">
+        <is>
+          <t>## Current gear / gifts from home</t>
+        </is>
+      </c>
     </row>
     <row r="132">
-      <c r="A132" s="6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="A132" s="6" t="inlineStr"/>
     </row>
     <row r="133">
-      <c r="A133" s="6" t="inlineStr"/>
+      <c r="A133" s="6" t="inlineStr">
+        <is>
+          <t>| Item | From | Notes |</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="6" t="inlineStr">
         <is>
-          <t>## Places</t>
+          <t>|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="6" t="inlineStr"/>
+      <c r="A135" s="6" t="inlineStr">
+        <is>
+          <t>| New sword | Dolkin | Hand forged goodbye; his love without saying the words |</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="6" t="inlineStr">
         <is>
-          <t>| Place | What it is |</t>
+          <t>| First smithing tools | Dolkin | His original set; “you are the master of your steel” |</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| 10 gold pieces | Fulfein | Travel money |</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
         <is>
-          <t>| Alzenhiem | Home hamlet; my center |</t>
+          <t>| Cooking pot | Fulfein | Eat warm when you can |</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
         <is>
-          <t>| Saltrock | Traveling town of people coming and going; I know it well |</t>
+          <t>| New clothing | Fulfein | Wearing them out of respect; left home in them |</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="6" t="inlineStr">
         <is>
-          <t>| Saltrock general building | Holds the protective magic staff; we are sealed inside it during the attack |</t>
+          <t>| Shovel | Fulfein | Funny gift for roadside “number two” duty; also quietly useful if not everyone makes it |</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="6" t="inlineStr">
         <is>
-          <t>| Saltrock protective staff | Used to float and block named monsters/creatures; has fallen; reason unknown |</t>
+          <t>| Tomb focus (recovered) | Saltrock quest | Faint glow; purpose unknown at first; mayor + Vita + Yeara restored town protection with it |</t>
         </is>
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="6" t="inlineStr">
-        <is>
-          <t>| Saltrock tavern | Where I lodged the night before the attack; “best bread” only with nostalgia |</t>
-        </is>
-      </c>
+      <c r="A142" s="6" t="inlineStr"/>
     </row>
     <row r="143">
-      <c r="A143" s="6" t="inlineStr"/>
+      <c r="A143" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
     </row>
     <row r="144">
-      <c r="A144" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">**First magic item I ever saw:** the floating protective staff in Saltrock.  </t>
-        </is>
-      </c>
+      <c r="A144" s="6" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="6" t="inlineStr">
         <is>
-          <t>**Current crisis:** staff down; crabs and other creatures overran the streets; unknown how many people remain outside.</t>
+          <t>## Places</t>
         </is>
       </c>
     </row>
@@ -5955,370 +7108,378 @@
     <row r="147">
       <c r="A147" s="6" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>| Place | What it is |</t>
         </is>
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="6" t="inlineStr"/>
+      <c r="A148" s="6" t="inlineStr">
+        <is>
+          <t>|---|---|</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="6" t="inlineStr">
         <is>
-          <t>## My Hero mission (from Yua)</t>
+          <t>| Alzenhiem | Home hamlet; my center |</t>
         </is>
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="6" t="inlineStr"/>
+      <c r="A150" s="6" t="inlineStr">
+        <is>
+          <t>| Saltrock | Traveling town; staff fell then focus restored; feast tonight; dawn choice pending |</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="6" t="inlineStr">
         <is>
-          <t>1. Restore magic before it disappears completely</t>
+          <t>| Saltrock keep / general building | Where townsfolk sheltered; back wall breached by troll; focus set back with Vita and Yeara |</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="6" t="inlineStr">
         <is>
-          <t>2. Stand against the darkness consuming the world</t>
+          <t>| Saltrock library | Old book with scrappy map to first King’s Lion tomb |</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="6" t="inlineStr">
         <is>
-          <t>3. Unite the fractured kingdoms and races</t>
+          <t>| Saltrock tavern | Where I lodged the night before the attack; “best bread” only with nostalgia |</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="6" t="inlineStr">
         <is>
-          <t>4. Become the symbol of hope the world has long forgotten</t>
+          <t>| Lyndor | Capital; Lord Keivan; mayor wants escort there |</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="6" t="inlineStr">
         <is>
-          <t>5. Bring together the two halves of the world</t>
+          <t>| Lořel | City of churches; priestess Yeara wants us to go there instead |</t>
         </is>
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="6" t="inlineStr"/>
+      <c r="A156" s="6" t="inlineStr">
+        <is>
+          <t>| First King’s Lion tomb | Hilltop beyond Saltrock; goblin hideout behind outer door; real tomb held the focus |</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="6" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>| Yolon statue | Stone dragon with rain bowl on tomb path; spoke when Jylia drank; pointed us onward |</t>
         </is>
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="6" t="inlineStr"/>
+      <c r="A158" s="6" t="inlineStr">
+        <is>
+          <t>| Owlbear bridge | Rickety crossing; sleeping giant owlbear in false boulder; gone on return trip |</t>
+        </is>
+      </c>
     </row>
     <row r="159">
-      <c r="A159" s="6" t="inlineStr">
-        <is>
-          <t>## Training under Rilock included</t>
-        </is>
-      </c>
+      <c r="A159" s="6" t="inlineStr"/>
     </row>
     <row r="160">
-      <c r="A160" s="6" t="inlineStr"/>
+      <c r="A160" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">**First magic item I ever saw:** the floating protective staff in Saltrock.  </t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="6" t="inlineStr">
         <is>
-          <t>1. Endless swordsmanship drills</t>
+          <t xml:space="preserve">**Current crisis resolved:** focus back in place; town shielded again.  </t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="6" t="inlineStr">
         <is>
-          <t>2. Physical conditioning beyond normal limits</t>
+          <t>**Current dilemma:** escort mayor to Lyndor vs travel with Yeara to Lořel; decide by morning.</t>
         </is>
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="6" t="inlineStr">
-        <is>
-          <t>3. Pain tolerance and endurance</t>
-        </is>
-      </c>
+      <c r="A163" s="6" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="6" t="inlineStr">
         <is>
-          <t>4. Tactical education</t>
+          <t>---</t>
         </is>
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="6" t="inlineStr">
-        <is>
-          <t>5. Real combat missions (not simulations; death was possible)</t>
-        </is>
-      </c>
+      <c r="A165" s="6" t="inlineStr"/>
     </row>
     <row r="166">
-      <c r="A166" s="6" t="inlineStr"/>
+      <c r="A166" s="6" t="inlineStr">
+        <is>
+          <t>## My Hero mission (from Yua)</t>
+        </is>
+      </c>
     </row>
     <row r="167">
-      <c r="A167" s="6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="A167" s="6" t="inlineStr"/>
     </row>
     <row r="168">
-      <c r="A168" s="6" t="inlineStr"/>
+      <c r="A168" s="6" t="inlineStr">
+        <is>
+          <t>1. Restore magic before it disappears completely</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="6" t="inlineStr">
         <is>
-          <t>## Colors, crest, sigil</t>
+          <t>2. Stand against the darkness consuming the world</t>
         </is>
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="6" t="inlineStr"/>
+      <c r="A170" s="6" t="inlineStr">
+        <is>
+          <t>3. Unite the fractured kingdoms and races</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="6" t="inlineStr">
         <is>
-          <t>| Item | Quick fact |</t>
+          <t>4. Become the symbol of hope the world has long forgotten</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>5. Bring together the two halves of the world</t>
         </is>
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="6" t="inlineStr">
-        <is>
-          <t>| Why I wear red + black | I have always loved them; deep reason not revealed to me yet |</t>
-        </is>
-      </c>
+      <c r="A173" s="6" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="6" t="inlineStr">
         <is>
-          <t>| My crest | Simple child crest: blade/flame between small parent marks |</t>
+          <t>---</t>
         </is>
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="6" t="inlineStr">
-        <is>
-          <t>| My sigil | One red/black blade or flame mark |</t>
-        </is>
-      </c>
+      <c r="A175" s="6" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="6" t="inlineStr">
         <is>
-          <t>| Crest tradition | Child crest = name + gender + both parents; simpler than parents; unique |</t>
+          <t>## Training under Rilock included</t>
         </is>
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="6" t="inlineStr">
-        <is>
-          <t>| Sigil tradition | Same day as crest; one quick seal mark |</t>
-        </is>
-      </c>
+      <c r="A177" s="6" t="inlineStr"/>
     </row>
     <row r="178">
-      <c r="A178" s="6" t="inlineStr"/>
+      <c r="A178" s="6" t="inlineStr">
+        <is>
+          <t>1. Endless swordsmanship drills</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="6" t="inlineStr">
         <is>
-          <t>### Family crest / sigil cheat sheet</t>
+          <t>2. Physical conditioning beyond normal limits</t>
         </is>
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="6" t="inlineStr"/>
+      <c r="A180" s="6" t="inlineStr">
+        <is>
+          <t>3. Pain tolerance and endurance</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="6" t="inlineStr">
         <is>
-          <t>| Person | Colors | Crest idea | Sigil idea |</t>
+          <t>4. Tactical education</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="6" t="inlineStr">
         <is>
-          <t>|---|---|---|---|</t>
+          <t>5. Real combat missions (not simulations; death was possible)</t>
         </is>
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="6" t="inlineStr">
-        <is>
-          <t>| Dolkin | charcoal / iron / bronze | stone arch + hammer | hammer in arch |</t>
-        </is>
-      </c>
+      <c r="A183" s="6" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="6" t="inlineStr">
         <is>
-          <t>| Fulfein | sage / silver / pale gold | leaf + crescent | leaf into crescent |</t>
+          <t>---</t>
         </is>
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="6" t="inlineStr">
-        <is>
-          <t>| Dezco | red / black | balanced blade/flame | red/black split blade |</t>
-        </is>
-      </c>
+      <c r="A185" s="6" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="6" t="inlineStr">
         <is>
-          <t>| Kalhien | blue / copper | forward eager mark | forward chevron |</t>
+          <t>## Colors, crest, sigil</t>
         </is>
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="6" t="inlineStr">
-        <is>
-          <t>| Astiale | rose / cream / sky | soft bud or star | soft bud/star |</t>
-        </is>
-      </c>
+      <c r="A187" s="6" t="inlineStr"/>
     </row>
     <row r="188">
-      <c r="A188" s="6" t="inlineStr"/>
+      <c r="A188" s="6" t="inlineStr">
+        <is>
+          <t>| Item | Quick fact |</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="6" t="inlineStr">
         <is>
-          <t>Images: `assets/crests/alzenhiem/`</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="6" t="inlineStr"/>
+      <c r="A190" s="6" t="inlineStr">
+        <is>
+          <t>| Why I wear red + black | I have always loved them; deep reason not revealed to me yet |</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="6" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>| My crest | Simple child crest: blade/flame between small parent marks |</t>
         </is>
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="6" t="inlineStr"/>
+      <c r="A192" s="6" t="inlineStr">
+        <is>
+          <t>| My sigil | One red/black blade or flame mark |</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="6" t="inlineStr">
         <is>
-          <t>## Secrets / do not spoil yet</t>
+          <t>| Crest tradition | Child crest = name + gender + both parents; simpler than parents; unique |</t>
         </is>
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="6" t="inlineStr"/>
+      <c r="A194" s="6" t="inlineStr">
+        <is>
+          <t>| Sigil tradition | Same day as crest; one quick seal mark |</t>
+        </is>
+      </c>
     </row>
     <row r="195">
-      <c r="A195" s="6" t="inlineStr">
-        <is>
-          <t>Use this when roleplaying what party members know.</t>
-        </is>
-      </c>
+      <c r="A195" s="6" t="inlineStr"/>
     </row>
     <row r="196">
-      <c r="A196" s="6" t="inlineStr"/>
+      <c r="A196" s="6" t="inlineStr">
+        <is>
+          <t>### Family crest / sigil cheat sheet</t>
+        </is>
+      </c>
     </row>
     <row r="197">
-      <c r="A197" s="6" t="inlineStr">
-        <is>
-          <t>| Topic | Party can know? | Notes |</t>
-        </is>
-      </c>
+      <c r="A197" s="6" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="6" t="inlineStr">
         <is>
-          <t>|---|---|---|</t>
+          <t>| Person | Colors | Crest idea | Sigil idea |</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="6" t="inlineStr">
         <is>
-          <t>| I am from Alzenhiem + family basics | Yes | Safe to share |</t>
+          <t>|---|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="6" t="inlineStr">
         <is>
-          <t>| Trained since 8 in the yard; from 12 under Rilock by Lion’s order | Yes | Clarify: Lion directed, Rilock taught |</t>
+          <t>| Dolkin | charcoal / iron / bronze | stone arch + hammer | hammer in arch |</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="6" t="inlineStr">
         <is>
-          <t>| People rumored I was Hero early | Yes | Emphasize it was rumor then |</t>
+          <t>| Fulfein | sage / silver / pale gold | leaf + crescent | leaf into crescent |</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="6" t="inlineStr">
         <is>
-          <t>| Yua made me Hero at 17 | Yes, if trust is there | She often looks like a pixie |</t>
+          <t>| Dezco | red / black | balanced blade/flame | red/black split blade |</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="6" t="inlineStr">
         <is>
-          <t>| Exact red/black blood meaning | No | Yua will tell me later; I do not know yet |</t>
+          <t>| Kalhien | blue / copper | forward eager mark | forward chevron |</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="6" t="inlineStr">
         <is>
-          <t>| Mana Well / sword imbue details | Not yet / soon | Yua stayed quiet on purpose; after my Saltrock faceplant she will explain |</t>
+          <t>| Astiale | rose / cream / sky | soft bud or star | soft bud/star |</t>
         </is>
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="6" t="inlineStr">
-        <is>
-          <t>| Full private family crest theology | Optional | Share lightly unless asked |</t>
-        </is>
-      </c>
+      <c r="A205" s="6" t="inlineStr"/>
     </row>
     <row r="206">
-      <c r="A206" s="6" t="inlineStr"/>
+      <c r="A206" s="6" t="inlineStr">
+        <is>
+          <t>Images: `assets/crests/alzenhiem/`</t>
+        </is>
+      </c>
     </row>
     <row r="207">
-      <c r="A207" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">**Red/black truth (for you / DM only, not my current knowledge):**  </t>
-        </is>
-      </c>
+      <c r="A207" s="6" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" s="6" t="inlineStr">
         <is>
-          <t>Black = Dwarven caves / void / dark over light. Red = Elven holy blood after ill happens. Together = balance.</t>
+          <t>---</t>
         </is>
       </c>
     </row>
@@ -6328,120 +7489,128 @@
     <row r="210">
       <c r="A210" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">**Mana Well truth (for you / DM; Yua explains after Saltrock biff):**  </t>
+          <t>## Secrets / do not spoil yet</t>
         </is>
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="6" t="inlineStr">
-        <is>
-          <t>Mana pool stored within soul confines but separate from the soul. Simple imbue makes sword lighter/sharper and grants a short agility burst. First accidental use: ~15 ft dash mid swing in journal 03, causing the faceplant. Needs training.</t>
-        </is>
-      </c>
+      <c r="A211" s="6" t="inlineStr"/>
     </row>
     <row r="212">
-      <c r="A212" s="6" t="inlineStr"/>
+      <c r="A212" s="6" t="inlineStr">
+        <is>
+          <t>Use this when roleplaying what party members know.</t>
+        </is>
+      </c>
     </row>
     <row r="213">
-      <c r="A213" s="6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="A213" s="6" t="inlineStr"/>
     </row>
     <row r="214">
-      <c r="A214" s="6" t="inlineStr"/>
+      <c r="A214" s="6" t="inlineStr">
+        <is>
+          <t>| Topic | Party can know? | Notes |</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="6" t="inlineStr">
         <is>
-          <t>## Abilities (Mana Well)</t>
+          <t>|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="6" t="inlineStr"/>
+      <c r="A216" s="6" t="inlineStr">
+        <is>
+          <t>| I am from Alzenhiem + family basics | Yes | Safe to share |</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="6" t="inlineStr">
         <is>
-          <t>| Piece | Quick fact |</t>
+          <t>| Trained since 8 in the yard; from 12 under Rilock by Lion’s order | Yes | Clarify: Lion directed, Rilock taught |</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| People rumored I was Hero early | Yes | Emphasize it was rumor then |</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="6" t="inlineStr">
         <is>
-          <t>| Source | Bestowed by Yua with the Hero charge; unexplained at first |</t>
+          <t>| Yua made me Hero at 17 | Yes, if trust is there | She often looks like a pixie |</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="6" t="inlineStr">
         <is>
-          <t>| Well | Stored mana pool within soul confines; separate from the soul |</t>
+          <t>| Yua walks with me daily | No | Only King’s Lion + Rilock know |</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="6" t="inlineStr">
         <is>
-          <t>| Simple imbue | Innate; should feel as easy as breathing once understood |</t>
+          <t>| A divine being was seen in the world | Yes | Public knowledge; not tied to me |</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="6" t="inlineStr">
         <is>
-          <t>| Sword effect | Lighter, sharper; short burst of swiftness / agility |</t>
+          <t>| I talk to empty air when stressed | They saw it | Bridge return; vine excuse worked for now |</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="6" t="inlineStr">
         <is>
-          <t>| First use | Saltrock battle (journal 03); accidental ~15 ft dash mid swing = faceplant |</t>
+          <t>| Exact red/black blood meaning | No | Yua will tell me later; I do not know yet |</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="6" t="inlineStr">
         <is>
-          <t>| Training needed | Control timing, avoid waste, move with the burst instead of being thrown |</t>
+          <t>| Mana Well / Lord AO gift | Partial | Yua named gift in private woods talk; training still ahead |</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="6" t="inlineStr">
         <is>
-          <t>| Yua’s plan | Stay quiet until I ask or figure it out; changed after watching me biff |</t>
+          <t>| Why I hide Yua from them | No | See yua-why-she-stays-hidden.md |</t>
         </is>
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="6" t="inlineStr"/>
+      <c r="A226" s="6" t="inlineStr">
+        <is>
+          <t>| Full private family crest theology | Optional | Share lightly unless asked |</t>
+        </is>
+      </c>
     </row>
     <row r="227">
-      <c r="A227" s="6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="A227" s="6" t="inlineStr"/>
     </row>
     <row r="228">
-      <c r="A228" s="6" t="inlineStr"/>
+      <c r="A228" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">**Red/black truth (for you / DM only, not my current knowledge):**  </t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="6" t="inlineStr">
         <is>
-          <t>## How I sound when I talk about myself</t>
+          <t>Black = Dwarven caves / void / dark over light. Red = Elven holy blood after ill happens. Together = balance.</t>
         </is>
       </c>
     </row>
@@ -6451,156 +7620,148 @@
     <row r="231">
       <c r="A231" s="6" t="inlineStr">
         <is>
-          <t>1. Honest, a little unsure about being chosen</t>
+          <t xml:space="preserve">**Mana Well truth (for you / DM; Yua explained partially in woods):**  </t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="6" t="inlineStr">
         <is>
-          <t>2. Proud of Alzenhiem without boasting</t>
+          <t>Mana pool stored within soul confines but separate from the soul. Gift from Lord AO per Yua after tomb road. Simple imbue makes sword lighter/sharper and grants a short agility burst. First accidental use: ~15 ft dash mid swing in street fight. Second use: deliberate cleave through two goblins in keep. Needs training. Yua senses unknown darkness ahead.</t>
         </is>
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="6" t="inlineStr">
-        <is>
-          <t>3. Corrects “Hero of centuries” rumors for the training years</t>
-        </is>
-      </c>
+      <c r="A233" s="6" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" s="6" t="inlineStr">
         <is>
-          <t>4. Speaks kindly about family, especially Astiale</t>
+          <t xml:space="preserve">**Yua hidden truth (for you / DM):**  </t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="6" t="inlineStr">
         <is>
-          <t>5. Does not claim to understand Yua fully</t>
+          <t>See `character/lore/yua-story-plots/yua-why-she-stays-hidden.md`. Hope must stay on mortal hands, not slide to worship of her presence.</t>
         </is>
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="6" t="inlineStr">
-        <is>
-          <t>6. Prefers no dramatic dash heavy speech; plain and direct</t>
-        </is>
-      </c>
+      <c r="A236" s="6" t="inlineStr"/>
     </row>
     <row r="237">
-      <c r="A237" s="6" t="inlineStr"/>
+      <c r="A237" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
     </row>
     <row r="238">
-      <c r="A238" s="6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="A238" s="6" t="inlineStr"/>
     </row>
     <row r="239">
-      <c r="A239" s="6" t="inlineStr"/>
+      <c r="A239" s="6" t="inlineStr">
+        <is>
+          <t>## Abilities (Mana Well)</t>
+        </is>
+      </c>
     </row>
     <row r="240">
-      <c r="A240" s="6" t="inlineStr">
-        <is>
-          <t>## Where the long versions are</t>
-        </is>
-      </c>
+      <c r="A240" s="6" t="inlineStr"/>
     </row>
     <row r="241">
-      <c r="A241" s="6" t="inlineStr"/>
+      <c r="A241" s="6" t="inlineStr">
+        <is>
+          <t>| Piece | Quick fact |</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="6" t="inlineStr">
         <is>
-          <t>| Need | File |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| Source | Bestowed by Yua with the Hero charge; unexplained at first |</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="6" t="inlineStr">
         <is>
-          <t>| Full character intro | `character/lore/dezco-knoleburn-character.md` |</t>
+          <t>| Well | Stored mana pool within soul confines; separate from the soul |</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="6" t="inlineStr">
         <is>
-          <t>| Journal index | `character/lore/journal/README.md` |</t>
+          <t>| Simple imbue | Innate; should feel as easy as breathing once understood |</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="6" t="inlineStr">
         <is>
-          <t>| Journal 01 (backstory) | `character/lore/journal/01-after-the-charge.md` |</t>
+          <t>| Sword effect | Lighter, sharper; short burst of swiftness / agility |</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="6" t="inlineStr">
         <is>
-          <t>| Journal 02 (leave home / Saltrock) | `character/lore/journal/02-leaving-home-for-saltrock.md` |</t>
+          <t>| First use | Saltrock street fight (journal 03); accidental ~15 ft dash mid swing = muddy faceplant |</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 (staff falls / mid siege) | `character/lore/journal/03-saltrock-staff-falls.md` |</t>
+          <t>| Second use | Keep goblin fight; cleaved one at waist, gutted another &gt;10 ft away |</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="6" t="inlineStr">
         <is>
-          <t>| Name meanings | `character/lore/knoleburn-names.md` |</t>
+          <t>| Yua’s explanation | Woods talk after tomb: gift from Lord AO; grow together through training |</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="6" t="inlineStr">
         <is>
-          <t>| Crest / sigil deep meanings | `assets/crests/alzenhiem/README.md` |</t>
+          <t>| Yua’s warning | Feels a darkness she has never known; source unknown |</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="6" t="inlineStr">
         <is>
-          <t>| Yua story plots index | `character/lore/yua-story-plots/README.md` |</t>
+          <t>| Training needed | Control timing, avoid waste, move with the burst instead of being thrown |</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="6" t="inlineStr">
         <is>
-          <t>| Red/black reveal (future) | `character/lore/yua-story-plots/yua-on-red-and-black.md` |</t>
+          <t>| Yua’s mood | Upset after bridge; said we need to talk later |</t>
         </is>
       </c>
     </row>
     <row r="253">
-      <c r="A253" s="6" t="inlineStr">
-        <is>
-          <t>| Mana Well / sword imbue | `character/lore/yua-story-plots/yua-mana-well.md` |</t>
-        </is>
-      </c>
+      <c r="A253" s="6" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" s="6" t="inlineStr">
         <is>
-          <t>| Downloadable Google export | `character/lore/exports/` (Sheets tabs `.xlsx` + Docs `.docx`) |</t>
+          <t>---</t>
         </is>
       </c>
     </row>
@@ -6610,7 +7771,7 @@
     <row r="256">
       <c r="A256" s="6" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>## How I sound when I talk about myself</t>
         </is>
       </c>
     </row>
@@ -6620,116 +7781,341 @@
     <row r="258">
       <c r="A258" s="6" t="inlineStr">
         <is>
-          <t>## Blank lines for new party facts</t>
+          <t>1. Honest, a little unsure about being chosen</t>
         </is>
       </c>
     </row>
     <row r="259">
-      <c r="A259" s="6" t="inlineStr"/>
+      <c r="A259" s="6" t="inlineStr">
+        <is>
+          <t>2. Proud of Alzenhiem without boasting</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="6" t="inlineStr">
         <is>
-          <t>Add new rows here whenever something new becomes true in play:</t>
+          <t>3. Corrects “Hero of centuries” rumors for the training years</t>
         </is>
       </c>
     </row>
     <row r="261">
-      <c r="A261" s="6" t="inlineStr"/>
+      <c r="A261" s="6" t="inlineStr">
+        <is>
+          <t>4. Speaks kindly about family, especially Astiale</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="6" t="inlineStr">
         <is>
-          <t>| Date / session | New fact | Share with party? |</t>
+          <t>5. Does not claim to understand Yua fully</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="6" t="inlineStr">
         <is>
-          <t>|---|---|---|</t>
+          <t>6. Prefers no dramatic dash heavy speech; plain and direct</t>
         </is>
       </c>
     </row>
     <row r="264">
-      <c r="A264" s="6" t="inlineStr">
-        <is>
-          <t>| Journal 02 | Left Alzenhiem with Dolkin’s sword + smithing tools; Fulfein’s gold, pot, clothes, shovel | Yes |</t>
-        </is>
-      </c>
+      <c r="A264" s="6" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" s="6" t="inlineStr">
         <is>
-          <t>| Journal 02 | Shovel is mom’s bathroom dig joke first; burial meaning is the quiet second read | Optional / tonal |</t>
+          <t>---</t>
         </is>
       </c>
     </row>
     <row r="266">
-      <c r="A266" s="6" t="inlineStr">
-        <is>
-          <t>| Journal 02 | In Saltrock tavern overnight; knows the floating protective staff | Yes |</t>
-        </is>
-      </c>
+      <c r="A266" s="6" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Saltrock staff fell; crabs + creatures attacked | Yes |</t>
+          <t>## Where the long versions are</t>
         </is>
       </c>
     </row>
     <row r="268">
-      <c r="A268" s="6" t="inlineStr">
-        <is>
-          <t>| Journal 03 | Missed a short bow creature; faceplant; nearly shot; saved by elf girl archer | Yes |</t>
-        </is>
-      </c>
+      <c r="A268" s="6" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Faceplant tied to accidental ~15 ft mana dash / simple imbue (not understood yet) | After Yua explains |</t>
+          <t>| Need | File |</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Sealed in general building with townsfolk; people outside unknown; story paused mid siege | Yes |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="6" t="inlineStr">
         <is>
-          <t>| Yua plots | Mana Well bestowed at Hero charge; Yua will explain after watching the biff | After she tells me |</t>
+          <t>| Full character intro | `character/lore/dezco-knoleburn-character.md` |</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="6" t="inlineStr">
         <is>
-          <t>| Lore | Birthday is November 6 | Yes |</t>
+          <t>| Journal index | `character/lore/journal/README.md` |</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="6" t="inlineStr">
         <is>
-          <t>| Export | Tabbed Sheets + Docs lore pack in character/lore/exports/ | Yes |</t>
+          <t>| Journal 01 (backstory) | `character/lore/journal/01-after-the-charge.md` |</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="6" t="inlineStr">
         <is>
-          <t>| Lore | Trainer is Rilock (royal master swordsman); King’s Lion directed him | Yes |</t>
+          <t>| Journal 02 (leave home / Saltrock) | `character/lore/journal/02-leaving-home-for-saltrock.md` |</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="6" t="inlineStr">
+        <is>
+          <t>| Journal 03 (full) | `character/lore/journal/03-saltrock-staff-falls.md` |</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="6" t="inlineStr">
+        <is>
+          <t>| Yua hidden from party | `character/lore/yua-story-plots/yua-why-she-stays-hidden.md` |</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="6" t="inlineStr">
+        <is>
+          <t>| Name meanings | `character/lore/knoleburn-names.md` |</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="6" t="inlineStr">
+        <is>
+          <t>| Crest / sigil deep meanings | `assets/crests/alzenhiem/README.md` |</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="6" t="inlineStr">
+        <is>
+          <t>| Yua story plots index | `character/lore/yua-story-plots/README.md` |</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="6" t="inlineStr">
+        <is>
+          <t>| Red/black reveal (future) | `character/lore/yua-story-plots/yua-on-red-and-black.md` |</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="6" t="inlineStr">
+        <is>
+          <t>| Mana Well / sword imbue | `character/lore/yua-story-plots/yua-mana-well.md` |</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="6" t="inlineStr">
+        <is>
+          <t>| Downloadable Google export | `character/lore/exports/` (Sheets tabs `.xlsx` + Docs `.docx`) |</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="6" t="inlineStr"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="6" t="inlineStr"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="6" t="inlineStr">
+        <is>
+          <t>## Blank lines for new party facts</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="6" t="inlineStr"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="6" t="inlineStr">
+        <is>
+          <t>Add new rows here whenever something new becomes true in play:</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="6" t="inlineStr"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="6" t="inlineStr">
+        <is>
+          <t>| Date / session | New fact | Share with party? |</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="6" t="inlineStr">
+        <is>
+          <t>|---|---|---|</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="6" t="inlineStr">
+        <is>
+          <t>| Journal 02 | Left Alzenhiem with Dolkin’s sword + smithing tools; Fulfein’s gold, pot, clothes, shovel | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="6" t="inlineStr">
+        <is>
+          <t>| Journal 02 | Shovel is mom’s bathroom dig joke first; burial meaning is the quiet second read | Optional / tonal |</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="6" t="inlineStr">
+        <is>
+          <t>| Journal 02 | In Saltrock tavern overnight; knows the floating protective staff | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="6" t="inlineStr">
+        <is>
+          <t>| Journal 03 | Saltrock staff fell; crabs + creatures attacked | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="6" t="inlineStr">
+        <is>
+          <t>| Journal 03 | Missed a short bow creature; faceplant in wet muddy gravel; nearly shot; saved by Eden | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="6" t="inlineStr">
+        <is>
+          <t>| Journal 03 | Faceplant tied to accidental ~15 ft mana dash / simple imbue (not understood yet) | After Yua explains |</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="6" t="inlineStr">
+        <is>
+          <t>| Journal 03 | Keep siege: troll (magic resistant, regenerating) + 5 goblins; Eden/fire; second imbue on goblins | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="6" t="inlineStr">
+        <is>
+          <t>| Journal 03 | Party names: Eden, Alice, Jylia, Vita, Alem | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="6" t="inlineStr">
+        <is>
+          <t>| Journal 03 | First King’s Lion tomb quest; library map; Yolon; owlbear bridge; focus recovered | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="6" t="inlineStr">
+        <is>
+          <t>| Journal 03 | Yua visible only to me; party doubts path until Vita confirms map | No (hide Yua) |</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="6" t="inlineStr">
+        <is>
+          <t>| Journal 03 | Talked to air on bridge; blamed dragon statue vines | They believe vine story |</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="6" t="inlineStr">
+        <is>
+          <t>| Journal 03 | Lord AO gift named in woods; Yua warns of unknown darkness | Private for now |</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="6" t="inlineStr">
+        <is>
+          <t>| Journal 03 | Focus restored Saltrock; feast; choose Lyndor escort vs Lořel with Yeara by dawn | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="6" t="inlineStr">
+        <is>
+          <t>| Journal 03 | Foot hurt from 15 ft cliff fall; Eden smacked my hand with bow; Alice + Vita saved me | Yes (embarrassing) |</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="6" t="inlineStr">
+        <is>
+          <t>| Yua plots | Mana Well bestowed at Hero charge; Yua will explain after watching the biff | After she tells me |</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="6" t="inlineStr">
+        <is>
+          <t>| Lore | Birthday is November 6 | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="6" t="inlineStr">
+        <is>
+          <t>| Export | Tabbed Sheets + Docs lore pack in character/lore/exports/ | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="6" t="inlineStr">
+        <is>
+          <t>| Lore | Trainer is Rilock (royal master swordsman); King’s Lion directed him | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="6" t="inlineStr">
         <is>
           <t>| | | |</t>
         </is>
@@ -6980,7 +8366,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Saltrock general building (doors sealed; under attack)</t>
+          <t>Saltrock (protection restored; feast over; dawn choice pending)</t>
         </is>
       </c>
     </row>
@@ -6992,7 +8378,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Adventure day 2 gone wrong; protective staff fell; mid siege</t>
+          <t>Adventure day 2; staff fell then focus restored; Lyndor vs Lořel by morning</t>
         </is>
       </c>
     </row>
@@ -7448,7 +8834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7616,7 +9002,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Protective staff fell; monster attack</t>
+          <t>Protective staff fell; storm attack; accidental mana dash / muddy faceplant; Eden saved him</t>
         </is>
       </c>
     </row>
@@ -7628,19 +9014,31 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Accidental mana dash / faceplant; elf girl archer save</t>
+          <t>Keep siege: troll + goblins; second imbue; first King’s Lion tomb quest; focus recovered</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Focus restored with mayor, Vita, Yeara; feast; choose Lyndor escort or Lořel</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Sealed in Saltrock general building; journal 03 open ended</t>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Resting after feast; foot bruised; Yua and Dezco still need to talk</t>
         </is>
       </c>
     </row>
@@ -7655,11 +9053,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="62" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -7720,7 +9118,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Traveling town; many come and go</t>
+          <t>Traveling town; focus restored; feast; dawn choice pending</t>
         </is>
       </c>
     </row>
@@ -7732,12 +9130,12 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Saltrock general building</t>
+          <t>Saltrock keep / general building</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Protective staff location; currently sealed inside during attack</t>
+          <t>Shelter during attack; focus set back with Vita and Yeara</t>
         </is>
       </c>
     </row>
@@ -7749,12 +9147,12 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Saltrock protective staff</t>
+          <t>Saltrock library</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Used to float and block named monsters; has fallen</t>
+          <t>Old map book to first King’s Lion tomb</t>
         </is>
       </c>
     </row>
@@ -7766,97 +9164,97 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Saltrock tavern</t>
+          <t>Lyndor</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Lodged night before attack; nostalgia bread</t>
+          <t>Capital; Lord Keivan; mayor wants escort</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Gear</t>
+          <t>Place</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>New sword</t>
+          <t>Lořel</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>From Dolkin; hand forged goodbye</t>
+          <t>City of churches; priestess Yeara wants the party there</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Gear</t>
+          <t>Place</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>First smithing tools</t>
+          <t>First King’s Lion tomb</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>From Dolkin; master of your steel</t>
+          <t>Hilltop beyond Saltrock; held the recovered focus</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Gear</t>
+          <t>Place</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>10 gold pieces</t>
+          <t>Yolon statue</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>From Fulfein</t>
+          <t>Stone dragon on tomb path; spoke after rain bowl drink</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Gear</t>
+          <t>Place</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Cooking pot</t>
+          <t>Owlbear bridge</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>From Fulfein</t>
+          <t>Rickety crossing past sleeping giant owlbear</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Gear</t>
+          <t>Place</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>New clothing</t>
+          <t>Saltrock tavern</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>From Fulfein; worn out of respect</t>
+          <t>Lodged night before attack; nostalgia bread</t>
         </is>
       </c>
     </row>
@@ -7868,12 +9266,114 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
+          <t>New sword</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>From Dolkin; hand forged goodbye</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Gear</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>First smithing tools</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>From Dolkin; master of your steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Gear</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>10 gold pieces</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>From Fulfein</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Gear</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Cooking pot</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>From Fulfein</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Gear</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>New clothing</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>From Fulfein; worn out of respect</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Gear</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
           <t>Shovel</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>From Fulfein; funny roadside duty + darker second meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Gear</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Tomb focus (recovered)</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Faint glow; restored Saltrock protection with mayor, Vita, Yeara</t>
         </is>
       </c>
     </row>
@@ -8313,7 +9813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -8355,7 +9855,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Bestowed by Yua with the Hero charge; unexplained at first</t>
+          <t>Gift from Lord AO per Yua; Well bestowed with Hero charge</t>
         </is>
       </c>
     </row>
@@ -8403,31 +9903,55 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Saltrock battle (journal 03); accidental ~15 ft dash mid swing = faceplant</t>
+          <t>Saltrock street fight; accidental ~15 ft dash mid swing = muddy faceplant</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Training needed</t>
+          <t>Second use</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Control timing, avoid waste, move with the burst instead of being thrown</t>
+          <t>Keep goblin fight; cleaved one at waist, gutted another &gt;10 ft away</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Yua’s plan</t>
+          <t>Yua’s explanation</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Stay quiet until Dezco asks or figures it out; changed after watching the biff</t>
+          <t>Woods talk: Lord AO gift; grow together through training</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Yua’s warning</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Feels unknown darkness; source not yet named</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Training needed</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Control timing, avoid waste, move with the burst instead of being thrown</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore missing Journal 03 details from original prompt
Clarify Yolon's right-fork direction, the river vs cliff split with
Eden and Alice, owlbear and bridge specifics, King's Lion library
quest, troll fight beats, and return journey details.

Co-authored-by: Dralorex <Dralorex@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/character/lore/exports/Dezco_Knoleburn_Lore_Tabs.xlsx
+++ b/character/lore/exports/Dezco_Knoleburn_Lore_Tabs.xlsx
@@ -2840,7 +2840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A173"/>
+  <dimension ref="A1:A183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -3108,7 +3108,7 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>A troll broke through with five goblins pouring behind it. The same defenders gathered again. A human priest joined us in the chaos, Vita, early thirties, robes soaked, voice steady. He had already healed a snake man among us, Alem, who speaks mind to mind when words are too slow.</t>
+          <t>A troll broke through the back wall with five goblins pouring behind it. The same defenders gathered again. A human priest joined us in the chaos, Vita, early thirties, robes soaked, voice steady. He had already healed a snake man among us, Alem, who speaks mind to mind when words are too slow.</t>
         </is>
       </c>
     </row>
@@ -3118,7 +3118,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>I had seen trolls in training records. I had never stood against one. This one was worse than the texts. Spells slid off it like rain off slate. Wounds closed as soon as they opened. Eden found the crack in its hide: fire. While the others hammered it from the front, I slipped to the rear to keep the goblins from flanking.</t>
+          <t>I had seen trolls in training records. I had never stood against one. From the first swing I knew this fight would not be easy. This one was worse than the texts. It resisted all magic. Spells slid off it like rain off slate. Wounds closed on the spot as soon as they opened. Eden found the crack in its hide: fire. While the others hammered it from the front, I slipped to the rear to keep the goblins from flanking and to hold the troll as the only problem worth fearing.</t>
         </is>
       </c>
     </row>
@@ -3148,7 +3148,7 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>Not fear this time. Not accident alone. The blade felt hungry. My legs felt ready. I surged forward through the space in front of me and cleaved the first goblin clean at the waist. The momentum did not stop. The edge found a second goblin more than ten feet away and opened his gut. He stumbled, ruined but not yet dead.</t>
+          <t>Again it felt as if the sword was eager to fight and my body was eager to move with it. I bolted forward through the space in front of me and sliced straight through the first goblin, cutting him in two at the waist. The momentum did not stop. The edge found a second goblin more than ten feet away and opened his gut. Not quite enough to kill him, but he was not looking good.</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>When I turned, the troll was a burning heap collapsing to the floor. Goblins broke and ran. The wounded one made it only a few strides before Eden put an arrow through his back.</t>
+          <t>When I turned, the troll was burning to a crisp. It thumped to the floor, motionless, while everyone watched it fall. Goblins broke and ran. The wounded one made it only a few strides before Eden shot him in the back and finished him off.</t>
         </is>
       </c>
     </row>
@@ -3178,7 +3178,7 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>Then the mayor found us and said the fight was not over.</t>
+          <t>Then the mayor found us and said the fight was not over. We still had work to do before Saltrock could breathe.</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>He spoke of a title I already knew from my own life, though not this far back in its bloodline.</t>
+          <t>He spoke of a grave, and of a title I already knew from my own life, though not this far back in its bloodline.</t>
         </is>
       </c>
     </row>
@@ -3208,7 +3208,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>The King’s Lion serves the holy city’s king and is said to be the realm’s greatest living swordsman. Each Lion succeeds the last. The first of that line is buried in a tomb somewhere beyond Saltrock. The mayor did not know where. The library might.</t>
+          <t>The King’s Lion is the name of the chief guard who stands at the holy city king’s side. Each generation’s Lion is believed to be the realm’s greatest living swordsman, and every Lion must succeed the one before him. The first of that line is buried in a tomb somewhere beyond Saltrock. The mayor did not know where. He said the library might hold answers.</t>
         </is>
       </c>
     </row>
@@ -3228,7 +3228,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>Vita deciphered an old book the rest of us could barely read. More than a hundred years of shifting land lay between its map and the world. Still, it gave a direction. We left at once.</t>
+          <t>We searched the library and found an old book with a location for the grave. Vita was the only one among us who could read it. The map inside was more than a hundred years old. Rivers had moved. Hills had softened. Roads had vanished. It was not precise, but it gave us a direction, and we set off at once.</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>On the path Yua appeared at my shoulder, visible only to me, and pointed the way the road should bend. The others doubted me. I told them to check the book. Vita did. The scrappy map inside matched the terrain in the direction I had named. They stopped arguing. They did not stop watching me oddly.</t>
+          <t>On the path Yua appeared at my shoulder, visible only to me, and pointed the way the road should bend. The group doubted me. I told them to look at the book. Vita looked back into it and, based on the old scrappy map inside, agreed the terrain matched the direction I had named. They stopped arguing. They did not stop watching me oddly.</t>
         </is>
       </c>
     </row>
@@ -3328,7 +3328,7 @@
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>It rose from the hillside crusted in moss, mud, and old vines: a dragon carved in stone with a bowl at its feet. Something in me wanted to pray there, not to the dragon itself, but near it. When I did, warmth moved through my chest like an ember carefully placed. I felt steadier on the road we were already walking.</t>
+          <t>It rose from the hillside crusted in grime from years upon years of weather: mud, moss, vines, and filth packed into every carved scale. Up close it was a dragon carved in stone with a wide bowl set before its feet.</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3338,7 @@
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>Jylia drank the rainwater pooled in the bowl.</t>
+          <t>Something in me wanted to pray there, not to the dragon itself, but simply to pray beside it. When I did, an odd warmth moved through my chest like an ember carefully placed. I felt inspired to keep walking the path we were already on.</t>
         </is>
       </c>
     </row>
@@ -3348,7 +3348,7 @@
     <row r="99">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>The statue spoke without moving its mouth.</t>
+          <t>Right as I finished, Jylia drank the rainwater pooled in the bowl.</t>
         </is>
       </c>
     </row>
@@ -3358,7 +3358,7 @@
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>His name is Yolon. He was a true dragon once, turned to stone as magic thinned from the world. He has stood there more than a hundred years waiting to be freed. When we asked about the first King’s Lion, he laughed until the sound rolled through the wet trees.</t>
+          <t>The statue spoke without moving its mouth.</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>He had fought that Lion many times. Battles that went on until both of them were spent. Every duel ended in a draw. Every duel made them stronger. In time they stopped trying to kill each other and simply tested one another, as if respect had outgrown victory. Yolon never learned the Lion’s final fate, but he knew where the tomb lay.</t>
+          <t>His name is Yolon. He was a true dragon once, turned to stone as magic thinned from the world. He has stood there more than a hundred years, waiting to be freed. We told him our quest: find the tomb of the first King’s Lion.</t>
         </is>
       </c>
     </row>
@@ -3378,7 +3378,7 @@
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>Keep on this path, he said. Eventually take the right fork.</t>
+          <t>At the name King’s Lion, he roared into laughter until the sound rolled through the wet trees.</t>
         </is>
       </c>
     </row>
@@ -3388,7 +3388,7 @@
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>We thanked him and went on.</t>
+          <t>He had fought that Lion many times. Battles that went on forever, never relenting, and each one always ended in a draw. Every duel made them both stronger. In time they realized neither truly wanted the other dead. They sparred instead, testing strength the way honest warriors do when respect outgrows victory. Yolon never learned the first Lion’s final fate, but he knew where the tomb lay.</t>
         </is>
       </c>
     </row>
@@ -3398,7 +3398,7 @@
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>## The Bridge and the Owlbear</t>
+          <t>Keep following the path you are on, he said. When you reach the next fork, take the right.</t>
         </is>
       </c>
     </row>
@@ -3408,7 +3408,7 @@
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>The right fork brought us to a wooden bridge so old it complained under its own weight. Across it sat a boulder that looked deliberately wrong, like a lump dropped by a careless giant.</t>
+          <t>We thanked him and went on.</t>
         </is>
       </c>
     </row>
@@ -3418,7 +3418,7 @@
     <row r="113">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>Eden vanished while we debated how to cross. By the time we noticed, she was already on the far side.</t>
+          <t>## The Bridge and the Owlbear</t>
         </is>
       </c>
     </row>
@@ -3428,7 +3428,7 @@
     <row r="115">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>Alem reached her with telepathy. Eden’s thoughts came back to us in pieces. Inside the stone slept an owlbear, the largest she had ever seen: bear body, owl head, claws long enough to split a person in two. Lucky for us, it was still sleeping.</t>
+          <t>Yolon’s path brought us to an old, rickety wooden bridge that groaned under its own weight. On the far side sat an odd shaped boulder we did not trust. It felt deliberately out of place, like a lump dropped by a careless giant.</t>
         </is>
       </c>
     </row>
@@ -3438,7 +3438,7 @@
     <row r="117">
       <c r="A117" s="6" t="inlineStr">
         <is>
-          <t>One by one we crossed as Eden directed our steps. One board. One breath. No sound. Somehow every one of us made it over.</t>
+          <t>Eden vanished while we debated how to cross. By the time we noticed, she was already on the other side.</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3448,7 @@
     <row r="119">
       <c r="A119" s="6" t="inlineStr">
         <is>
-          <t>At the next split, the elven sisters went down toward the river. The rest of us climbed the cliff stairs.</t>
+          <t>Alem reached her with telepathy, speaking mind to mind. Eden relayed what she found. Inside that false boulder slept an owlbear, the largest she had ever seen: the body of a bear, the head and beak of an owl, giant claws jutting from its fists, claws long enough to slash a person in half. Lucky for us, it was still sleeping.</t>
         </is>
       </c>
     </row>
@@ -3458,7 +3458,7 @@
     <row r="121">
       <c r="A121" s="6" t="inlineStr">
         <is>
-          <t>## The Tomb and the Focus</t>
+          <t>The bridge was so old and so rickety that crossing it wrong could wake the beast. We had to figure out how to get across without a sound. One at a time, we took the steps Eden told us to take. One board. One breath. No creak we could avoid. Somehow, by the luck of our skin, every one of us made it over.</t>
         </is>
       </c>
     </row>
@@ -3468,7 +3468,7 @@
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
         <is>
-          <t>At the hilltop we found a heavy door set into stone.</t>
+          <t>## The Fork Yolon Named</t>
         </is>
       </c>
     </row>
@@ -3478,7 +3478,7 @@
     <row r="125">
       <c r="A125" s="6" t="inlineStr">
         <is>
-          <t>Jylia pushed it open without hesitation.</t>
+          <t>Farther on we reached the fork he had warned us about.</t>
         </is>
       </c>
     </row>
@@ -3488,7 +3488,7 @@
     <row r="127">
       <c r="A127" s="6" t="inlineStr">
         <is>
-          <t>Goblins. Maybe five. The same breed that hit the keep. We cut them down fast, almost embarrassingly so. We dragged the bodies aside and went deeper.</t>
+          <t>One path dropped toward the rivers below. The other climbed a cliff in a long run of stone stairs to the hilltop. Yolon had said to go right. The right path was the stairs.</t>
         </is>
       </c>
     </row>
@@ -3498,7 +3498,7 @@
     <row r="129">
       <c r="A129" s="6" t="inlineStr">
         <is>
-          <t>The real tomb waited beyond.</t>
+          <t>Eden and Alice went left, down toward the water. The rest of us went right, up the cliff. I do not know yet what the sisters found by the river. We had a tomb to reach.</t>
         </is>
       </c>
     </row>
@@ -3508,7 +3508,7 @@
     <row r="131">
       <c r="A131" s="6" t="inlineStr">
         <is>
-          <t>Inside we found a focus, faintly glowing, beautiful, and completely mysterious. None of us knew what it did. I wanted to hold it longer than I should have.</t>
+          <t>## The Tomb and the Focus</t>
         </is>
       </c>
     </row>
@@ -3518,7 +3518,7 @@
     <row r="133">
       <c r="A133" s="6" t="inlineStr">
         <is>
-          <t>When we climbed back out, sunlight hit my face for the first time since the attack began. I thought that meant relief.</t>
+          <t>At the hilltop we found a tomb with a large door set into the stone.</t>
         </is>
       </c>
     </row>
@@ -3528,7 +3528,7 @@
     <row r="135">
       <c r="A135" s="6" t="inlineStr">
         <is>
-          <t>I spoke to Yua about the tingling in battle. She knew what it was and could not say. Like the knowledge lived beneath language and would not come up when I demanded it. I did not ask well. I think I angered her.</t>
+          <t>Jylia pushed it open without hesitation.</t>
         </is>
       </c>
     </row>
@@ -3538,7 +3538,7 @@
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>On the return path something lifted me two feet off the ground and dropped me over a fifteen foot edge. No proof. Strong suspicion. My foot hurts. So does whatever pride I had left.</t>
+          <t>Goblins. Five of them, maybe the same breed that hit the keep. We took them out fast, without much issue. We moved the bodies aside and went deeper.</t>
         </is>
       </c>
     </row>
@@ -3548,7 +3548,7 @@
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
         <is>
-          <t>At the bridge the owlbear was gone. We saw no sign of it. We counted that as blessing and did not question fortune too loudly.</t>
+          <t>The real tomb waited beyond.</t>
         </is>
       </c>
     </row>
@@ -3558,7 +3558,7 @@
     <row r="141">
       <c r="A141" s="6" t="inlineStr">
         <is>
-          <t>I tried to recreate the lift Yua had given me, if it was her at all. I attempted to leap a gap back onto the bridge. Nothing answered. I fell. One hand caught the edge. Eden reached with her bow to help. She smacked my fingers instead. I dropped farther. Alice caught my other hand. Vita hauled us both up.</t>
+          <t>We opened it and found a focus inside. It had a slight glow to it and looked genuinely cool sitting there in the dark. None of us had any idea what it did. I wanted to hold it longer than I should have.</t>
         </is>
       </c>
     </row>
@@ -3568,7 +3568,7 @@
     <row r="143">
       <c r="A143" s="6" t="inlineStr">
         <is>
-          <t>I shouted at empty air afterward. Yua was furious, or hurt, or both. She said we would need to talk later. The party saw only a boy cursing at nothing. I blamed the vines on Yolon’s statue. That lie held.</t>
+          <t>When we climbed back out, sunlight hit my face for the first time since the battles started. I thought that meant relief.</t>
         </is>
       </c>
     </row>
@@ -3578,7 +3578,7 @@
     <row r="145">
       <c r="A145" s="6" t="inlineStr">
         <is>
-          <t>On the way back Vita collected those same vines for herbs, or so he said. I hope that is true. The vines did nothing to me. I was only scrambling for an excuse.</t>
+          <t>I spoke to Yua about the tingling in battle. She knew what it was, but she could not pull the answer forward, as if the knowledge lived in some subconscious place she could feel but not reach. I did not bring it up in the best way. I think I angered her.</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3588,7 @@
     <row r="147">
       <c r="A147" s="6" t="inlineStr">
         <is>
-          <t>## What Yua Told Me in the Woods</t>
+          <t>On the return path something lifted me two feet off the ground and dropped me over a fifteen foot cliff edge. No proof. Strong suspicion. My foot hurts. So does whatever pride I had left.</t>
         </is>
       </c>
     </row>
@@ -3598,7 +3598,7 @@
     <row r="149">
       <c r="A149" s="6" t="inlineStr">
         <is>
-          <t>When Saltrock came into view again, I slipped away to speak with her alone.</t>
+          <t>When we reached the bridge again, the owlbear was gone. We did not even search properly. We simply could not see it anywhere. We counted that as a blessing.</t>
         </is>
       </c>
     </row>
@@ -3608,7 +3608,7 @@
     <row r="151">
       <c r="A151" s="6" t="inlineStr">
         <is>
-          <t>She remembered more there than she had on the mountain. She said I had received a gift directly from Lord AO. We would have to grow together and learn the power through training. No shortcuts. No temper.</t>
+          <t>I tried to recreate the lift Yua had given me, if it was her at all. I attempted to jump a gap back onto the bridge. Nothing answered. I started to fall into the deep cavern below. One hand barely hooked the edge. Eden reached with her bow to help me grab it. She smacked my fingers instead. I lost my grip and dropped farther. Alice caught my other hand just in time. Vita came over and helped pull me all the way up.</t>
         </is>
       </c>
     </row>
@@ -3618,7 +3618,7 @@
     <row r="153">
       <c r="A153" s="6" t="inlineStr">
         <is>
-          <t>She also said she feels a darkness unlike any she has known. She does not know its source yet. Only that I should be careful.</t>
+          <t>I shouted at empty air afterward. Yua was furious, or hurt, or both. She said we would need to talk later. The party saw only a boy cursing at nothing. I blamed the vines on Yolon’s statue. That lie held.</t>
         </is>
       </c>
     </row>
@@ -3628,7 +3628,7 @@
     <row r="155">
       <c r="A155" s="6" t="inlineStr">
         <is>
-          <t>I rejoined the group with mud on my knees and no good answers for their questions.</t>
+          <t>On the way back we passed the dragon statue again. Vita collected those same vines for herbs, or so he said. I hope that is true. The vines did nothing to me. I was only scrambling for an excuse.</t>
         </is>
       </c>
     </row>
@@ -3638,7 +3638,7 @@
     <row r="157">
       <c r="A157" s="6" t="inlineStr">
         <is>
-          <t>## The Focus Restored</t>
+          <t>## What Yua Told Me in the Woods</t>
         </is>
       </c>
     </row>
@@ -3648,7 +3648,7 @@
     <row r="159">
       <c r="A159" s="6" t="inlineStr">
         <is>
-          <t>We brought the glowing focus home.</t>
+          <t>When Saltrock came into view again, I walked away from the group into the woods to speak with her alone.</t>
         </is>
       </c>
     </row>
@@ -3658,7 +3658,7 @@
     <row r="161">
       <c r="A161" s="6" t="inlineStr">
         <is>
-          <t>The mayor, Vita, and a priestess named Yeara set it back into place. Protection returned to Saltrock. For the first time since the staff fell, the town felt like it might hold.</t>
+          <t>She remembered more there than she had on the mountain. She said I had received a gift directly from Lord AO. Yua and I would have to grow together and learn the power through training. No shortcuts. No temper.</t>
         </is>
       </c>
     </row>
@@ -3668,7 +3668,7 @@
     <row r="163">
       <c r="A163" s="6" t="inlineStr">
         <is>
-          <t>Then choice arrived with gratitude.</t>
+          <t>She also said she feels a darkness she has never felt before. She is not sure from what or whom. Only that I should be careful.</t>
         </is>
       </c>
     </row>
@@ -3678,7 +3678,7 @@
     <row r="165">
       <c r="A165" s="6" t="inlineStr">
         <is>
-          <t>The mayor wants us to escort him to Lyndor, the capital, to stand before Lord Keivan. Yeara wants us instead to travel with her to Lořel, the city of churches. We are to decide by morning.</t>
+          <t>I rejoined the group with mud on my knees and no good answers for their questions.</t>
         </is>
       </c>
     </row>
@@ -3688,7 +3688,7 @@
     <row r="167">
       <c r="A167" s="6" t="inlineStr">
         <is>
-          <t>Tonight they threw a feast to celebrate survival. After the food, the music, and too many eyes on me, I finally slept.</t>
+          <t>## The Focus Restored</t>
         </is>
       </c>
     </row>
@@ -3698,7 +3698,7 @@
     <row r="169">
       <c r="A169" s="6" t="inlineStr">
         <is>
-          <t>Tomorrow we choose a road.</t>
+          <t>We brought the focus back to the mayor.</t>
         </is>
       </c>
     </row>
@@ -3708,19 +3708,69 @@
     <row r="171">
       <c r="A171" s="6" t="inlineStr">
         <is>
-          <t>*Dezco Knoleburn*</t>
+          <t>He worked with Vita and a priestess named Yeara to set it back into place. Protection returned to Saltrock. For the first time since the staff fell, the town felt like it might hold.</t>
         </is>
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="6" t="inlineStr">
-        <is>
-          <t>*Saltrock, after the feast*</t>
-        </is>
-      </c>
+      <c r="A172" s="6" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="6" t="inlineStr">
+        <is>
+          <t>Then choice arrived with gratitude.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="6" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="6" t="inlineStr">
+        <is>
+          <t>The mayor wants us to escort him to Lyndor, the capital, to stand before Lord Keivan. Yeara wants us instead to travel with her to Lořel, the city of churches. They have asked us to decide by morning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="6" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="6" t="inlineStr">
+        <is>
+          <t>Tonight they threw a feast to celebrate survival. After the food, the music, and too many eyes on me, I finally got to rest for the night.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="6" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="6" t="inlineStr">
+        <is>
+          <t>Tomorrow we choose a road.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="6" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="6" t="inlineStr">
+        <is>
+          <t>*Dezco Knoleburn*</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="6" t="inlineStr">
+        <is>
+          <t>*Saltrock, after the feast*</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="6" t="inlineStr">
         <is>
           <t>*To be continued*</t>
         </is>
@@ -6204,7 +6254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A310"/>
+  <dimension ref="A1:A311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -6254,7 +6304,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">**Last updated:** 2026-08-23 (Journal 03 complete: tomb quest, focus restored, feast, dawn choice)  </t>
+          <t xml:space="preserve">**Last updated:** 2026-08-23 (Journal 03 detail pass: Yolon fork, river split, owlbear bridge)  </t>
         </is>
       </c>
     </row>
@@ -6978,7 +7028,7 @@
     <row r="125">
       <c r="A125" s="6" t="inlineStr">
         <is>
-          <t>| Yolon | Stone dragon statue (&gt;100 years); spoke after Jylia drank bowl rain; fought first King’s Lion to endless draws; gave tomb direction |</t>
+          <t>| Yolon | Stone dragon statue (&gt;100 years); spoke after Jylia drank bowl rain; fought first King’s Lion to endless draws; said take the right fork at the next split |</t>
         </is>
       </c>
     </row>
@@ -7178,944 +7228,951 @@
     <row r="157">
       <c r="A157" s="6" t="inlineStr">
         <is>
-          <t>| Yolon statue | Stone dragon with rain bowl on tomb path; spoke when Jylia drank; pointed us onward |</t>
+          <t>| Yolon statue | Stone dragon with rain bowl on tomb path; grime, moss, vines; spoke when Jylia drank; said keep path then take right at fork |</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="6" t="inlineStr">
         <is>
-          <t>| Owlbear bridge | Rickety crossing; sleeping giant owlbear in false boulder; gone on return trip |</t>
+          <t>| Tomb road fork | Left path down to rivers (Eden + Alice went); right path cliff stairs to hilltop tomb (rest of party) |</t>
         </is>
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="6" t="inlineStr"/>
+      <c r="A159" s="6" t="inlineStr">
+        <is>
+          <t>| Owlbear bridge | Rickety crossing past false boulder; sleeping giant owlbear inside; gone on return trip |</t>
+        </is>
+      </c>
     </row>
     <row r="160">
-      <c r="A160" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">**First magic item I ever saw:** the floating protective staff in Saltrock.  </t>
-        </is>
-      </c>
+      <c r="A160" s="6" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">**Current crisis resolved:** focus back in place; town shielded again.  </t>
+          <t xml:space="preserve">**First magic item I ever saw:** the floating protective staff in Saltrock.  </t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">**Current crisis resolved:** focus back in place; town shielded again.  </t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="6" t="inlineStr">
+        <is>
           <t>**Current dilemma:** escort mayor to Lyndor vs travel with Yeara to Lořel; decide by morning.</t>
         </is>
       </c>
     </row>
-    <row r="163">
-      <c r="A163" s="6" t="inlineStr"/>
-    </row>
     <row r="164">
-      <c r="A164" s="6" t="inlineStr">
+      <c r="A164" s="6" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="165">
-      <c r="A165" s="6" t="inlineStr"/>
-    </row>
     <row r="166">
-      <c r="A166" s="6" t="inlineStr">
+      <c r="A166" s="6" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="6" t="inlineStr">
         <is>
           <t>## My Hero mission (from Yua)</t>
         </is>
       </c>
     </row>
-    <row r="167">
-      <c r="A167" s="6" t="inlineStr"/>
-    </row>
     <row r="168">
-      <c r="A168" s="6" t="inlineStr">
-        <is>
-          <t>1. Restore magic before it disappears completely</t>
-        </is>
-      </c>
+      <c r="A168" s="6" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="6" t="inlineStr">
         <is>
-          <t>2. Stand against the darkness consuming the world</t>
+          <t>1. Restore magic before it disappears completely</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="6" t="inlineStr">
         <is>
-          <t>3. Unite the fractured kingdoms and races</t>
+          <t>2. Stand against the darkness consuming the world</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="6" t="inlineStr">
         <is>
-          <t>4. Become the symbol of hope the world has long forgotten</t>
+          <t>3. Unite the fractured kingdoms and races</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="6" t="inlineStr">
         <is>
+          <t>4. Become the symbol of hope the world has long forgotten</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="6" t="inlineStr">
+        <is>
           <t>5. Bring together the two halves of the world</t>
         </is>
       </c>
     </row>
-    <row r="173">
-      <c r="A173" s="6" t="inlineStr"/>
-    </row>
     <row r="174">
-      <c r="A174" s="6" t="inlineStr">
+      <c r="A174" s="6" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="175">
-      <c r="A175" s="6" t="inlineStr"/>
-    </row>
     <row r="176">
-      <c r="A176" s="6" t="inlineStr">
+      <c r="A176" s="6" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="6" t="inlineStr">
         <is>
           <t>## Training under Rilock included</t>
         </is>
       </c>
     </row>
-    <row r="177">
-      <c r="A177" s="6" t="inlineStr"/>
-    </row>
     <row r="178">
-      <c r="A178" s="6" t="inlineStr">
-        <is>
-          <t>1. Endless swordsmanship drills</t>
-        </is>
-      </c>
+      <c r="A178" s="6" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="6" t="inlineStr">
         <is>
-          <t>2. Physical conditioning beyond normal limits</t>
+          <t>1. Endless swordsmanship drills</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="6" t="inlineStr">
         <is>
-          <t>3. Pain tolerance and endurance</t>
+          <t>2. Physical conditioning beyond normal limits</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="6" t="inlineStr">
         <is>
-          <t>4. Tactical education</t>
+          <t>3. Pain tolerance and endurance</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="6" t="inlineStr">
         <is>
+          <t>4. Tactical education</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="6" t="inlineStr">
+        <is>
           <t>5. Real combat missions (not simulations; death was possible)</t>
         </is>
       </c>
     </row>
-    <row r="183">
-      <c r="A183" s="6" t="inlineStr"/>
-    </row>
     <row r="184">
-      <c r="A184" s="6" t="inlineStr">
+      <c r="A184" s="6" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="185">
-      <c r="A185" s="6" t="inlineStr"/>
-    </row>
     <row r="186">
-      <c r="A186" s="6" t="inlineStr">
+      <c r="A186" s="6" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="6" t="inlineStr">
         <is>
           <t>## Colors, crest, sigil</t>
         </is>
       </c>
     </row>
-    <row r="187">
-      <c r="A187" s="6" t="inlineStr"/>
-    </row>
     <row r="188">
-      <c r="A188" s="6" t="inlineStr">
-        <is>
-          <t>| Item | Quick fact |</t>
-        </is>
-      </c>
+      <c r="A188" s="6" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| Item | Quick fact |</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="6" t="inlineStr">
         <is>
-          <t>| Why I wear red + black | I have always loved them; deep reason not revealed to me yet |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="6" t="inlineStr">
         <is>
-          <t>| My crest | Simple child crest: blade/flame between small parent marks |</t>
+          <t>| Why I wear red + black | I have always loved them; deep reason not revealed to me yet |</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="6" t="inlineStr">
         <is>
-          <t>| My sigil | One red/black blade or flame mark |</t>
+          <t>| My crest | Simple child crest: blade/flame between small parent marks |</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="6" t="inlineStr">
         <is>
-          <t>| Crest tradition | Child crest = name + gender + both parents; simpler than parents; unique |</t>
+          <t>| My sigil | One red/black blade or flame mark |</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="6" t="inlineStr">
         <is>
+          <t>| Crest tradition | Child crest = name + gender + both parents; simpler than parents; unique |</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="6" t="inlineStr">
+        <is>
           <t>| Sigil tradition | Same day as crest; one quick seal mark |</t>
         </is>
       </c>
     </row>
-    <row r="195">
-      <c r="A195" s="6" t="inlineStr"/>
-    </row>
     <row r="196">
-      <c r="A196" s="6" t="inlineStr">
+      <c r="A196" s="6" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="6" t="inlineStr">
         <is>
           <t>### Family crest / sigil cheat sheet</t>
         </is>
       </c>
     </row>
-    <row r="197">
-      <c r="A197" s="6" t="inlineStr"/>
-    </row>
     <row r="198">
-      <c r="A198" s="6" t="inlineStr">
-        <is>
-          <t>| Person | Colors | Crest idea | Sigil idea |</t>
-        </is>
-      </c>
+      <c r="A198" s="6" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" s="6" t="inlineStr">
         <is>
-          <t>|---|---|---|---|</t>
+          <t>| Person | Colors | Crest idea | Sigil idea |</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="6" t="inlineStr">
         <is>
-          <t>| Dolkin | charcoal / iron / bronze | stone arch + hammer | hammer in arch |</t>
+          <t>|---|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="6" t="inlineStr">
         <is>
-          <t>| Fulfein | sage / silver / pale gold | leaf + crescent | leaf into crescent |</t>
+          <t>| Dolkin | charcoal / iron / bronze | stone arch + hammer | hammer in arch |</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="6" t="inlineStr">
         <is>
-          <t>| Dezco | red / black | balanced blade/flame | red/black split blade |</t>
+          <t>| Fulfein | sage / silver / pale gold | leaf + crescent | leaf into crescent |</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="6" t="inlineStr">
         <is>
-          <t>| Kalhien | blue / copper | forward eager mark | forward chevron |</t>
+          <t>| Dezco | red / black | balanced blade/flame | red/black split blade |</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="6" t="inlineStr">
         <is>
+          <t>| Kalhien | blue / copper | forward eager mark | forward chevron |</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="6" t="inlineStr">
+        <is>
           <t>| Astiale | rose / cream / sky | soft bud or star | soft bud/star |</t>
         </is>
       </c>
     </row>
-    <row r="205">
-      <c r="A205" s="6" t="inlineStr"/>
-    </row>
     <row r="206">
-      <c r="A206" s="6" t="inlineStr">
+      <c r="A206" s="6" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="6" t="inlineStr">
         <is>
           <t>Images: `assets/crests/alzenhiem/`</t>
         </is>
       </c>
     </row>
-    <row r="207">
-      <c r="A207" s="6" t="inlineStr"/>
-    </row>
     <row r="208">
-      <c r="A208" s="6" t="inlineStr">
+      <c r="A208" s="6" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="209">
-      <c r="A209" s="6" t="inlineStr"/>
-    </row>
     <row r="210">
-      <c r="A210" s="6" t="inlineStr">
+      <c r="A210" s="6" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="6" t="inlineStr">
         <is>
           <t>## Secrets / do not spoil yet</t>
         </is>
       </c>
     </row>
-    <row r="211">
-      <c r="A211" s="6" t="inlineStr"/>
-    </row>
     <row r="212">
-      <c r="A212" s="6" t="inlineStr">
+      <c r="A212" s="6" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="6" t="inlineStr">
         <is>
           <t>Use this when roleplaying what party members know.</t>
         </is>
       </c>
     </row>
-    <row r="213">
-      <c r="A213" s="6" t="inlineStr"/>
-    </row>
     <row r="214">
-      <c r="A214" s="6" t="inlineStr">
-        <is>
-          <t>| Topic | Party can know? | Notes |</t>
-        </is>
-      </c>
+      <c r="A214" s="6" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" s="6" t="inlineStr">
         <is>
-          <t>|---|---|---|</t>
+          <t>| Topic | Party can know? | Notes |</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="6" t="inlineStr">
         <is>
-          <t>| I am from Alzenhiem + family basics | Yes | Safe to share |</t>
+          <t>|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="6" t="inlineStr">
         <is>
-          <t>| Trained since 8 in the yard; from 12 under Rilock by Lion’s order | Yes | Clarify: Lion directed, Rilock taught |</t>
+          <t>| I am from Alzenhiem + family basics | Yes | Safe to share |</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="6" t="inlineStr">
         <is>
-          <t>| People rumored I was Hero early | Yes | Emphasize it was rumor then |</t>
+          <t>| Trained since 8 in the yard; from 12 under Rilock by Lion’s order | Yes | Clarify: Lion directed, Rilock taught |</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="6" t="inlineStr">
         <is>
-          <t>| Yua made me Hero at 17 | Yes, if trust is there | She often looks like a pixie |</t>
+          <t>| People rumored I was Hero early | Yes | Emphasize it was rumor then |</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="6" t="inlineStr">
         <is>
-          <t>| Yua walks with me daily | No | Only King’s Lion + Rilock know |</t>
+          <t>| Yua made me Hero at 17 | Yes, if trust is there | She often looks like a pixie |</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="6" t="inlineStr">
         <is>
-          <t>| A divine being was seen in the world | Yes | Public knowledge; not tied to me |</t>
+          <t>| Yua walks with me daily | No | Only King’s Lion + Rilock know |</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="6" t="inlineStr">
         <is>
-          <t>| I talk to empty air when stressed | They saw it | Bridge return; vine excuse worked for now |</t>
+          <t>| A divine being was seen in the world | Yes | Public knowledge; not tied to me |</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="6" t="inlineStr">
         <is>
-          <t>| Exact red/black blood meaning | No | Yua will tell me later; I do not know yet |</t>
+          <t>| I talk to empty air when stressed | They saw it | Bridge return; vine excuse worked for now |</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="6" t="inlineStr">
         <is>
-          <t>| Mana Well / Lord AO gift | Partial | Yua named gift in private woods talk; training still ahead |</t>
+          <t>| Exact red/black blood meaning | No | Yua will tell me later; I do not know yet |</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="6" t="inlineStr">
         <is>
-          <t>| Why I hide Yua from them | No | See yua-why-she-stays-hidden.md |</t>
+          <t>| Mana Well / Lord AO gift | Partial | Yua named gift in private woods talk; training still ahead |</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="6" t="inlineStr">
         <is>
+          <t>| Why I hide Yua from them | No | See yua-why-she-stays-hidden.md |</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="6" t="inlineStr">
+        <is>
           <t>| Full private family crest theology | Optional | Share lightly unless asked |</t>
         </is>
       </c>
     </row>
-    <row r="227">
-      <c r="A227" s="6" t="inlineStr"/>
-    </row>
     <row r="228">
-      <c r="A228" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">**Red/black truth (for you / DM only, not my current knowledge):**  </t>
-        </is>
-      </c>
+      <c r="A228" s="6" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">**Red/black truth (for you / DM only, not my current knowledge):**  </t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="6" t="inlineStr">
+        <is>
           <t>Black = Dwarven caves / void / dark over light. Red = Elven holy blood after ill happens. Together = balance.</t>
         </is>
       </c>
     </row>
-    <row r="230">
-      <c r="A230" s="6" t="inlineStr"/>
-    </row>
     <row r="231">
-      <c r="A231" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">**Mana Well truth (for you / DM; Yua explained partially in woods):**  </t>
-        </is>
-      </c>
+      <c r="A231" s="6" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">**Mana Well truth (for you / DM; Yua explained partially in woods):**  </t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="6" t="inlineStr">
+        <is>
           <t>Mana pool stored within soul confines but separate from the soul. Gift from Lord AO per Yua after tomb road. Simple imbue makes sword lighter/sharper and grants a short agility burst. First accidental use: ~15 ft dash mid swing in street fight. Second use: deliberate cleave through two goblins in keep. Needs training. Yua senses unknown darkness ahead.</t>
         </is>
       </c>
     </row>
-    <row r="233">
-      <c r="A233" s="6" t="inlineStr"/>
-    </row>
     <row r="234">
-      <c r="A234" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">**Yua hidden truth (for you / DM):**  </t>
-        </is>
-      </c>
+      <c r="A234" s="6" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">**Yua hidden truth (for you / DM):**  </t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="6" t="inlineStr">
+        <is>
           <t>See `character/lore/yua-story-plots/yua-why-she-stays-hidden.md`. Hope must stay on mortal hands, not slide to worship of her presence.</t>
         </is>
       </c>
     </row>
-    <row r="236">
-      <c r="A236" s="6" t="inlineStr"/>
-    </row>
     <row r="237">
-      <c r="A237" s="6" t="inlineStr">
+      <c r="A237" s="6" t="inlineStr"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="238">
-      <c r="A238" s="6" t="inlineStr"/>
-    </row>
     <row r="239">
-      <c r="A239" s="6" t="inlineStr">
+      <c r="A239" s="6" t="inlineStr"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="6" t="inlineStr">
         <is>
           <t>## Abilities (Mana Well)</t>
         </is>
       </c>
     </row>
-    <row r="240">
-      <c r="A240" s="6" t="inlineStr"/>
-    </row>
     <row r="241">
-      <c r="A241" s="6" t="inlineStr">
-        <is>
-          <t>| Piece | Quick fact |</t>
-        </is>
-      </c>
+      <c r="A241" s="6" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| Piece | Quick fact |</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="6" t="inlineStr">
         <is>
-          <t>| Source | Bestowed by Yua with the Hero charge; unexplained at first |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="6" t="inlineStr">
         <is>
-          <t>| Well | Stored mana pool within soul confines; separate from the soul |</t>
+          <t>| Source | Bestowed by Yua with the Hero charge; unexplained at first |</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="6" t="inlineStr">
         <is>
-          <t>| Simple imbue | Innate; should feel as easy as breathing once understood |</t>
+          <t>| Well | Stored mana pool within soul confines; separate from the soul |</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="6" t="inlineStr">
         <is>
-          <t>| Sword effect | Lighter, sharper; short burst of swiftness / agility |</t>
+          <t>| Simple imbue | Innate; should feel as easy as breathing once understood |</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="6" t="inlineStr">
         <is>
-          <t>| First use | Saltrock street fight (journal 03); accidental ~15 ft dash mid swing = muddy faceplant |</t>
+          <t>| Sword effect | Lighter, sharper; short burst of swiftness / agility |</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="6" t="inlineStr">
         <is>
-          <t>| Second use | Keep goblin fight; cleaved one at waist, gutted another &gt;10 ft away |</t>
+          <t>| First use | Saltrock street fight (journal 03); accidental ~15 ft dash mid swing = muddy faceplant |</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="6" t="inlineStr">
         <is>
-          <t>| Yua’s explanation | Woods talk after tomb: gift from Lord AO; grow together through training |</t>
+          <t>| Second use | Keep goblin fight; cleaved one at waist, gutted another &gt;10 ft away |</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="6" t="inlineStr">
         <is>
-          <t>| Yua’s warning | Feels a darkness she has never known; source unknown |</t>
+          <t>| Yua’s explanation | Woods talk after tomb: gift from Lord AO; grow together through training |</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="6" t="inlineStr">
         <is>
-          <t>| Training needed | Control timing, avoid waste, move with the burst instead of being thrown |</t>
+          <t>| Yua’s warning | Feels a darkness she has never known; source unknown |</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="6" t="inlineStr">
         <is>
+          <t>| Training needed | Control timing, avoid waste, move with the burst instead of being thrown |</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="6" t="inlineStr">
+        <is>
           <t>| Yua’s mood | Upset after bridge; said we need to talk later |</t>
         </is>
       </c>
     </row>
-    <row r="253">
-      <c r="A253" s="6" t="inlineStr"/>
-    </row>
     <row r="254">
-      <c r="A254" s="6" t="inlineStr">
+      <c r="A254" s="6" t="inlineStr"/>
+    </row>
+    <row r="255">
+      <c r="A255" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="255">
-      <c r="A255" s="6" t="inlineStr"/>
-    </row>
     <row r="256">
-      <c r="A256" s="6" t="inlineStr">
+      <c r="A256" s="6" t="inlineStr"/>
+    </row>
+    <row r="257">
+      <c r="A257" s="6" t="inlineStr">
         <is>
           <t>## How I sound when I talk about myself</t>
         </is>
       </c>
     </row>
-    <row r="257">
-      <c r="A257" s="6" t="inlineStr"/>
-    </row>
     <row r="258">
-      <c r="A258" s="6" t="inlineStr">
-        <is>
-          <t>1. Honest, a little unsure about being chosen</t>
-        </is>
-      </c>
+      <c r="A258" s="6" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" s="6" t="inlineStr">
         <is>
-          <t>2. Proud of Alzenhiem without boasting</t>
+          <t>1. Honest, a little unsure about being chosen</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="6" t="inlineStr">
         <is>
-          <t>3. Corrects “Hero of centuries” rumors for the training years</t>
+          <t>2. Proud of Alzenhiem without boasting</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="6" t="inlineStr">
         <is>
-          <t>4. Speaks kindly about family, especially Astiale</t>
+          <t>3. Corrects “Hero of centuries” rumors for the training years</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="6" t="inlineStr">
         <is>
-          <t>5. Does not claim to understand Yua fully</t>
+          <t>4. Speaks kindly about family, especially Astiale</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="6" t="inlineStr">
         <is>
+          <t>5. Does not claim to understand Yua fully</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="6" t="inlineStr">
+        <is>
           <t>6. Prefers no dramatic dash heavy speech; plain and direct</t>
         </is>
       </c>
     </row>
-    <row r="264">
-      <c r="A264" s="6" t="inlineStr"/>
-    </row>
     <row r="265">
-      <c r="A265" s="6" t="inlineStr">
+      <c r="A265" s="6" t="inlineStr"/>
+    </row>
+    <row r="266">
+      <c r="A266" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="266">
-      <c r="A266" s="6" t="inlineStr"/>
-    </row>
     <row r="267">
-      <c r="A267" s="6" t="inlineStr">
+      <c r="A267" s="6" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" s="6" t="inlineStr">
         <is>
           <t>## Where the long versions are</t>
         </is>
       </c>
     </row>
-    <row r="268">
-      <c r="A268" s="6" t="inlineStr"/>
-    </row>
     <row r="269">
-      <c r="A269" s="6" t="inlineStr">
-        <is>
-          <t>| Need | File |</t>
-        </is>
-      </c>
+      <c r="A269" s="6" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| Need | File |</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="6" t="inlineStr">
         <is>
-          <t>| Full character intro | `character/lore/dezco-knoleburn-character.md` |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="6" t="inlineStr">
         <is>
-          <t>| Journal index | `character/lore/journal/README.md` |</t>
+          <t>| Full character intro | `character/lore/dezco-knoleburn-character.md` |</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="6" t="inlineStr">
         <is>
-          <t>| Journal 01 (backstory) | `character/lore/journal/01-after-the-charge.md` |</t>
+          <t>| Journal index | `character/lore/journal/README.md` |</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="6" t="inlineStr">
         <is>
-          <t>| Journal 02 (leave home / Saltrock) | `character/lore/journal/02-leaving-home-for-saltrock.md` |</t>
+          <t>| Journal 01 (backstory) | `character/lore/journal/01-after-the-charge.md` |</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 (full) | `character/lore/journal/03-saltrock-staff-falls.md` |</t>
+          <t>| Journal 02 (leave home / Saltrock) | `character/lore/journal/02-leaving-home-for-saltrock.md` |</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="6" t="inlineStr">
         <is>
-          <t>| Yua hidden from party | `character/lore/yua-story-plots/yua-why-she-stays-hidden.md` |</t>
+          <t>| Journal 03 (full) | `character/lore/journal/03-saltrock-staff-falls.md` |</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="6" t="inlineStr">
         <is>
-          <t>| Name meanings | `character/lore/knoleburn-names.md` |</t>
+          <t>| Yua hidden from party | `character/lore/yua-story-plots/yua-why-she-stays-hidden.md` |</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="6" t="inlineStr">
         <is>
-          <t>| Crest / sigil deep meanings | `assets/crests/alzenhiem/README.md` |</t>
+          <t>| Name meanings | `character/lore/knoleburn-names.md` |</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="6" t="inlineStr">
         <is>
-          <t>| Yua story plots index | `character/lore/yua-story-plots/README.md` |</t>
+          <t>| Crest / sigil deep meanings | `assets/crests/alzenhiem/README.md` |</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="6" t="inlineStr">
         <is>
-          <t>| Red/black reveal (future) | `character/lore/yua-story-plots/yua-on-red-and-black.md` |</t>
+          <t>| Yua story plots index | `character/lore/yua-story-plots/README.md` |</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="6" t="inlineStr">
         <is>
-          <t>| Mana Well / sword imbue | `character/lore/yua-story-plots/yua-mana-well.md` |</t>
+          <t>| Red/black reveal (future) | `character/lore/yua-story-plots/yua-on-red-and-black.md` |</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="6" t="inlineStr">
         <is>
+          <t>| Mana Well / sword imbue | `character/lore/yua-story-plots/yua-mana-well.md` |</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="6" t="inlineStr">
+        <is>
           <t>| Downloadable Google export | `character/lore/exports/` (Sheets tabs `.xlsx` + Docs `.docx`) |</t>
         </is>
       </c>
     </row>
-    <row r="283">
-      <c r="A283" s="6" t="inlineStr"/>
-    </row>
     <row r="284">
-      <c r="A284" s="6" t="inlineStr">
+      <c r="A284" s="6" t="inlineStr"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="285">
-      <c r="A285" s="6" t="inlineStr"/>
-    </row>
     <row r="286">
-      <c r="A286" s="6" t="inlineStr">
+      <c r="A286" s="6" t="inlineStr"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="6" t="inlineStr">
         <is>
           <t>## Blank lines for new party facts</t>
         </is>
       </c>
     </row>
-    <row r="287">
-      <c r="A287" s="6" t="inlineStr"/>
-    </row>
     <row r="288">
-      <c r="A288" s="6" t="inlineStr">
+      <c r="A288" s="6" t="inlineStr"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="6" t="inlineStr">
         <is>
           <t>Add new rows here whenever something new becomes true in play:</t>
         </is>
       </c>
     </row>
-    <row r="289">
-      <c r="A289" s="6" t="inlineStr"/>
-    </row>
     <row r="290">
-      <c r="A290" s="6" t="inlineStr">
-        <is>
-          <t>| Date / session | New fact | Share with party? |</t>
-        </is>
-      </c>
+      <c r="A290" s="6" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" s="6" t="inlineStr">
         <is>
-          <t>|---|---|---|</t>
+          <t>| Date / session | New fact | Share with party? |</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="6" t="inlineStr">
         <is>
-          <t>| Journal 02 | Left Alzenhiem with Dolkin’s sword + smithing tools; Fulfein’s gold, pot, clothes, shovel | Yes |</t>
+          <t>|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="6" t="inlineStr">
         <is>
-          <t>| Journal 02 | Shovel is mom’s bathroom dig joke first; burial meaning is the quiet second read | Optional / tonal |</t>
+          <t>| Journal 02 | Left Alzenhiem with Dolkin’s sword + smithing tools; Fulfein’s gold, pot, clothes, shovel | Yes |</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="6" t="inlineStr">
         <is>
-          <t>| Journal 02 | In Saltrock tavern overnight; knows the floating protective staff | Yes |</t>
+          <t>| Journal 02 | Shovel is mom’s bathroom dig joke first; burial meaning is the quiet second read | Optional / tonal |</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Saltrock staff fell; crabs + creatures attacked | Yes |</t>
+          <t>| Journal 02 | In Saltrock tavern overnight; knows the floating protective staff | Yes |</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Missed a short bow creature; faceplant in wet muddy gravel; nearly shot; saved by Eden | Yes |</t>
+          <t>| Journal 03 | Saltrock staff fell; crabs + creatures attacked | Yes |</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Faceplant tied to accidental ~15 ft mana dash / simple imbue (not understood yet) | After Yua explains |</t>
+          <t>| Journal 03 | Missed a short bow creature; faceplant in wet muddy gravel; nearly shot; saved by Eden | Yes |</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Keep siege: troll (magic resistant, regenerating) + 5 goblins; Eden/fire; second imbue on goblins | Yes |</t>
+          <t>| Journal 03 | Faceplant tied to accidental ~15 ft mana dash / simple imbue (not understood yet) | After Yua explains |</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Party names: Eden, Alice, Jylia, Vita, Alem | Yes |</t>
+          <t>| Journal 03 | Keep siege: troll (magic resistant, regenerating) + 5 goblins; Eden/fire; second imbue on goblins | Yes |</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | First King’s Lion tomb quest; library map; Yolon; owlbear bridge; focus recovered | Yes |</t>
+          <t>| Journal 03 | Party names: Eden, Alice, Jylia, Vita, Alem | Yes |</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Yua visible only to me; party doubts path until Vita confirms map | No (hide Yua) |</t>
+          <t>| Journal 03 | Yolon fork: right = cliff stairs to tomb; Eden + Alice went left to rivers (their find unknown) | Yes |</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Talked to air on bridge; blamed dragon statue vines | They believe vine story |</t>
+          <t>| Journal 03 | Yua visible only to me; party doubts path until Vita confirms map | No (hide Yua) |</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Lord AO gift named in woods; Yua warns of unknown darkness | Private for now |</t>
+          <t>| Journal 03 | Talked to air on bridge; blamed dragon statue vines | They believe vine story |</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Focus restored Saltrock; feast; choose Lyndor escort vs Lořel with Yeara by dawn | Yes |</t>
+          <t>| Journal 03 | Lord AO gift named in woods; Yua warns of unknown darkness | Private for now |</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Foot hurt from 15 ft cliff fall; Eden smacked my hand with bow; Alice + Vita saved me | Yes (embarrassing) |</t>
+          <t>| Journal 03 | Focus restored Saltrock; feast; choose Lyndor escort vs Lořel with Yeara by dawn | Yes |</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="6" t="inlineStr">
         <is>
-          <t>| Yua plots | Mana Well bestowed at Hero charge; Yua will explain after watching the biff | After she tells me |</t>
+          <t>| Journal 03 | Foot hurt from 15 ft cliff fall; Eden smacked my hand with bow; Alice + Vita saved me | Yes (embarrassing) |</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="6" t="inlineStr">
         <is>
-          <t>| Lore | Birthday is November 6 | Yes |</t>
+          <t>| Yua plots | Mana Well bestowed at Hero charge; Yua will explain after watching the biff | After she tells me |</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="6" t="inlineStr">
         <is>
-          <t>| Export | Tabbed Sheets + Docs lore pack in character/lore/exports/ | Yes |</t>
+          <t>| Lore | Birthday is November 6 | Yes |</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="6" t="inlineStr">
         <is>
-          <t>| Lore | Trainer is Rilock (royal master swordsman); King’s Lion directed him | Yes |</t>
+          <t>| Export | Tabbed Sheets + Docs lore pack in character/lore/exports/ | Yes |</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="6" t="inlineStr">
+        <is>
+          <t>| Lore | Trainer is Rilock (royal master swordsman); King’s Lion directed him | Yes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="6" t="inlineStr">
         <is>
           <t>| | | |</t>
         </is>

</xml_diff>

<commit_message>
Remove Alice from Dezco lore; reassign beats to Eden and Vita
Eden is no longer a twin. She scouts the river fork alone. Vita
dives to his stomach to catch Dezco on the owlbear bridge after Eden
smacks his hand with her bow. Party reference and exports updated.

Co-authored-by: Dralorex <Dralorex@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/character/lore/exports/Dezco_Knoleburn_Lore_Tabs.xlsx
+++ b/character/lore/exports/Dezco_Knoleburn_Lore_Tabs.xlsx
@@ -3058,7 +3058,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>The fallen staff lay near enough that its wrongness ached in my teeth. Rain kept drumming the roof. People breathed too loud. The elf archer who saved me turned out to have a twin sister. Her name is Eden. She handles a bow like punishment made elegant. She is also, I learned quickly, terrible with frightened children. Her sister Alice is the opposite: soft voice, steady hands, the kind of presence that makes panic sit down.</t>
+          <t>The fallen staff lay near enough that its wrongness ached in my teeth. Rain kept drumming the roof. People breathed too loud. The elf archer who saved me is Eden. She handles a bow like punishment made elegant. She is also, I learned quickly, terrible with frightened children.</t>
         </is>
       </c>
     </row>
@@ -3498,7 +3498,7 @@
     <row r="129">
       <c r="A129" s="6" t="inlineStr">
         <is>
-          <t>Eden and Alice went left, down toward the water. The rest of us went right, up the cliff. I do not know yet what the sisters found by the river. We had a tomb to reach.</t>
+          <t>Eden went left alone to scout the river road. The rest of us went right, up the cliff. I do not know yet what she found by the water. We had a tomb to reach.</t>
         </is>
       </c>
     </row>
@@ -3608,7 +3608,7 @@
     <row r="151">
       <c r="A151" s="6" t="inlineStr">
         <is>
-          <t>I tried to recreate the lift Yua had given me, if it was her at all. I attempted to jump a gap back onto the bridge. Nothing answered. I started to fall into the deep cavern below. One hand barely hooked the edge. Eden reached with her bow to help me grab it. She smacked my fingers instead. I lost my grip and dropped farther. Alice caught my other hand just in time. Vita came over and helped pull me all the way up.</t>
+          <t>I tried to recreate the lift Yua had given me, if it was her at all. I attempted to jump a gap back onto the bridge. Nothing answered. I started to fall into the deep cavern below. One hand barely hooked the edge. Eden reached with her bow to help me grab it. She smacked my fingers instead. I lost my grip and dropped farther. Vita dove to his stomach, slid to the edge, and caught my wrist just in time. He helped pull me all the way up.</t>
         </is>
       </c>
     </row>
@@ -4831,7 +4831,7 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>| Saltrock party (Eden, Alice, Jylia, Vita, Alem, etc.) | No |</t>
+          <t>| Saltrock party (Eden, Jylia, Vita, Alem, etc.) | No |</t>
         </is>
       </c>
     </row>
@@ -6254,7 +6254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A311"/>
+  <dimension ref="A1:A310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -6304,7 +6304,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">**Last updated:** 2026-08-23 (Journal 03 detail pass: Yolon fork, river split, owlbear bridge)  </t>
+          <t xml:space="preserve">**Last updated:** 2026-08-30 (removed Alice; Eden solo scout; Vita bridge save)  </t>
         </is>
       </c>
     </row>
@@ -6986,1193 +6986,1186 @@
     <row r="119">
       <c r="A119" s="6" t="inlineStr">
         <is>
-          <t>| Eden | Elf archer; twin to Alice; bow like punishment made elegant; terrible with frightened children; saved me in the street fight |</t>
+          <t>| Eden | Elf archer; bow like punishment made elegant; terrible with frightened children; saved me in the street fight; scouted river fork alone |</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="6" t="inlineStr">
         <is>
-          <t>| Alice | Eden’s twin; soft with scared people; good with children; pulled me up on the owlbear bridge |</t>
+          <t>| Jylia | Halfling dancer; fought in the keep; danced to calm the hall; pushed open the tomb door without hesitation |</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="6" t="inlineStr">
         <is>
-          <t>| Jylia | Halfling dancer; fought in the keep; danced to calm the hall; pushed open the tomb door without hesitation |</t>
+          <t>| Vita | Human priest (~30s); healer and spellcaster; read the old library map; dove to catch me on the owlbear bridge; helped restore the focus; collected Yolon statue vines |</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="6" t="inlineStr">
         <is>
-          <t>| Vita | Human priest (~30s); healer and spellcaster; read the old library map; helped restore the focus; collected Yolon statue vines |</t>
+          <t>| Alem | Snake man; telepathy mind to mind; healed before I met him properly; relayed Eden’s owlbear scouting |</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
         <is>
-          <t>| Alem | Snake man; telepathy mind to mind; healed before I met him properly; relayed Eden’s owlbear scouting |</t>
+          <t>| Yeara | Priestess in Saltrock; worked with Vita and the mayor to set the focus back; wants us at Lořel by morning decision |</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="6" t="inlineStr">
         <is>
-          <t>| Yeara | Priestess in Saltrock; worked with Vita and the mayor to set the focus back; wants us at Lořel by morning decision |</t>
+          <t>| Yolon | Stone dragon statue (&gt;100 years); spoke after Jylia drank bowl rain; fought first King’s Lion to endless draws; said take the right fork at the next split |</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="6" t="inlineStr">
         <is>
-          <t>| Yolon | Stone dragon statue (&gt;100 years); spoke after Jylia drank bowl rain; fought first King’s Lion to endless draws; said take the right fork at the next split |</t>
+          <t>| Saltrock mayor | Town leader; sent us to the tomb; wants escort to Lord Keivan in Lyndor |</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="6" t="inlineStr">
         <is>
-          <t>| Saltrock mayor | Town leader; sent us to the tomb; wants escort to Lord Keivan in Lyndor |</t>
+          <t>| Lord Keivan | Ruler in capital Lyndor; mayor wants to present us there |</t>
         </is>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="6" t="inlineStr">
-        <is>
-          <t>| Lord Keivan | Ruler in capital Lyndor; mayor wants to present us there |</t>
-        </is>
-      </c>
+      <c r="A127" s="6" t="inlineStr"/>
     </row>
     <row r="128">
-      <c r="A128" s="6" t="inlineStr"/>
+      <c r="A128" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
     </row>
     <row r="129">
-      <c r="A129" s="6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="A129" s="6" t="inlineStr"/>
     </row>
     <row r="130">
-      <c r="A130" s="6" t="inlineStr"/>
+      <c r="A130" s="6" t="inlineStr">
+        <is>
+          <t>## Current gear / gifts from home</t>
+        </is>
+      </c>
     </row>
     <row r="131">
-      <c r="A131" s="6" t="inlineStr">
-        <is>
-          <t>## Current gear / gifts from home</t>
-        </is>
-      </c>
+      <c r="A131" s="6" t="inlineStr"/>
     </row>
     <row r="132">
-      <c r="A132" s="6" t="inlineStr"/>
+      <c r="A132" s="6" t="inlineStr">
+        <is>
+          <t>| Item | From | Notes |</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="6" t="inlineStr">
         <is>
-          <t>| Item | From | Notes |</t>
+          <t>|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="6" t="inlineStr">
         <is>
-          <t>|---|---|---|</t>
+          <t>| New sword | Dolkin | Hand forged goodbye; his love without saying the words |</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="6" t="inlineStr">
         <is>
-          <t>| New sword | Dolkin | Hand forged goodbye; his love without saying the words |</t>
+          <t>| First smithing tools | Dolkin | His original set; “you are the master of your steel” |</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="6" t="inlineStr">
         <is>
-          <t>| First smithing tools | Dolkin | His original set; “you are the master of your steel” |</t>
+          <t>| 10 gold pieces | Fulfein | Travel money |</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>| 10 gold pieces | Fulfein | Travel money |</t>
+          <t>| Cooking pot | Fulfein | Eat warm when you can |</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
         <is>
-          <t>| Cooking pot | Fulfein | Eat warm when you can |</t>
+          <t>| New clothing | Fulfein | Wearing them out of respect; left home in them |</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
         <is>
-          <t>| New clothing | Fulfein | Wearing them out of respect; left home in them |</t>
+          <t>| Shovel | Fulfein | Funny gift for roadside “number two” duty; also quietly useful if not everyone makes it |</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="6" t="inlineStr">
         <is>
-          <t>| Shovel | Fulfein | Funny gift for roadside “number two” duty; also quietly useful if not everyone makes it |</t>
+          <t>| Tomb focus (recovered) | Saltrock quest | Faint glow; purpose unknown at first; mayor + Vita + Yeara restored town protection with it |</t>
         </is>
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="6" t="inlineStr">
-        <is>
-          <t>| Tomb focus (recovered) | Saltrock quest | Faint glow; purpose unknown at first; mayor + Vita + Yeara restored town protection with it |</t>
-        </is>
-      </c>
+      <c r="A141" s="6" t="inlineStr"/>
     </row>
     <row r="142">
-      <c r="A142" s="6" t="inlineStr"/>
+      <c r="A142" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
     </row>
     <row r="143">
-      <c r="A143" s="6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="A143" s="6" t="inlineStr"/>
     </row>
     <row r="144">
-      <c r="A144" s="6" t="inlineStr"/>
+      <c r="A144" s="6" t="inlineStr">
+        <is>
+          <t>## Places</t>
+        </is>
+      </c>
     </row>
     <row r="145">
-      <c r="A145" s="6" t="inlineStr">
-        <is>
-          <t>## Places</t>
-        </is>
-      </c>
+      <c r="A145" s="6" t="inlineStr"/>
     </row>
     <row r="146">
-      <c r="A146" s="6" t="inlineStr"/>
+      <c r="A146" s="6" t="inlineStr">
+        <is>
+          <t>| Place | What it is |</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="6" t="inlineStr">
         <is>
-          <t>| Place | What it is |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| Alzenhiem | Home hamlet; my center |</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="6" t="inlineStr">
         <is>
-          <t>| Alzenhiem | Home hamlet; my center |</t>
+          <t>| Saltrock | Traveling town; staff fell then focus restored; feast tonight; dawn choice pending |</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="6" t="inlineStr">
         <is>
-          <t>| Saltrock | Traveling town; staff fell then focus restored; feast tonight; dawn choice pending |</t>
+          <t>| Saltrock keep / general building | Where townsfolk sheltered; back wall breached by troll; focus set back with Vita and Yeara |</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="6" t="inlineStr">
         <is>
-          <t>| Saltrock keep / general building | Where townsfolk sheltered; back wall breached by troll; focus set back with Vita and Yeara |</t>
+          <t>| Saltrock library | Old book with scrappy map to first King’s Lion tomb |</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="6" t="inlineStr">
         <is>
-          <t>| Saltrock library | Old book with scrappy map to first King’s Lion tomb |</t>
+          <t>| Saltrock tavern | Where I lodged the night before the attack; “best bread” only with nostalgia |</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="6" t="inlineStr">
         <is>
-          <t>| Saltrock tavern | Where I lodged the night before the attack; “best bread” only with nostalgia |</t>
+          <t>| Lyndor | Capital; Lord Keivan; mayor wants escort there |</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="6" t="inlineStr">
         <is>
-          <t>| Lyndor | Capital; Lord Keivan; mayor wants escort there |</t>
+          <t>| Lořel | City of churches; priestess Yeara wants us to go there instead |</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="6" t="inlineStr">
         <is>
-          <t>| Lořel | City of churches; priestess Yeara wants us to go there instead |</t>
+          <t>| First King’s Lion tomb | Hilltop beyond Saltrock; goblin hideout behind outer door; real tomb held the focus |</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="6" t="inlineStr">
         <is>
-          <t>| First King’s Lion tomb | Hilltop beyond Saltrock; goblin hideout behind outer door; real tomb held the focus |</t>
+          <t>| Yolon statue | Stone dragon with rain bowl on tomb path; grime, moss, vines; spoke when Jylia drank; said keep path then take right at fork |</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="6" t="inlineStr">
         <is>
-          <t>| Yolon statue | Stone dragon with rain bowl on tomb path; grime, moss, vines; spoke when Jylia drank; said keep path then take right at fork |</t>
+          <t>| Tomb road fork | Left path down to rivers (Eden scouted alone); right path cliff stairs to hilltop tomb (rest of party) |</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="6" t="inlineStr">
         <is>
-          <t>| Tomb road fork | Left path down to rivers (Eden + Alice went); right path cliff stairs to hilltop tomb (rest of party) |</t>
+          <t>| Owlbear bridge | Rickety crossing past false boulder; sleeping giant owlbear inside; gone on return trip |</t>
         </is>
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="6" t="inlineStr">
-        <is>
-          <t>| Owlbear bridge | Rickety crossing past false boulder; sleeping giant owlbear inside; gone on return trip |</t>
-        </is>
-      </c>
+      <c r="A159" s="6" t="inlineStr"/>
     </row>
     <row r="160">
-      <c r="A160" s="6" t="inlineStr"/>
+      <c r="A160" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">**First magic item I ever saw:** the floating protective staff in Saltrock.  </t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">**First magic item I ever saw:** the floating protective staff in Saltrock.  </t>
+          <t xml:space="preserve">**Current crisis resolved:** focus back in place; town shielded again.  </t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">**Current crisis resolved:** focus back in place; town shielded again.  </t>
+          <t>**Current dilemma:** escort mayor to Lyndor vs travel with Yeara to Lořel; decide by morning.</t>
         </is>
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="6" t="inlineStr">
-        <is>
-          <t>**Current dilemma:** escort mayor to Lyndor vs travel with Yeara to Lořel; decide by morning.</t>
-        </is>
-      </c>
+      <c r="A163" s="6" t="inlineStr"/>
     </row>
     <row r="164">
-      <c r="A164" s="6" t="inlineStr"/>
+      <c r="A164" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
     </row>
     <row r="165">
-      <c r="A165" s="6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="A165" s="6" t="inlineStr"/>
     </row>
     <row r="166">
-      <c r="A166" s="6" t="inlineStr"/>
+      <c r="A166" s="6" t="inlineStr">
+        <is>
+          <t>## My Hero mission (from Yua)</t>
+        </is>
+      </c>
     </row>
     <row r="167">
-      <c r="A167" s="6" t="inlineStr">
-        <is>
-          <t>## My Hero mission (from Yua)</t>
-        </is>
-      </c>
+      <c r="A167" s="6" t="inlineStr"/>
     </row>
     <row r="168">
-      <c r="A168" s="6" t="inlineStr"/>
+      <c r="A168" s="6" t="inlineStr">
+        <is>
+          <t>1. Restore magic before it disappears completely</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="6" t="inlineStr">
         <is>
-          <t>1. Restore magic before it disappears completely</t>
+          <t>2. Stand against the darkness consuming the world</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="6" t="inlineStr">
         <is>
-          <t>2. Stand against the darkness consuming the world</t>
+          <t>3. Unite the fractured kingdoms and races</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="6" t="inlineStr">
         <is>
-          <t>3. Unite the fractured kingdoms and races</t>
+          <t>4. Become the symbol of hope the world has long forgotten</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="6" t="inlineStr">
         <is>
-          <t>4. Become the symbol of hope the world has long forgotten</t>
+          <t>5. Bring together the two halves of the world</t>
         </is>
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="6" t="inlineStr">
-        <is>
-          <t>5. Bring together the two halves of the world</t>
-        </is>
-      </c>
+      <c r="A173" s="6" t="inlineStr"/>
     </row>
     <row r="174">
-      <c r="A174" s="6" t="inlineStr"/>
+      <c r="A174" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
     </row>
     <row r="175">
-      <c r="A175" s="6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="A175" s="6" t="inlineStr"/>
     </row>
     <row r="176">
-      <c r="A176" s="6" t="inlineStr"/>
+      <c r="A176" s="6" t="inlineStr">
+        <is>
+          <t>## Training under Rilock included</t>
+        </is>
+      </c>
     </row>
     <row r="177">
-      <c r="A177" s="6" t="inlineStr">
-        <is>
-          <t>## Training under Rilock included</t>
-        </is>
-      </c>
+      <c r="A177" s="6" t="inlineStr"/>
     </row>
     <row r="178">
-      <c r="A178" s="6" t="inlineStr"/>
+      <c r="A178" s="6" t="inlineStr">
+        <is>
+          <t>1. Endless swordsmanship drills</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="6" t="inlineStr">
         <is>
-          <t>1. Endless swordsmanship drills</t>
+          <t>2. Physical conditioning beyond normal limits</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="6" t="inlineStr">
         <is>
-          <t>2. Physical conditioning beyond normal limits</t>
+          <t>3. Pain tolerance and endurance</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="6" t="inlineStr">
         <is>
-          <t>3. Pain tolerance and endurance</t>
+          <t>4. Tactical education</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="6" t="inlineStr">
         <is>
-          <t>4. Tactical education</t>
+          <t>5. Real combat missions (not simulations; death was possible)</t>
         </is>
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="6" t="inlineStr">
-        <is>
-          <t>5. Real combat missions (not simulations; death was possible)</t>
-        </is>
-      </c>
+      <c r="A183" s="6" t="inlineStr"/>
     </row>
     <row r="184">
-      <c r="A184" s="6" t="inlineStr"/>
+      <c r="A184" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
     </row>
     <row r="185">
-      <c r="A185" s="6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="A185" s="6" t="inlineStr"/>
     </row>
     <row r="186">
-      <c r="A186" s="6" t="inlineStr"/>
+      <c r="A186" s="6" t="inlineStr">
+        <is>
+          <t>## Colors, crest, sigil</t>
+        </is>
+      </c>
     </row>
     <row r="187">
-      <c r="A187" s="6" t="inlineStr">
-        <is>
-          <t>## Colors, crest, sigil</t>
-        </is>
-      </c>
+      <c r="A187" s="6" t="inlineStr"/>
     </row>
     <row r="188">
-      <c r="A188" s="6" t="inlineStr"/>
+      <c r="A188" s="6" t="inlineStr">
+        <is>
+          <t>| Item | Quick fact |</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="6" t="inlineStr">
         <is>
-          <t>| Item | Quick fact |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| Why I wear red + black | I have always loved them; deep reason not revealed to me yet |</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="6" t="inlineStr">
         <is>
-          <t>| Why I wear red + black | I have always loved them; deep reason not revealed to me yet |</t>
+          <t>| My crest | Simple child crest: blade/flame between small parent marks |</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="6" t="inlineStr">
         <is>
-          <t>| My crest | Simple child crest: blade/flame between small parent marks |</t>
+          <t>| My sigil | One red/black blade or flame mark |</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="6" t="inlineStr">
         <is>
-          <t>| My sigil | One red/black blade or flame mark |</t>
+          <t>| Crest tradition | Child crest = name + gender + both parents; simpler than parents; unique |</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="6" t="inlineStr">
         <is>
-          <t>| Crest tradition | Child crest = name + gender + both parents; simpler than parents; unique |</t>
+          <t>| Sigil tradition | Same day as crest; one quick seal mark |</t>
         </is>
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="6" t="inlineStr">
-        <is>
-          <t>| Sigil tradition | Same day as crest; one quick seal mark |</t>
-        </is>
-      </c>
+      <c r="A195" s="6" t="inlineStr"/>
     </row>
     <row r="196">
-      <c r="A196" s="6" t="inlineStr"/>
+      <c r="A196" s="6" t="inlineStr">
+        <is>
+          <t>### Family crest / sigil cheat sheet</t>
+        </is>
+      </c>
     </row>
     <row r="197">
-      <c r="A197" s="6" t="inlineStr">
-        <is>
-          <t>### Family crest / sigil cheat sheet</t>
-        </is>
-      </c>
+      <c r="A197" s="6" t="inlineStr"/>
     </row>
     <row r="198">
-      <c r="A198" s="6" t="inlineStr"/>
+      <c r="A198" s="6" t="inlineStr">
+        <is>
+          <t>| Person | Colors | Crest idea | Sigil idea |</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="6" t="inlineStr">
         <is>
-          <t>| Person | Colors | Crest idea | Sigil idea |</t>
+          <t>|---|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="6" t="inlineStr">
         <is>
-          <t>|---|---|---|---|</t>
+          <t>| Dolkin | charcoal / iron / bronze | stone arch + hammer | hammer in arch |</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="6" t="inlineStr">
         <is>
-          <t>| Dolkin | charcoal / iron / bronze | stone arch + hammer | hammer in arch |</t>
+          <t>| Fulfein | sage / silver / pale gold | leaf + crescent | leaf into crescent |</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="6" t="inlineStr">
         <is>
-          <t>| Fulfein | sage / silver / pale gold | leaf + crescent | leaf into crescent |</t>
+          <t>| Dezco | red / black | balanced blade/flame | red/black split blade |</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="6" t="inlineStr">
         <is>
-          <t>| Dezco | red / black | balanced blade/flame | red/black split blade |</t>
+          <t>| Kalhien | blue / copper | forward eager mark | forward chevron |</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="6" t="inlineStr">
         <is>
-          <t>| Kalhien | blue / copper | forward eager mark | forward chevron |</t>
+          <t>| Astiale | rose / cream / sky | soft bud or star | soft bud/star |</t>
         </is>
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="6" t="inlineStr">
-        <is>
-          <t>| Astiale | rose / cream / sky | soft bud or star | soft bud/star |</t>
-        </is>
-      </c>
+      <c r="A205" s="6" t="inlineStr"/>
     </row>
     <row r="206">
-      <c r="A206" s="6" t="inlineStr"/>
+      <c r="A206" s="6" t="inlineStr">
+        <is>
+          <t>Images: `assets/crests/alzenhiem/`</t>
+        </is>
+      </c>
     </row>
     <row r="207">
-      <c r="A207" s="6" t="inlineStr">
-        <is>
-          <t>Images: `assets/crests/alzenhiem/`</t>
-        </is>
-      </c>
+      <c r="A207" s="6" t="inlineStr"/>
     </row>
     <row r="208">
-      <c r="A208" s="6" t="inlineStr"/>
+      <c r="A208" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
     </row>
     <row r="209">
-      <c r="A209" s="6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="A209" s="6" t="inlineStr"/>
     </row>
     <row r="210">
-      <c r="A210" s="6" t="inlineStr"/>
+      <c r="A210" s="6" t="inlineStr">
+        <is>
+          <t>## Secrets / do not spoil yet</t>
+        </is>
+      </c>
     </row>
     <row r="211">
-      <c r="A211" s="6" t="inlineStr">
-        <is>
-          <t>## Secrets / do not spoil yet</t>
-        </is>
-      </c>
+      <c r="A211" s="6" t="inlineStr"/>
     </row>
     <row r="212">
-      <c r="A212" s="6" t="inlineStr"/>
+      <c r="A212" s="6" t="inlineStr">
+        <is>
+          <t>Use this when roleplaying what party members know.</t>
+        </is>
+      </c>
     </row>
     <row r="213">
-      <c r="A213" s="6" t="inlineStr">
-        <is>
-          <t>Use this when roleplaying what party members know.</t>
-        </is>
-      </c>
+      <c r="A213" s="6" t="inlineStr"/>
     </row>
     <row r="214">
-      <c r="A214" s="6" t="inlineStr"/>
+      <c r="A214" s="6" t="inlineStr">
+        <is>
+          <t>| Topic | Party can know? | Notes |</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="6" t="inlineStr">
         <is>
-          <t>| Topic | Party can know? | Notes |</t>
+          <t>|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="6" t="inlineStr">
         <is>
-          <t>|---|---|---|</t>
+          <t>| I am from Alzenhiem + family basics | Yes | Safe to share |</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="6" t="inlineStr">
         <is>
-          <t>| I am from Alzenhiem + family basics | Yes | Safe to share |</t>
+          <t>| Trained since 8 in the yard; from 12 under Rilock by Lion’s order | Yes | Clarify: Lion directed, Rilock taught |</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="6" t="inlineStr">
         <is>
-          <t>| Trained since 8 in the yard; from 12 under Rilock by Lion’s order | Yes | Clarify: Lion directed, Rilock taught |</t>
+          <t>| People rumored I was Hero early | Yes | Emphasize it was rumor then |</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="6" t="inlineStr">
         <is>
-          <t>| People rumored I was Hero early | Yes | Emphasize it was rumor then |</t>
+          <t>| Yua made me Hero at 17 | Yes, if trust is there | She often looks like a pixie |</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="6" t="inlineStr">
         <is>
-          <t>| Yua made me Hero at 17 | Yes, if trust is there | She often looks like a pixie |</t>
+          <t>| Yua walks with me daily | No | Only King’s Lion + Rilock know |</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="6" t="inlineStr">
         <is>
-          <t>| Yua walks with me daily | No | Only King’s Lion + Rilock know |</t>
+          <t>| A divine being was seen in the world | Yes | Public knowledge; not tied to me |</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="6" t="inlineStr">
         <is>
-          <t>| A divine being was seen in the world | Yes | Public knowledge; not tied to me |</t>
+          <t>| I talk to empty air when stressed | They saw it | Bridge return; vine excuse worked for now |</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="6" t="inlineStr">
         <is>
-          <t>| I talk to empty air when stressed | They saw it | Bridge return; vine excuse worked for now |</t>
+          <t>| Exact red/black blood meaning | No | Yua will tell me later; I do not know yet |</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="6" t="inlineStr">
         <is>
-          <t>| Exact red/black blood meaning | No | Yua will tell me later; I do not know yet |</t>
+          <t>| Mana Well / Lord AO gift | Partial | Yua named gift in private woods talk; training still ahead |</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="6" t="inlineStr">
         <is>
-          <t>| Mana Well / Lord AO gift | Partial | Yua named gift in private woods talk; training still ahead |</t>
+          <t>| Why I hide Yua from them | No | See yua-why-she-stays-hidden.md |</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="6" t="inlineStr">
         <is>
-          <t>| Why I hide Yua from them | No | See yua-why-she-stays-hidden.md |</t>
+          <t>| Full private family crest theology | Optional | Share lightly unless asked |</t>
         </is>
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="6" t="inlineStr">
-        <is>
-          <t>| Full private family crest theology | Optional | Share lightly unless asked |</t>
-        </is>
-      </c>
+      <c r="A227" s="6" t="inlineStr"/>
     </row>
     <row r="228">
-      <c r="A228" s="6" t="inlineStr"/>
+      <c r="A228" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">**Red/black truth (for you / DM only, not my current knowledge):**  </t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">**Red/black truth (for you / DM only, not my current knowledge):**  </t>
+          <t>Black = Dwarven caves / void / dark over light. Red = Elven holy blood after ill happens. Together = balance.</t>
         </is>
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="6" t="inlineStr">
-        <is>
-          <t>Black = Dwarven caves / void / dark over light. Red = Elven holy blood after ill happens. Together = balance.</t>
-        </is>
-      </c>
+      <c r="A230" s="6" t="inlineStr"/>
     </row>
     <row r="231">
-      <c r="A231" s="6" t="inlineStr"/>
+      <c r="A231" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">**Mana Well truth (for you / DM; Yua explained partially in woods):**  </t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">**Mana Well truth (for you / DM; Yua explained partially in woods):**  </t>
+          <t>Mana pool stored within soul confines but separate from the soul. Gift from Lord AO per Yua after tomb road. Simple imbue makes sword lighter/sharper and grants a short agility burst. First accidental use: ~15 ft dash mid swing in street fight. Second use: deliberate cleave through two goblins in keep. Needs training. Yua senses unknown darkness ahead.</t>
         </is>
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="6" t="inlineStr">
-        <is>
-          <t>Mana pool stored within soul confines but separate from the soul. Gift from Lord AO per Yua after tomb road. Simple imbue makes sword lighter/sharper and grants a short agility burst. First accidental use: ~15 ft dash mid swing in street fight. Second use: deliberate cleave through two goblins in keep. Needs training. Yua senses unknown darkness ahead.</t>
-        </is>
-      </c>
+      <c r="A233" s="6" t="inlineStr"/>
     </row>
     <row r="234">
-      <c r="A234" s="6" t="inlineStr"/>
+      <c r="A234" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">**Yua hidden truth (for you / DM):**  </t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">**Yua hidden truth (for you / DM):**  </t>
+          <t>See `character/lore/yua-story-plots/yua-why-she-stays-hidden.md`. Hope must stay on mortal hands, not slide to worship of her presence.</t>
         </is>
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="6" t="inlineStr">
-        <is>
-          <t>See `character/lore/yua-story-plots/yua-why-she-stays-hidden.md`. Hope must stay on mortal hands, not slide to worship of her presence.</t>
-        </is>
-      </c>
+      <c r="A236" s="6" t="inlineStr"/>
     </row>
     <row r="237">
-      <c r="A237" s="6" t="inlineStr"/>
+      <c r="A237" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
     </row>
     <row r="238">
-      <c r="A238" s="6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="A238" s="6" t="inlineStr"/>
     </row>
     <row r="239">
-      <c r="A239" s="6" t="inlineStr"/>
+      <c r="A239" s="6" t="inlineStr">
+        <is>
+          <t>## Abilities (Mana Well)</t>
+        </is>
+      </c>
     </row>
     <row r="240">
-      <c r="A240" s="6" t="inlineStr">
-        <is>
-          <t>## Abilities (Mana Well)</t>
-        </is>
-      </c>
+      <c r="A240" s="6" t="inlineStr"/>
     </row>
     <row r="241">
-      <c r="A241" s="6" t="inlineStr"/>
+      <c r="A241" s="6" t="inlineStr">
+        <is>
+          <t>| Piece | Quick fact |</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="6" t="inlineStr">
         <is>
-          <t>| Piece | Quick fact |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| Source | Bestowed by Yua with the Hero charge; unexplained at first |</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="6" t="inlineStr">
         <is>
-          <t>| Source | Bestowed by Yua with the Hero charge; unexplained at first |</t>
+          <t>| Well | Stored mana pool within soul confines; separate from the soul |</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="6" t="inlineStr">
         <is>
-          <t>| Well | Stored mana pool within soul confines; separate from the soul |</t>
+          <t>| Simple imbue | Innate; should feel as easy as breathing once understood |</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="6" t="inlineStr">
         <is>
-          <t>| Simple imbue | Innate; should feel as easy as breathing once understood |</t>
+          <t>| Sword effect | Lighter, sharper; short burst of swiftness / agility |</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="6" t="inlineStr">
         <is>
-          <t>| Sword effect | Lighter, sharper; short burst of swiftness / agility |</t>
+          <t>| First use | Saltrock street fight (journal 03); accidental ~15 ft dash mid swing = muddy faceplant |</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="6" t="inlineStr">
         <is>
-          <t>| First use | Saltrock street fight (journal 03); accidental ~15 ft dash mid swing = muddy faceplant |</t>
+          <t>| Second use | Keep goblin fight; cleaved one at waist, gutted another &gt;10 ft away |</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="6" t="inlineStr">
         <is>
-          <t>| Second use | Keep goblin fight; cleaved one at waist, gutted another &gt;10 ft away |</t>
+          <t>| Yua’s explanation | Woods talk after tomb: gift from Lord AO; grow together through training |</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="6" t="inlineStr">
         <is>
-          <t>| Yua’s explanation | Woods talk after tomb: gift from Lord AO; grow together through training |</t>
+          <t>| Yua’s warning | Feels a darkness she has never known; source unknown |</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="6" t="inlineStr">
         <is>
-          <t>| Yua’s warning | Feels a darkness she has never known; source unknown |</t>
+          <t>| Training needed | Control timing, avoid waste, move with the burst instead of being thrown |</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="6" t="inlineStr">
         <is>
-          <t>| Training needed | Control timing, avoid waste, move with the burst instead of being thrown |</t>
+          <t>| Yua’s mood | Upset after bridge; said we need to talk later |</t>
         </is>
       </c>
     </row>
     <row r="253">
-      <c r="A253" s="6" t="inlineStr">
-        <is>
-          <t>| Yua’s mood | Upset after bridge; said we need to talk later |</t>
-        </is>
-      </c>
+      <c r="A253" s="6" t="inlineStr"/>
     </row>
     <row r="254">
-      <c r="A254" s="6" t="inlineStr"/>
+      <c r="A254" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
     </row>
     <row r="255">
-      <c r="A255" s="6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="A255" s="6" t="inlineStr"/>
     </row>
     <row r="256">
-      <c r="A256" s="6" t="inlineStr"/>
+      <c r="A256" s="6" t="inlineStr">
+        <is>
+          <t>## How I sound when I talk about myself</t>
+        </is>
+      </c>
     </row>
     <row r="257">
-      <c r="A257" s="6" t="inlineStr">
-        <is>
-          <t>## How I sound when I talk about myself</t>
-        </is>
-      </c>
+      <c r="A257" s="6" t="inlineStr"/>
     </row>
     <row r="258">
-      <c r="A258" s="6" t="inlineStr"/>
+      <c r="A258" s="6" t="inlineStr">
+        <is>
+          <t>1. Honest, a little unsure about being chosen</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="6" t="inlineStr">
         <is>
-          <t>1. Honest, a little unsure about being chosen</t>
+          <t>2. Proud of Alzenhiem without boasting</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="6" t="inlineStr">
         <is>
-          <t>2. Proud of Alzenhiem without boasting</t>
+          <t>3. Corrects “Hero of centuries” rumors for the training years</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="6" t="inlineStr">
         <is>
-          <t>3. Corrects “Hero of centuries” rumors for the training years</t>
+          <t>4. Speaks kindly about family, especially Astiale</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="6" t="inlineStr">
         <is>
-          <t>4. Speaks kindly about family, especially Astiale</t>
+          <t>5. Does not claim to understand Yua fully</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="6" t="inlineStr">
         <is>
-          <t>5. Does not claim to understand Yua fully</t>
+          <t>6. Prefers no dramatic dash heavy speech; plain and direct</t>
         </is>
       </c>
     </row>
     <row r="264">
-      <c r="A264" s="6" t="inlineStr">
-        <is>
-          <t>6. Prefers no dramatic dash heavy speech; plain and direct</t>
-        </is>
-      </c>
+      <c r="A264" s="6" t="inlineStr"/>
     </row>
     <row r="265">
-      <c r="A265" s="6" t="inlineStr"/>
+      <c r="A265" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
     </row>
     <row r="266">
-      <c r="A266" s="6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="A266" s="6" t="inlineStr"/>
     </row>
     <row r="267">
-      <c r="A267" s="6" t="inlineStr"/>
+      <c r="A267" s="6" t="inlineStr">
+        <is>
+          <t>## Where the long versions are</t>
+        </is>
+      </c>
     </row>
     <row r="268">
-      <c r="A268" s="6" t="inlineStr">
-        <is>
-          <t>## Where the long versions are</t>
-        </is>
-      </c>
+      <c r="A268" s="6" t="inlineStr"/>
     </row>
     <row r="269">
-      <c r="A269" s="6" t="inlineStr"/>
+      <c r="A269" s="6" t="inlineStr">
+        <is>
+          <t>| Need | File |</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="6" t="inlineStr">
         <is>
-          <t>| Need | File |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="6" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| Full character intro | `character/lore/dezco-knoleburn-character.md` |</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="6" t="inlineStr">
         <is>
-          <t>| Full character intro | `character/lore/dezco-knoleburn-character.md` |</t>
+          <t>| Journal index | `character/lore/journal/README.md` |</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="6" t="inlineStr">
         <is>
-          <t>| Journal index | `character/lore/journal/README.md` |</t>
+          <t>| Journal 01 (backstory) | `character/lore/journal/01-after-the-charge.md` |</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="6" t="inlineStr">
         <is>
-          <t>| Journal 01 (backstory) | `character/lore/journal/01-after-the-charge.md` |</t>
+          <t>| Journal 02 (leave home / Saltrock) | `character/lore/journal/02-leaving-home-for-saltrock.md` |</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="6" t="inlineStr">
         <is>
-          <t>| Journal 02 (leave home / Saltrock) | `character/lore/journal/02-leaving-home-for-saltrock.md` |</t>
+          <t>| Journal 03 (full) | `character/lore/journal/03-saltrock-staff-falls.md` |</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 (full) | `character/lore/journal/03-saltrock-staff-falls.md` |</t>
+          <t>| Yua hidden from party | `character/lore/yua-story-plots/yua-why-she-stays-hidden.md` |</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="6" t="inlineStr">
         <is>
-          <t>| Yua hidden from party | `character/lore/yua-story-plots/yua-why-she-stays-hidden.md` |</t>
+          <t>| Name meanings | `character/lore/knoleburn-names.md` |</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="6" t="inlineStr">
         <is>
-          <t>| Name meanings | `character/lore/knoleburn-names.md` |</t>
+          <t>| Crest / sigil deep meanings | `assets/crests/alzenhiem/README.md` |</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="6" t="inlineStr">
         <is>
-          <t>| Crest / sigil deep meanings | `assets/crests/alzenhiem/README.md` |</t>
+          <t>| Yua story plots index | `character/lore/yua-story-plots/README.md` |</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="6" t="inlineStr">
         <is>
-          <t>| Yua story plots index | `character/lore/yua-story-plots/README.md` |</t>
+          <t>| Red/black reveal (future) | `character/lore/yua-story-plots/yua-on-red-and-black.md` |</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="6" t="inlineStr">
         <is>
-          <t>| Red/black reveal (future) | `character/lore/yua-story-plots/yua-on-red-and-black.md` |</t>
+          <t>| Mana Well / sword imbue | `character/lore/yua-story-plots/yua-mana-well.md` |</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="6" t="inlineStr">
         <is>
-          <t>| Mana Well / sword imbue | `character/lore/yua-story-plots/yua-mana-well.md` |</t>
+          <t>| Downloadable Google export | `character/lore/exports/` (Sheets tabs `.xlsx` + Docs `.docx`) |</t>
         </is>
       </c>
     </row>
     <row r="283">
-      <c r="A283" s="6" t="inlineStr">
-        <is>
-          <t>| Downloadable Google export | `character/lore/exports/` (Sheets tabs `.xlsx` + Docs `.docx`) |</t>
-        </is>
-      </c>
+      <c r="A283" s="6" t="inlineStr"/>
     </row>
     <row r="284">
-      <c r="A284" s="6" t="inlineStr"/>
+      <c r="A284" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
     </row>
     <row r="285">
-      <c r="A285" s="6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="A285" s="6" t="inlineStr"/>
     </row>
     <row r="286">
-      <c r="A286" s="6" t="inlineStr"/>
+      <c r="A286" s="6" t="inlineStr">
+        <is>
+          <t>## Blank lines for new party facts</t>
+        </is>
+      </c>
     </row>
     <row r="287">
-      <c r="A287" s="6" t="inlineStr">
-        <is>
-          <t>## Blank lines for new party facts</t>
-        </is>
-      </c>
+      <c r="A287" s="6" t="inlineStr"/>
     </row>
     <row r="288">
-      <c r="A288" s="6" t="inlineStr"/>
+      <c r="A288" s="6" t="inlineStr">
+        <is>
+          <t>Add new rows here whenever something new becomes true in play:</t>
+        </is>
+      </c>
     </row>
     <row r="289">
-      <c r="A289" s="6" t="inlineStr">
-        <is>
-          <t>Add new rows here whenever something new becomes true in play:</t>
-        </is>
-      </c>
+      <c r="A289" s="6" t="inlineStr"/>
     </row>
     <row r="290">
-      <c r="A290" s="6" t="inlineStr"/>
+      <c r="A290" s="6" t="inlineStr">
+        <is>
+          <t>| Date / session | New fact | Share with party? |</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="6" t="inlineStr">
         <is>
-          <t>| Date / session | New fact | Share with party? |</t>
+          <t>|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="6" t="inlineStr">
         <is>
-          <t>|---|---|---|</t>
+          <t>| Journal 02 | Left Alzenhiem with Dolkin’s sword + smithing tools; Fulfein’s gold, pot, clothes, shovel | Yes |</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="6" t="inlineStr">
         <is>
-          <t>| Journal 02 | Left Alzenhiem with Dolkin’s sword + smithing tools; Fulfein’s gold, pot, clothes, shovel | Yes |</t>
+          <t>| Journal 02 | Shovel is mom’s bathroom dig joke first; burial meaning is the quiet second read | Optional / tonal |</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="6" t="inlineStr">
         <is>
-          <t>| Journal 02 | Shovel is mom’s bathroom dig joke first; burial meaning is the quiet second read | Optional / tonal |</t>
+          <t>| Journal 02 | In Saltrock tavern overnight; knows the floating protective staff | Yes |</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="6" t="inlineStr">
         <is>
-          <t>| Journal 02 | In Saltrock tavern overnight; knows the floating protective staff | Yes |</t>
+          <t>| Journal 03 | Saltrock staff fell; crabs + creatures attacked | Yes |</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Saltrock staff fell; crabs + creatures attacked | Yes |</t>
+          <t>| Journal 03 | Missed a short bow creature; faceplant in wet muddy gravel; nearly shot; saved by Eden | Yes |</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Missed a short bow creature; faceplant in wet muddy gravel; nearly shot; saved by Eden | Yes |</t>
+          <t>| Journal 03 | Faceplant tied to accidental ~15 ft mana dash / simple imbue (not understood yet) | After Yua explains |</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Faceplant tied to accidental ~15 ft mana dash / simple imbue (not understood yet) | After Yua explains |</t>
+          <t>| Journal 03 | Keep siege: troll (magic resistant, regenerating) + 5 goblins; Eden/fire; second imbue on goblins | Yes |</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Keep siege: troll (magic resistant, regenerating) + 5 goblins; Eden/fire; second imbue on goblins | Yes |</t>
+          <t>| Journal 03 | Party names: Eden, Jylia, Vita, Alem | Yes |</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Party names: Eden, Alice, Jylia, Vita, Alem | Yes |</t>
+          <t>| Journal 03 | Yolon fork: right = cliff stairs to tomb; Eden scouted left to rivers alone (her find unknown) | Yes |</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Yolon fork: right = cliff stairs to tomb; Eden + Alice went left to rivers (their find unknown) | Yes |</t>
+          <t>| Journal 03 | Yua visible only to me; party doubts path until Vita confirms map | No (hide Yua) |</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Yua visible only to me; party doubts path until Vita confirms map | No (hide Yua) |</t>
+          <t>| Journal 03 | Talked to air on bridge; blamed dragon statue vines | They believe vine story |</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Talked to air on bridge; blamed dragon statue vines | They believe vine story |</t>
+          <t>| Journal 03 | Lord AO gift named in woods; Yua warns of unknown darkness | Private for now |</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Lord AO gift named in woods; Yua warns of unknown darkness | Private for now |</t>
+          <t>| Journal 03 | Focus restored Saltrock; feast; choose Lyndor escort vs Lořel with Yeara by dawn | Yes |</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Focus restored Saltrock; feast; choose Lyndor escort vs Lořel with Yeara by dawn | Yes |</t>
+          <t>| Journal 03 | Foot hurt from 15 ft cliff fall; Eden smacked my hand with bow; Vita dove and caught my wrist on bridge | Yes (embarrassing) |</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="6" t="inlineStr">
         <is>
-          <t>| Journal 03 | Foot hurt from 15 ft cliff fall; Eden smacked my hand with bow; Alice + Vita saved me | Yes (embarrassing) |</t>
+          <t>| Yua plots | Mana Well bestowed at Hero charge; Yua will explain after watching the biff | After she tells me |</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="6" t="inlineStr">
         <is>
-          <t>| Yua plots | Mana Well bestowed at Hero charge; Yua will explain after watching the biff | After she tells me |</t>
+          <t>| Lore | Birthday is November 6 | Yes |</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="6" t="inlineStr">
         <is>
-          <t>| Lore | Birthday is November 6 | Yes |</t>
+          <t>| Export | Tabbed Sheets + Docs lore pack in character/lore/exports/ | Yes |</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="6" t="inlineStr">
         <is>
-          <t>| Export | Tabbed Sheets + Docs lore pack in character/lore/exports/ | Yes |</t>
+          <t>| Lore | Trainer is Rilock (royal master swordsman); King’s Lion directed him | Yes |</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="6" t="inlineStr">
-        <is>
-          <t>| Lore | Trainer is Rilock (royal master swordsman); King’s Lion directed him | Yes |</t>
-        </is>
-      </c>
-    </row>
-    <row r="311">
-      <c r="A311" s="6" t="inlineStr">
         <is>
           <t>| | | |</t>
         </is>

</xml_diff>